<commit_message>
Track scrape status in the workbook without counting it as a university tab.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -3,12 +3,15 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="National Universities" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liberal Arts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Universities" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Christian Colleges" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="National Universities" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liberal Arts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Universities" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Christian Colleges" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$I$11</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -16,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -67,6 +70,9 @@
       <strike val="1"/>
       <color rgb="FF0000FF"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -88,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -100,9 +106,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -113,6 +117,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -385,6 +392,549 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" style="19" min="1" max="1"/>
+    <col width="26" customWidth="1" style="19" min="2" max="2"/>
+    <col width="14" customWidth="1" style="19" min="3" max="3"/>
+    <col width="28" customWidth="1" style="19" min="4" max="4"/>
+    <col width="42" customWidth="1" style="19" min="5" max="5"/>
+    <col width="12" customWidth="1" style="19" min="6" max="6"/>
+    <col width="12" customWidth="1" style="19" min="7" max="7"/>
+    <col width="12" customWidth="1" style="19" min="8" max="8"/>
+    <col width="56" customWidth="1" style="19" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>university</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>site_key</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>domain</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>machine</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>started</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>University of Chicago</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>The Chicago Maroon</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>chicago</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>chicagomaroon.com</t>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F2" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I2" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@chicago</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Northwestern University</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>The Daily Northwestern</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>northwestern</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>dailynorthwestern.com</t>
+        </is>
+      </c>
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@northwestern</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Southern Methodist University</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>The Daily Campus</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>smu</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>smudailycampus.com</t>
+        </is>
+      </c>
+      <c r="E4" s="0" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H4" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I4" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@smu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Texas Christian University</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>TCU 360</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>tcu</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>tcu360.com</t>
+        </is>
+      </c>
+      <c r="E5" s="0" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F5" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tcu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Biola University</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>The Chimes</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>biola</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>chimesnewspaper.com</t>
+        </is>
+      </c>
+      <c r="E6" s="0" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F6" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G6" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H6" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@biola; high empty_body on old archive</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Union College (NY)</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>Concordiensis</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>union</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>concordiensis.com</t>
+        </is>
+      </c>
+      <c r="E7" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F7" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G7" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H7" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I7" s="0" t="inlineStr">
+        <is>
+          <t>Finished: 1604 articles of 1626 URLs; 44 empty_body skipped. systemd exited 0 and stayed inactive (Restart=on-failure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I8" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@stolaf; near complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Connecticut College</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>The College Voice</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>conncoll</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>thecollegevoice.org</t>
+        </is>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>testing</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H9" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>200-article test; not a full run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Franklin &amp; Marshall College</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>The College Reporter</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>fandm</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>the-college-reporter.com</t>
+        </is>
+      </c>
+      <c r="E10" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t>testing</t>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H10" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t>200-article test; not a full run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Hillsdale College</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>The Collegian</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>hillsdale</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>hillsdalecollegian.com</t>
+        </is>
+      </c>
+      <c r="E11" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F11" s="0" t="inlineStr">
+        <is>
+          <t>testing</t>
+        </is>
+      </c>
+      <c r="G11" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="H11" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t>200-article test; not a full run yet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -422,12 +972,12 @@
       <c r="F1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Princeton University 🌿</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
@@ -439,12 +989,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>MIT</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>#2</t>
         </is>
@@ -454,19 +1004,19 @@
           <t>https://thetech.com/</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Harvard 🌿</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>#3</t>
         </is>
@@ -478,12 +1028,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Stanford University</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
@@ -495,12 +1045,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Yale Universty 🌿</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
@@ -512,12 +1062,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>University of Chicago</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>#6</t>
         </is>
@@ -530,12 +1080,12 @@
       <c r="E7" s="9" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Duke University</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -547,12 +1097,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Johns Hopkins University</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -564,12 +1114,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Northwestern Univeristy</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -581,12 +1131,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Univeristy of Pennsylvania 🌿</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -598,12 +1148,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Cornell University 🌿</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>#12</t>
         </is>
@@ -615,12 +1165,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Brown University 🌿</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -632,12 +1182,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Dartmouth College 🌿</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -649,12 +1199,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Columbia Univeristy 🌿</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>#15</t>
         </is>
@@ -664,7 +1214,7 @@
           <t>https://www.columbiaspectator.com/</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>done</t>
         </is>
@@ -698,12 +1248,12 @@
       <c r="E17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Rice University</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>#17</t>
         </is>
@@ -734,12 +1284,12 @@
       <c r="E19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Vanderbilt University</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>#17</t>
         </is>
@@ -751,12 +1301,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Carnegie Mellon Univeristy</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>#20</t>
         </is>
@@ -787,12 +1337,12 @@
       <c r="E22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Univeristy of Notre Dame</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>#20</t>
         </is>
@@ -805,12 +1355,12 @@
       <c r="E23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Washington Univeristy in St. Louis</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>#20</t>
         </is>
@@ -822,12 +1372,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Emory University</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>#24</t>
         </is>
@@ -839,12 +1389,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Georgetown University</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>#24</t>
         </is>
@@ -856,12 +1406,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Univeristy of North Carolina, Chapel Hill</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>#26</t>
         </is>
@@ -873,12 +1423,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>Univeristy of Virginia</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>#26</t>
         </is>
@@ -890,12 +1440,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>University of Southern California</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
@@ -907,12 +1457,12 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Univeristy of California San Diego</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>#29</t>
         </is>
@@ -924,12 +1474,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>Univeristy of Florida</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>#30</t>
         </is>
@@ -941,12 +1491,12 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>The University of Texas, Austin</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>#30</t>
         </is>
@@ -958,12 +1508,12 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>Georgia Institute of Technology</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>#32</t>
         </is>
@@ -975,12 +1525,12 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>New York University</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>#32</t>
         </is>
@@ -992,12 +1542,12 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>University of California, Davis</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>#32</t>
         </is>
@@ -1009,12 +1559,12 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>Univeristy of California, Irvine</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>#32</t>
         </is>
@@ -1026,12 +1576,12 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>Boston College</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
@@ -1043,12 +1593,12 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>Tufts University</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
@@ -1060,12 +1610,12 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>University of Illinois Urbana, Champaign</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
@@ -1077,12 +1627,12 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>University of Wisconsin, Madison</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
@@ -1094,12 +1644,12 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>University of California, Santa Barbara</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>#40</t>
         </is>
@@ -1111,12 +1661,12 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>The Ohio State University</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>#41</t>
         </is>
@@ -1128,12 +1678,12 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>Boston University</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>#42</t>
         </is>
@@ -1145,12 +1695,12 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t>Rutgers University, New Brunswick</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>#42</t>
         </is>
@@ -1162,12 +1712,12 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>University of Maryland, College Park</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
         <is>
           <t>#42</t>
         </is>
@@ -1179,12 +1729,12 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>University of Washington</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B46" s="9" t="inlineStr">
         <is>
           <t>#42</t>
         </is>
@@ -1196,12 +1746,12 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>Lehigh University</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>#46</t>
         </is>
@@ -1213,12 +1763,12 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="A48" s="9" t="inlineStr">
         <is>
           <t>Northeastern University</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>#46</t>
         </is>
@@ -1230,12 +1780,12 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>Purdue Univeristy</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>#46</t>
         </is>
@@ -1247,12 +1797,12 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="A50" s="9" t="inlineStr">
         <is>
           <t>University of Georgia</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>#46</t>
         </is>
@@ -1264,12 +1814,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>University of Rochester</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>#46</t>
         </is>
@@ -1281,12 +1831,12 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>Case Western Reserve University</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>#51</t>
         </is>
@@ -1298,12 +1848,12 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="A53" s="9" t="inlineStr">
         <is>
           <t>Florida State University</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="9" t="inlineStr">
         <is>
           <t>#51</t>
         </is>
@@ -1315,12 +1865,12 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>Texas A&amp;M University</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B54" s="9" t="inlineStr">
         <is>
           <t>#51</t>
         </is>
@@ -1332,12 +1882,12 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>Virginia Tech</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B55" s="9" t="inlineStr">
         <is>
           <t>#51</t>
         </is>
@@ -1349,12 +1899,12 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>Wake Forest University</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B56" s="9" t="inlineStr">
         <is>
           <t>#51</t>
         </is>
@@ -1366,12 +1916,12 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>William &amp; Mary</t>
         </is>
       </c>
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B57" s="9" t="inlineStr">
         <is>
           <t>#51</t>
         </is>
@@ -1383,12 +1933,12 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="A58" s="9" t="inlineStr">
         <is>
           <t>Univeristy of California, Merced</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B58" s="9" t="inlineStr">
         <is>
           <t>#57</t>
         </is>
@@ -1400,12 +1950,12 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="A59" s="9" t="inlineStr">
         <is>
           <t>Villanova University</t>
         </is>
       </c>
-      <c r="B59" s="8" t="inlineStr">
+      <c r="B59" s="9" t="inlineStr">
         <is>
           <t>#57</t>
         </is>
@@ -1417,12 +1967,12 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="A60" s="9" t="inlineStr">
         <is>
           <t>George Washington University</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B60" s="9" t="inlineStr">
         <is>
           <t>#59</t>
         </is>
@@ -1434,12 +1984,12 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="A61" s="9" t="inlineStr">
         <is>
           <t>The Pennsylvania State University, University Park</t>
         </is>
       </c>
-      <c r="B61" s="8" t="inlineStr">
+      <c r="B61" s="9" t="inlineStr">
         <is>
           <t>#59</t>
         </is>
@@ -1451,12 +2001,12 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="A62" s="9" t="inlineStr">
         <is>
           <t>Santa Clara University</t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
         <is>
           <t>#59</t>
         </is>
@@ -1468,12 +2018,12 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="A63" s="9" t="inlineStr">
         <is>
           <t>Stony Brook University, SUNY</t>
         </is>
       </c>
-      <c r="B63" s="8" t="inlineStr">
+      <c r="B63" s="9" t="inlineStr">
         <is>
           <t>#59</t>
         </is>
@@ -1485,12 +2035,12 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="A64" s="9" t="inlineStr">
         <is>
           <t>University of Minnesota, Twin Cities</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B64" s="9" t="inlineStr">
         <is>
           <t>#59</t>
         </is>
@@ -1502,12 +2052,12 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="A65" s="9" t="inlineStr">
         <is>
           <t>Michigan State University</t>
         </is>
       </c>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B65" s="9" t="inlineStr">
         <is>
           <t>#64</t>
         </is>
@@ -1519,12 +2069,12 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="A66" s="9" t="inlineStr">
         <is>
           <t>North Carolina State University</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B66" s="9" t="inlineStr">
         <is>
           <t>#64</t>
         </is>
@@ -1536,12 +2086,12 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="A67" s="9" t="inlineStr">
         <is>
           <t>Rensselaer Polytechnic Institute</t>
         </is>
       </c>
-      <c r="B67" s="8" t="inlineStr">
+      <c r="B67" s="9" t="inlineStr">
         <is>
           <t>#64</t>
         </is>
@@ -1553,12 +2103,12 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="A68" s="9" t="inlineStr">
         <is>
           <t>University of Massachusetts, Amherst</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B68" s="9" t="inlineStr">
         <is>
           <t>#64</t>
         </is>
@@ -1570,12 +2120,12 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="A69" s="9" t="inlineStr">
         <is>
           <t>University of Miami</t>
         </is>
       </c>
-      <c r="B69" s="8" t="inlineStr">
+      <c r="B69" s="9" t="inlineStr">
         <is>
           <t>#64</t>
         </is>
@@ -1587,12 +2137,12 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+      <c r="A70" s="9" t="inlineStr">
         <is>
           <t>Brandeis University</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B70" s="9" t="inlineStr">
         <is>
           <t>#69</t>
         </is>
@@ -1604,12 +2154,12 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="A71" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Tulane University of Louisiana </t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>#69</t>
         </is>
@@ -1621,12 +2171,12 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="A72" s="9" t="inlineStr">
         <is>
           <t>University of Connecticut</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B72" s="9" t="inlineStr">
         <is>
           <t>#69</t>
         </is>
@@ -1638,12 +2188,12 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="inlineStr">
+      <c r="A73" s="9" t="inlineStr">
         <is>
           <t>University of Pittsburgh</t>
         </is>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B73" s="9" t="inlineStr">
         <is>
           <t>#69</t>
         </is>
@@ -1655,12 +2205,12 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="A74" s="9" t="inlineStr">
         <is>
           <t>Binghamton University, SUNY</t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B74" s="9" t="inlineStr">
         <is>
           <t>#73</t>
         </is>
@@ -1672,12 +2222,12 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>Indiana University, Bloomington</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B75" s="9" t="inlineStr">
         <is>
           <t>#73</t>
         </is>
@@ -1689,12 +2239,12 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="A76" s="9" t="inlineStr">
         <is>
           <t>Clemson University</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B76" s="9" t="inlineStr">
         <is>
           <t>#75</t>
         </is>
@@ -1706,12 +2256,12 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="inlineStr">
+      <c r="A77" s="9" t="inlineStr">
         <is>
           <t>Rutgers University, Newark</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B77" s="9" t="inlineStr">
         <is>
           <t>#75</t>
         </is>
@@ -1723,12 +2273,12 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
+      <c r="A78" s="9" t="inlineStr">
         <is>
           <t>Syracuse University</t>
         </is>
       </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="B78" s="9" t="inlineStr">
         <is>
           <t>#75</t>
         </is>
@@ -1740,12 +2290,12 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="inlineStr">
+      <c r="A79" s="9" t="inlineStr">
         <is>
           <t>University at Buffalo, SUNY</t>
         </is>
       </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="B79" s="9" t="inlineStr">
         <is>
           <t>#75</t>
         </is>
@@ -1757,12 +2307,12 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
+      <c r="A80" s="9" t="inlineStr">
         <is>
           <t>University of California, Riverside</t>
         </is>
       </c>
-      <c r="B80" s="8" t="inlineStr">
+      <c r="B80" s="9" t="inlineStr">
         <is>
           <t>#75</t>
         </is>
@@ -1774,12 +2324,12 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="8" t="inlineStr">
+      <c r="A81" s="9" t="inlineStr">
         <is>
           <t>Colorado School of Mines</t>
         </is>
       </c>
-      <c r="B81" s="8" t="inlineStr">
+      <c r="B81" s="9" t="inlineStr">
         <is>
           <t>#80</t>
         </is>
@@ -1791,12 +2341,12 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
+      <c r="A82" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drexel University </t>
         </is>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>#80</t>
         </is>
@@ -1808,12 +2358,12 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="inlineStr">
+      <c r="A83" s="9" t="inlineStr">
         <is>
           <t>New Jersy Institute of Technology</t>
         </is>
       </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="B83" s="9" t="inlineStr">
         <is>
           <t>#80</t>
         </is>
@@ -1825,12 +2375,12 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="inlineStr">
+      <c r="A84" s="9" t="inlineStr">
         <is>
           <t>Stevens Institute of Technology</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B84" s="9" t="inlineStr">
         <is>
           <t>#80</t>
         </is>
@@ -1842,12 +2392,12 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="inlineStr">
+      <c r="A85" s="9" t="inlineStr">
         <is>
           <t>Pepperdine University</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B85" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
@@ -1859,12 +2409,12 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="inlineStr">
+      <c r="A86" s="9" t="inlineStr">
         <is>
           <t>University of Illinois Chicago</t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B86" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
@@ -1876,12 +2426,12 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="inlineStr">
+      <c r="A87" s="9" t="inlineStr">
         <is>
           <t>Worcester Polytechnic Institute</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B87" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
@@ -1893,12 +2443,12 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="inlineStr">
+      <c r="A88" s="9" t="inlineStr">
         <is>
           <t>Yashiva University</t>
         </is>
       </c>
-      <c r="B88" s="8" t="inlineStr">
+      <c r="B88" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
@@ -1910,12 +2460,12 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="inlineStr">
+      <c r="A89" s="9" t="inlineStr">
         <is>
           <t>American University</t>
         </is>
       </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="B89" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -1927,12 +2477,12 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="inlineStr">
+      <c r="A90" s="9" t="inlineStr">
         <is>
           <t>Baylor University</t>
         </is>
       </c>
-      <c r="B90" s="8" t="inlineStr">
+      <c r="B90" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -1944,12 +2494,12 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="inlineStr">
+      <c r="A91" s="9" t="inlineStr">
         <is>
           <t>Howard University</t>
         </is>
       </c>
-      <c r="B91" s="8" t="inlineStr">
+      <c r="B91" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -1961,12 +2511,12 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="inlineStr">
+      <c r="A92" s="9" t="inlineStr">
         <is>
           <t>Marquette University</t>
         </is>
       </c>
-      <c r="B92" s="8" t="inlineStr">
+      <c r="B92" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -1978,12 +2528,12 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="inlineStr">
+      <c r="A93" s="9" t="inlineStr">
         <is>
           <t>Rochester Institute of Technology</t>
         </is>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B93" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -1995,12 +2545,12 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
+      <c r="A94" s="9" t="inlineStr">
         <is>
           <t>Southern Methodist University</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B94" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -2012,12 +2562,12 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="inlineStr">
+      <c r="A95" s="9" t="inlineStr">
         <is>
           <t>University of California Santa Cruz</t>
         </is>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B95" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -2029,12 +2579,12 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="8" t="inlineStr">
+      <c r="A96" s="9" t="inlineStr">
         <is>
           <t>University of Delaware</t>
         </is>
       </c>
-      <c r="B96" s="8" t="inlineStr">
+      <c r="B96" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -2046,12 +2596,12 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="inlineStr">
+      <c r="A97" s="9" t="inlineStr">
         <is>
           <t>University of South Florida</t>
         </is>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B97" s="9" t="inlineStr">
         <is>
           <t>#88</t>
         </is>
@@ -2063,12 +2613,12 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="inlineStr">
+      <c r="A98" s="9" t="inlineStr">
         <is>
           <t>Florida International University</t>
         </is>
       </c>
-      <c r="B98" s="8" t="inlineStr">
+      <c r="B98" s="9" t="inlineStr">
         <is>
           <t>#97</t>
         </is>
@@ -2080,12 +2630,12 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
+      <c r="A99" s="9" t="inlineStr">
         <is>
           <t>Fordham University</t>
         </is>
       </c>
-      <c r="B99" s="8" t="inlineStr">
+      <c r="B99" s="9" t="inlineStr">
         <is>
           <t>#97</t>
         </is>
@@ -2097,12 +2647,12 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="inlineStr">
+      <c r="A100" s="9" t="inlineStr">
         <is>
           <t>Rutgers University, Camden</t>
         </is>
       </c>
-      <c r="B100" s="8" t="inlineStr">
+      <c r="B100" s="9" t="inlineStr">
         <is>
           <t>#97</t>
         </is>
@@ -2114,12 +2664,12 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="inlineStr">
+      <c r="A101" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Texas Christian University </t>
         </is>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B101" s="9" t="inlineStr">
         <is>
           <t>#97</t>
         </is>
@@ -2131,12 +2681,12 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="inlineStr">
+      <c r="A102" s="9" t="inlineStr">
         <is>
           <t>University of Colorado Boulder</t>
         </is>
       </c>
-      <c r="B102" s="8" t="inlineStr">
+      <c r="B102" s="9" t="inlineStr">
         <is>
           <t>#97</t>
         </is>
@@ -2148,12 +2698,12 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="8" t="inlineStr">
+      <c r="A103" s="9" t="inlineStr">
         <is>
           <t>Auburn University</t>
         </is>
       </c>
-      <c r="B103" s="8" t="inlineStr">
+      <c r="B103" s="9" t="inlineStr">
         <is>
           <t>#102</t>
         </is>
@@ -2273,7 +2823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2304,12 +2854,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Williams College</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
@@ -2321,12 +2871,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Amherst College</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>#2</t>
         </is>
@@ -2338,12 +2888,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>United States Naval Academy</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>#3</t>
         </is>
@@ -2355,12 +2905,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Swarthmore College</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
@@ -2372,12 +2922,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Bowdoin College</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>#5</t>
         </is>
@@ -2389,29 +2939,29 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>United States Air Force Academy</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>#5</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Claremont McKenna College</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -2423,12 +2973,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Pomona College</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -2440,12 +2990,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Wellesley College</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -2457,12 +3007,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Carleton College</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>#10</t>
         </is>
@@ -2474,12 +3024,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Harvey Mudd College</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>#10</t>
         </is>
@@ -2491,29 +3041,29 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">United States Military Academy at West Point </t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>#10</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Barnard College</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2525,12 +3075,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Davidson College</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2542,12 +3092,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Grinnell College</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2559,12 +3109,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Hamilton College</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2576,12 +3126,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Middlebury College</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2593,12 +3143,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Smith College</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2610,12 +3160,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Vassar College</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2628,12 +3178,12 @@
       <c r="E20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Wesleyan University</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2645,12 +3195,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Washington and Lee Univeristy</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -2667,12 +3217,12 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Colgate Univeristy</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>#22</t>
         </is>
@@ -2684,12 +3234,12 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Univeristy of Richmond</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>#22</t>
         </is>
@@ -2701,12 +3251,12 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>Bates College</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>#24</t>
         </is>
@@ -2718,12 +3268,12 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Colby College</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>#24</t>
         </is>
@@ -2735,12 +3285,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Haverford College</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>#24</t>
         </is>
@@ -2752,12 +3302,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>College of the Holy Cross</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>#27</t>
         </is>
@@ -2769,12 +3319,12 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>Macalester College</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
@@ -2786,12 +3336,12 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Mount Holyoke College</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>#29</t>
         </is>
@@ -2803,12 +3353,12 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>Bryn Mawr College</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>#30</t>
         </is>
@@ -2820,12 +3370,12 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Bucknell University</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>#30</t>
         </is>
@@ -2837,12 +3387,12 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>Colorado College</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>#30</t>
         </is>
@@ -2854,12 +3404,12 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>Lafayette College</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>#30</t>
         </is>
@@ -2871,12 +3421,12 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="9" t="inlineStr">
         <is>
           <t>Denison University</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>#34</t>
         </is>
@@ -2888,12 +3438,12 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>Franklin &amp; Marshell College</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>#35</t>
         </is>
@@ -2905,12 +3455,12 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>Occidental College</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>#35</t>
         </is>
@@ -2922,12 +3472,12 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Pitzer College </t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
@@ -2939,12 +3489,12 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>Scripps College</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
@@ -2956,12 +3506,12 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>Skidmore College</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
@@ -2973,12 +3523,12 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Soka Univeristy of America</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
@@ -2990,12 +3540,12 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>Spelman College</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
@@ -3007,12 +3557,12 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>Trinity College</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
@@ -3024,12 +3574,12 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Trinity University </t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
@@ -3041,12 +3591,12 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>Union College</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
         <is>
           <t>#44</t>
         </is>
@@ -3058,12 +3608,12 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>Berea College</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B46" s="9" t="inlineStr">
         <is>
           <t>#45</t>
         </is>
@@ -3075,12 +3625,12 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>Dickinson College</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>#45</t>
         </is>
@@ -3092,12 +3642,12 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="A48" s="9" t="inlineStr">
         <is>
           <t>Furman Univeristy</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>#45</t>
         </is>
@@ -3109,12 +3659,12 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="A49" s="9" t="inlineStr">
         <is>
           <t>Kenyon College</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B49" s="9" t="inlineStr">
         <is>
           <t>#45</t>
         </is>
@@ -3126,12 +3676,12 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="A50" s="9" t="inlineStr">
         <is>
           <t>The Univeristy of the South</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>#45</t>
         </is>
@@ -3143,12 +3693,12 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>Connecticut College</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>#50</t>
         </is>
@@ -3160,12 +3710,12 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>Hillsdale College</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>#50</t>
         </is>
@@ -3177,612 +3727,612 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="inlineStr">
+      <c r="A53" s="9" t="inlineStr">
         <is>
           <t>St. Olaf College</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="9" t="inlineStr">
         <is>
           <t>#50</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>Wabash College</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B54" s="9" t="inlineStr">
         <is>
           <t>#50</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>Wheaton College</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B55" s="9" t="inlineStr">
         <is>
           <t>#50</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>Centre College</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B56" s="9" t="inlineStr">
         <is>
           <t>#55</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>Rhodes College</t>
         </is>
       </c>
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B57" s="9" t="inlineStr">
         <is>
           <t>#55</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="A58" s="9" t="inlineStr">
         <is>
           <t>Thomas Aquinas College</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B58" s="9" t="inlineStr">
         <is>
           <t>#55</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="inlineStr">
+      <c r="A59" s="9" t="inlineStr">
         <is>
           <t>DePauw University</t>
         </is>
       </c>
-      <c r="B59" s="8" t="inlineStr">
+      <c r="B59" s="9" t="inlineStr">
         <is>
           <t>#58</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+      <c r="A60" s="9" t="inlineStr">
         <is>
           <t>Gettysburg College</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B60" s="9" t="inlineStr">
         <is>
           <t>#58</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="8" t="inlineStr">
+      <c r="A61" s="9" t="inlineStr">
         <is>
           <t>Oberlin College</t>
         </is>
       </c>
-      <c r="B61" s="8" t="inlineStr">
+      <c r="B61" s="9" t="inlineStr">
         <is>
           <t>#58</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="8" t="inlineStr">
+      <c r="A62" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">St. Lawrence University </t>
         </is>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
         <is>
           <t>#58</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="8" t="inlineStr">
+      <c r="A63" s="9" t="inlineStr">
         <is>
           <t>Whitman College</t>
         </is>
       </c>
-      <c r="B63" s="8" t="inlineStr">
+      <c r="B63" s="9" t="inlineStr">
         <is>
           <t>#58</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="A64" s="9" t="inlineStr">
         <is>
           <t>Principia College</t>
         </is>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B64" s="9" t="inlineStr">
         <is>
           <t>#63</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="8" t="inlineStr">
+      <c r="A65" s="9" t="inlineStr">
         <is>
           <t>Reed College</t>
         </is>
       </c>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B65" s="9" t="inlineStr">
         <is>
           <t>#63</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="8" t="inlineStr">
+      <c r="A66" s="9" t="inlineStr">
         <is>
           <t>Lawrence University</t>
         </is>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B66" s="9" t="inlineStr">
         <is>
           <t>#65</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="inlineStr">
+      <c r="A67" s="9" t="inlineStr">
         <is>
           <t>Virginia Military Institute</t>
         </is>
       </c>
-      <c r="B67" s="8" t="inlineStr">
+      <c r="B67" s="9" t="inlineStr">
         <is>
           <t>#65</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="A68" s="9" t="inlineStr">
         <is>
           <t>Agnes Scott College</t>
         </is>
       </c>
-      <c r="B68" s="8" t="inlineStr">
+      <c r="B68" s="9" t="inlineStr">
         <is>
           <t>#67</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="A69" s="9" t="inlineStr">
         <is>
           <t>Kalamazoo College</t>
         </is>
       </c>
-      <c r="B69" s="8" t="inlineStr">
+      <c r="B69" s="9" t="inlineStr">
         <is>
           <t>#67</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="inlineStr">
+      <c r="A70" s="9" t="inlineStr">
         <is>
           <t>Wofford College</t>
         </is>
       </c>
-      <c r="B70" s="8" t="inlineStr">
+      <c r="B70" s="9" t="inlineStr">
         <is>
           <t>#67</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="8" t="inlineStr">
+      <c r="A71" s="9" t="inlineStr">
         <is>
           <t>Bard College</t>
         </is>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>#70</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="8" t="inlineStr">
+      <c r="A72" s="9" t="inlineStr">
         <is>
           <t>Gustavus Adolphus College</t>
         </is>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B72" s="9" t="inlineStr">
         <is>
           <t>#70</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="8" t="inlineStr">
+      <c r="A73" s="9" t="inlineStr">
         <is>
           <t>Muhlenberg College</t>
         </is>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B73" s="9" t="inlineStr">
         <is>
           <t>#70</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="A74" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">College of St. Benedict </t>
         </is>
       </c>
-      <c r="B74" s="8" t="inlineStr">
+      <c r="B74" s="9" t="inlineStr">
         <is>
           <t>#73</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>Hobart and William Smith Colleges</t>
         </is>
       </c>
-      <c r="B75" s="8" t="inlineStr">
+      <c r="B75" s="9" t="inlineStr">
         <is>
           <t>#73</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="A76" s="9" t="inlineStr">
         <is>
           <t>Lake Forest College</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B76" s="9" t="inlineStr">
         <is>
           <t>#75</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="8" t="inlineStr">
+      <c r="A77" s="9" t="inlineStr">
         <is>
           <t>Allegheny College</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B77" s="9" t="inlineStr">
         <is>
           <t>#76</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="8" t="inlineStr">
+      <c r="A78" s="9" t="inlineStr">
         <is>
           <t>The College of Wooster</t>
         </is>
       </c>
-      <c r="B78" s="8" t="inlineStr">
+      <c r="B78" s="9" t="inlineStr">
         <is>
           <t>#76</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="inlineStr">
+      <c r="A79" s="9" t="inlineStr">
         <is>
           <t>Earlham College</t>
         </is>
       </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="B79" s="9" t="inlineStr">
         <is>
           <t>#76</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
+      <c r="A80" s="9" t="inlineStr">
         <is>
           <t>Knox College</t>
         </is>
       </c>
-      <c r="B80" s="8" t="inlineStr">
+      <c r="B80" s="9" t="inlineStr">
         <is>
           <t>#76</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="8" t="inlineStr">
+      <c r="A81" s="9" t="inlineStr">
         <is>
           <t>Wheaton College</t>
         </is>
       </c>
-      <c r="B81" s="8" t="inlineStr">
+      <c r="B81" s="9" t="inlineStr">
         <is>
           <t>#76</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="8" t="inlineStr">
+      <c r="A82" s="9" t="inlineStr">
         <is>
           <t>Willamette University</t>
         </is>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>#76</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="8" t="inlineStr">
+      <c r="A83" s="9" t="inlineStr">
         <is>
           <t>Saint Johns University</t>
         </is>
       </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="B83" s="9" t="inlineStr">
         <is>
           <t>#82</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="inlineStr">
+      <c r="A84" s="9" t="inlineStr">
         <is>
           <t>Stonehill College</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B84" s="9" t="inlineStr">
         <is>
           <t>#82</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="8" t="inlineStr">
+      <c r="A85" s="9" t="inlineStr">
         <is>
           <t>Austin College</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B85" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="8" t="inlineStr">
+      <c r="A86" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Drew University </t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B86" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#84 </t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="inlineStr">
+      <c r="A87" s="9" t="inlineStr">
         <is>
           <t>Hope College</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B87" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="8" t="inlineStr">
+      <c r="A88" s="9" t="inlineStr">
         <is>
           <t>Saint Mary's College</t>
         </is>
       </c>
-      <c r="B88" s="8" t="inlineStr">
+      <c r="B88" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="8" t="inlineStr">
+      <c r="A89" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Southwestern Univeristy </t>
         </is>
       </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="B89" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="inlineStr">
+      <c r="A90" s="9" t="inlineStr">
         <is>
           <t>St. John's College (MD)</t>
         </is>
       </c>
-      <c r="B90" s="8" t="inlineStr">
+      <c r="B90" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="8" t="inlineStr">
+      <c r="A91" s="9" t="inlineStr">
         <is>
           <t>Ursinus College</t>
         </is>
       </c>
-      <c r="B91" s="8" t="inlineStr">
+      <c r="B91" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="8" t="inlineStr">
+      <c r="A92" s="9" t="inlineStr">
         <is>
           <t>Washington &amp; Jefferson College</t>
         </is>
       </c>
-      <c r="B92" s="8" t="inlineStr">
+      <c r="B92" s="9" t="inlineStr">
         <is>
           <t>#84</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="inlineStr">
+      <c r="A93" s="9" t="inlineStr">
         <is>
           <t>Beloit College</t>
         </is>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B93" s="9" t="inlineStr">
         <is>
           <t>#92</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
+      <c r="A94" s="9" t="inlineStr">
         <is>
           <t>Juniata College</t>
         </is>
       </c>
-      <c r="B94" s="8" t="inlineStr">
+      <c r="B94" s="9" t="inlineStr">
         <is>
           <t>#92</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="inlineStr">
+      <c r="A95" s="9" t="inlineStr">
         <is>
           <t>Washington College</t>
         </is>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B95" s="9" t="inlineStr">
         <is>
           <t>#92</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="8" t="inlineStr">
+      <c r="A96" s="9" t="inlineStr">
         <is>
           <t>Whittier College</t>
         </is>
       </c>
-      <c r="B96" s="8" t="inlineStr">
+      <c r="B96" s="9" t="inlineStr">
         <is>
           <t>#92</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="8" t="inlineStr">
+      <c r="A97" s="9" t="inlineStr">
         <is>
           <t>Augustana College</t>
         </is>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B97" s="9" t="inlineStr">
         <is>
           <t>#96</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="inlineStr">
+      <c r="A98" s="9" t="inlineStr">
         <is>
           <t>Lewis &amp; Clark College</t>
         </is>
       </c>
-      <c r="B98" s="8" t="inlineStr">
+      <c r="B98" s="9" t="inlineStr">
         <is>
           <t>#96</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="8" t="inlineStr">
+      <c r="A99" s="9" t="inlineStr">
         <is>
           <t>Lycoming College</t>
         </is>
       </c>
-      <c r="B99" s="8" t="inlineStr">
+      <c r="B99" s="9" t="inlineStr">
         <is>
           <t>#96</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="8" t="inlineStr">
+      <c r="A100" s="9" t="inlineStr">
         <is>
           <t>Morehouse College</t>
         </is>
       </c>
-      <c r="B100" s="8" t="inlineStr">
+      <c r="B100" s="9" t="inlineStr">
         <is>
           <t>#96</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="8" t="inlineStr">
+      <c r="A101" s="9" t="inlineStr">
         <is>
           <t>Randolph-Macon College</t>
         </is>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B101" s="9" t="inlineStr">
         <is>
           <t>#96</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="8" t="inlineStr">
+      <c r="A102" s="9" t="inlineStr">
         <is>
           <t>Saint Anselm College</t>
         </is>
       </c>
-      <c r="B102" s="8" t="inlineStr">
+      <c r="B102" s="9" t="inlineStr">
         <is>
           <t>#96</t>
         </is>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="8" t="inlineStr">
+      <c r="A103" s="9" t="inlineStr">
         <is>
           <t>St. Mary's College of Maryland</t>
         </is>
       </c>
-      <c r="B103" s="8" t="inlineStr">
+      <c r="B103" s="9" t="inlineStr">
         <is>
           <t>#96</t>
         </is>
@@ -3845,7 +4395,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3881,7 +4431,7 @@
           <t>University of California, Berkeley</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
@@ -3894,12 +4444,12 @@
       <c r="D2" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>University of California, Los Angeles</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>#2</t>
         </is>
@@ -3916,7 +4466,7 @@
           <t>University of Michigan--Ann Arbor</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>#3</t>
         </is>
@@ -3933,7 +4483,7 @@
           <t>University of North Carolina--Chapel Hill</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
@@ -3945,12 +4495,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>University of Virginia</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
@@ -3962,12 +4512,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>University of California San Diego</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>#6</t>
         </is>
@@ -3979,12 +4529,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>University of Florida</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -4001,7 +4551,7 @@
           <t>The University of Texas--Austin</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
@@ -4013,12 +4563,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Georgia Institute of Technology</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#9 </t>
         </is>
@@ -4035,7 +4585,7 @@
           <t>University of California, Davis</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#9 </t>
         </is>
@@ -4052,7 +4602,7 @@
           <t>University of California, Irvine</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">#9 </t>
         </is>
@@ -4064,12 +4614,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>University of Illinois Urbana-Champaign</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>#12</t>
         </is>
@@ -4081,12 +4631,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>University of Wisconsin--Madison</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>#12</t>
         </is>
@@ -4098,12 +4648,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>University of California, Santa Barbara</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>#14</t>
         </is>
@@ -4120,7 +4670,7 @@
           <t>The Ohio State University</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>#15</t>
         </is>
@@ -4132,12 +4682,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Rutgers University--New Brunswick</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>#16</t>
         </is>
@@ -4154,7 +4704,7 @@
           <t>University of Maryland, College Park</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>#16</t>
         </is>
@@ -4166,12 +4716,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>University of Washington</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>#16</t>
         </is>
@@ -4183,12 +4733,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Purdue University--Main Campus</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>#19</t>
         </is>
@@ -4200,12 +4750,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>University of Georgia</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>#19</t>
         </is>
@@ -4244,7 +4794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -4275,12 +4825,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Texas Christian University </t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
@@ -4292,12 +4842,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Southern Methodist Univeristy </t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>#2</t>
         </is>
@@ -4309,12 +4859,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>College of the Ozarks</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>#3</t>
         </is>
@@ -4326,12 +4876,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>St. Olaf College</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
@@ -4343,12 +4893,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Oklahoma City Univeristy </t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>#5</t>
         </is>
@@ -4360,12 +4910,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Wheaton College--Illinois</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>#6</t>
         </is>
@@ -4377,29 +4927,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Moody Bible Institute</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>#7</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Newspaper was the "The Moody Standard" but was discontinued in 2019</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Harding Univeristy </t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>#8</t>
         </is>
@@ -4411,12 +4961,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Biola Univeristy </t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>#9</t>
         </is>
@@ -4428,12 +4978,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Union Univeristy</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>#10</t>
         </is>
@@ -4445,12 +4995,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Hope College</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>#11</t>
         </is>
@@ -4462,12 +5012,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Baylor Univeristy</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>#12</t>
         </is>
@@ -4479,12 +5029,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Lipscomb Univeristy</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>#13</t>
         </is>
@@ -4496,12 +5046,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Point Loma Nazarene Univeristy</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>#14</t>
         </is>
@@ -4513,12 +5063,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>California Baptist University</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>#15</t>
         </is>
@@ -4530,12 +5080,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Cedarville University</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>#16</t>
         </is>

</xml_diff>

<commit_message>
Add Swarthmore, Occidental, and Lipscomb as the next open WordPress wave.
These sites reuse the generic adapter and avoid extra Cloudflare load on the server IP.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Christian Colleges" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$J$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -120,6 +120,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -395,7 +396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="19" min="1" max="1"/>
@@ -406,7 +407,8 @@
     <col width="12" customWidth="1" style="19" min="6" max="6"/>
     <col width="12" customWidth="1" style="19" min="7" max="7"/>
     <col width="12" customWidth="1" style="19" min="8" max="8"/>
-    <col width="56" customWidth="1" style="19" min="9" max="9"/>
+    <col width="12" customWidth="1" style="19" min="9" max="9"/>
+    <col width="64" customWidth="1" style="19" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,15 +444,20 @@
       </c>
       <c r="G1" s="20" t="inlineStr">
         <is>
+          <t>articles</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
           <t>machine</t>
         </is>
       </c>
-      <c r="H1" s="20" t="inlineStr">
+      <c r="I1" s="20" t="inlineStr">
         <is>
           <t>started</t>
         </is>
       </c>
-      <c r="I1" s="20" t="inlineStr">
+      <c r="J1" s="20" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -487,17 +494,17 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="H2" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="I2" s="0" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="I2" s="0" t="inlineStr">
+      <c r="J2" s="0" t="inlineStr">
         <is>
           <t>newspaper-scraper@chicago</t>
         </is>
@@ -534,17 +541,17 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G3" s="0" t="inlineStr">
+      <c r="H3" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H3" s="0" t="inlineStr">
+      <c r="I3" s="0" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="I3" s="0" t="inlineStr">
+      <c r="J3" s="0" t="inlineStr">
         <is>
           <t>newspaper-scraper@northwestern</t>
         </is>
@@ -581,17 +588,17 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G4" s="0" t="inlineStr">
+      <c r="H4" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H4" s="0" t="inlineStr">
+      <c r="I4" s="0" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="I4" s="0" t="inlineStr">
+      <c r="J4" s="0" t="inlineStr">
         <is>
           <t>newspaper-scraper@smu</t>
         </is>
@@ -628,17 +635,17 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G5" s="0" t="inlineStr">
+      <c r="H5" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H5" s="0" t="inlineStr">
+      <c r="I5" s="0" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="I5" s="0" t="inlineStr">
+      <c r="J5" s="0" t="inlineStr">
         <is>
           <t>newspaper-scraper@tcu</t>
         </is>
@@ -675,19 +682,19 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G6" s="0" t="inlineStr">
+      <c r="H6" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H6" s="0" t="inlineStr">
+      <c r="I6" s="0" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="I6" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@biola; high empty_body on old archive</t>
+      <c r="J6" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@biola; resumed after href crash fix</t>
         </is>
       </c>
     </row>
@@ -722,19 +729,22 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G7" s="0" t="inlineStr">
+      <c r="G7" s="21" t="n">
+        <v>1604</v>
+      </c>
+      <c r="H7" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H7" s="0" t="inlineStr">
+      <c r="I7" s="0" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="I7" s="0" t="inlineStr">
-        <is>
-          <t>Finished: 1604 articles of 1626 URLs; 44 empty_body skipped. systemd exited 0 and stayed inactive (Restart=on-failure).</t>
+      <c r="J7" s="0" t="inlineStr">
+        <is>
+          <t>Finished. 1604 articles (44 empty_body skipped). Downloaded separately if needed.</t>
         </is>
       </c>
     </row>
@@ -766,22 +776,25 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G8" s="0" t="inlineStr">
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H8" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H8" s="0" t="inlineStr">
+      <c r="I8" s="0" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="I8" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@stolaf; near complete</t>
+      <c r="J8" s="0" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); rest empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
         </is>
       </c>
     </row>
@@ -813,22 +826,22 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>testing</t>
-        </is>
-      </c>
-      <c r="G9" s="0" t="inlineStr">
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H9" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H9" s="0" t="inlineStr">
+      <c r="I9" s="0" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="I9" s="0" t="inlineStr">
-        <is>
-          <t>200-article test; not a full run yet</t>
+      <c r="J9" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@conncoll full run</t>
         </is>
       </c>
     </row>
@@ -860,22 +873,22 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>testing</t>
-        </is>
-      </c>
-      <c r="G10" s="0" t="inlineStr">
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H10" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H10" s="0" t="inlineStr">
+      <c r="I10" s="0" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="I10" s="0" t="inlineStr">
-        <is>
-          <t>200-article test; not a full run yet</t>
+      <c r="J10" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@fandm full run</t>
         </is>
       </c>
     </row>
@@ -907,27 +920,168 @@
       </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H11" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J11" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@hillsdale full run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>testing</t>
         </is>
       </c>
-      <c r="G11" s="0" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="H11" s="0" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="I11" s="0" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>200-article test; not a full run yet</t>
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Occidental College</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>The Occidental</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>occidental</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>theoccidentalnews.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>testing</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>200-article test; not a full run yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lipscomb University</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lipscomb Media</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>lipscomb</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>lipscombmedia.com</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>testing</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>200-article test; not a full run yet</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I11"/>
+  <autoFilter ref="A1:J14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Skip pre-2000 permalinks before fetching so Swarthmore does not crawl the 1990s.
A 200-URL test spent every request on 1998 pages and wrote zero rows; URL-dated years can be dropped without a GET.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -494,6 +494,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G2" s="21" t="n">
+        <v>14400</v>
+      </c>
       <c r="H2" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -506,7 +509,7 @@
       </c>
       <c r="J2" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@chicago</t>
+          <t>newspaper-scraper@chicago; 14400/22493 at last check</t>
         </is>
       </c>
     </row>
@@ -541,6 +544,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G3" s="21" t="n">
+        <v>17400</v>
+      </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -553,7 +559,7 @@
       </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@northwestern</t>
+          <t>newspaper-scraper@northwestern; 17400/70720; 403s still 32</t>
         </is>
       </c>
     </row>
@@ -588,6 +594,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G4" s="21" t="n">
+        <v>8800</v>
+      </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -600,7 +609,7 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@smu</t>
+          <t>newspaper-scraper@smu; 8800/26572 at last check</t>
         </is>
       </c>
     </row>
@@ -635,6 +644,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G5" s="21" t="n">
+        <v>8546</v>
+      </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -647,7 +659,7 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tcu</t>
+          <t>newspaper-scraper@tcu; 8546/26172 at last check</t>
         </is>
       </c>
     </row>
@@ -682,6 +694,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G6" s="21" t="n">
+        <v>5150</v>
+      </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -694,7 +709,7 @@
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@biola; resumed after href crash fix</t>
+          <t>newspaper-scraper@biola; 5150/11390 after href fix</t>
         </is>
       </c>
     </row>
@@ -744,7 +759,7 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t>Finished. 1604 articles (44 empty_body skipped). Downloaded separately if needed.</t>
+          <t>Finished. 1604 articles of 1626 URLs; 44 empty_body skipped.</t>
         </is>
       </c>
     </row>
@@ -794,7 +809,7 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); rest empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
         </is>
       </c>
     </row>
@@ -829,6 +844,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G9" s="21" t="n">
+        <v>3098</v>
+      </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -841,7 +859,7 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@conncoll full run</t>
+          <t>newspaper-scraper@conncoll; 3098/4320 at last check</t>
         </is>
       </c>
     </row>
@@ -876,6 +894,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G10" s="21" t="n">
+        <v>1946</v>
+      </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -888,7 +909,7 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@fandm full run</t>
+          <t>newspaper-scraper@fandm; 1946/3583 at last check</t>
         </is>
       </c>
     </row>
@@ -923,6 +944,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G11" s="21" t="n">
+        <v>3393</v>
+      </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -935,148 +959,157 @@
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@hillsdale full run</t>
+          <t>newspaper-scraper@hillsdale; 3393/15690 at last check</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>Swarthmore College</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>The Phoenix</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>swarthmore</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>swarthmorephoenix.com</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="0" t="inlineStr">
         <is>
           <t>testing</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="0" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>200-article test; not a full run yet</t>
+      <c r="J12" s="0" t="inlineStr">
+        <is>
+          <t>200-test wrote 0: first 200 URLs were 1998 (pre-2000 skip). Wait for URL-skip fix before full run.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>Occidental College</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>The Occidental</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>occidental</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>theoccidentalnews.com</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t>testing</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="G13" t="n">
+        <v>183</v>
+      </c>
+      <c r="H13" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="0" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>200-article test; not a full run yet</t>
+      <c r="J13" s="0" t="inlineStr">
+        <is>
+          <t>200-test done: 183 articles. Ready for systemd full run.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>Lipscomb University</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>Lipscomb Media</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>lipscomb</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>lipscombmedia.com</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="0" t="inlineStr">
         <is>
           <t>testing</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="G14" t="n">
+        <v>186</v>
+      </c>
+      <c r="H14" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="0" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>200-article test; not a full run yet</t>
+      <c r="J14" s="0" t="inlineStr">
+        <is>
+          <t>200-test done: 186 articles. Ready for systemd full run.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add four open papers to start Public Universities coverage.
Michigan Daily and UC Irvine fill the empty Public tab; Miami and RIT add National papers without more Cloudflare load.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="11">
     <font>
       <name val="Arial"/>
@@ -94,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -121,6 +123,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -396,7 +402,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="19" min="1" max="1"/>
@@ -495,7 +501,7 @@
         </is>
       </c>
       <c r="G2" s="21" t="n">
-        <v>14400</v>
+        <v>20750</v>
       </c>
       <c r="H2" s="0" t="inlineStr">
         <is>
@@ -509,7 +515,7 @@
       </c>
       <c r="J2" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@chicago; 14400/22493 at last check</t>
+          <t>newspaper-scraper@chicago; 20750/22493 at 2026-09-28 15:48 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +551,7 @@
         </is>
       </c>
       <c r="G3" s="21" t="n">
-        <v>17400</v>
+        <v>21000</v>
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
@@ -559,7 +565,7 @@
       </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@northwestern; 17400/70720; 403s still 32</t>
+          <t>newspaper-scraper@northwestern; 21000/70720 at 2026-09-28 15:48 UTC; 403s still 32, network_error=1083</t>
         </is>
       </c>
     </row>
@@ -595,7 +601,7 @@
         </is>
       </c>
       <c r="G4" s="21" t="n">
-        <v>8800</v>
+        <v>12650</v>
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
@@ -609,7 +615,7 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@smu; 8800/26572 at last check</t>
+          <t>newspaper-scraper@smu; 12650/26572 at 2026-09-28 15:48 UTC</t>
         </is>
       </c>
     </row>
@@ -645,7 +651,7 @@
         </is>
       </c>
       <c r="G5" s="21" t="n">
-        <v>8546</v>
+        <v>12296</v>
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
@@ -659,7 +665,7 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tcu; 8546/26172 at last check</t>
+          <t>newspaper-scraper@tcu; 12296/26172 at 2026-09-28 15:48 UTC</t>
         </is>
       </c>
     </row>
@@ -695,7 +701,7 @@
         </is>
       </c>
       <c r="G6" s="21" t="n">
-        <v>5150</v>
+        <v>9000</v>
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
@@ -709,7 +715,7 @@
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@biola; 5150/11390 after href fix</t>
+          <t>newspaper-scraper@biola; 9000/11390 at 2026-09-28 15:48 UTC</t>
         </is>
       </c>
     </row>
@@ -841,11 +847,11 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G9" s="21" t="n">
-        <v>3098</v>
+        <v>4039</v>
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
@@ -859,7 +865,7 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@conncoll; 3098/4320 at last check</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
         </is>
       </c>
     </row>
@@ -891,11 +897,11 @@
       </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G10" s="21" t="n">
-        <v>1946</v>
+        <v>3449</v>
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
@@ -909,7 +915,7 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@fandm; 1946/3583 at last check</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
         </is>
       </c>
     </row>
@@ -945,7 +951,7 @@
         </is>
       </c>
       <c r="G11" s="21" t="n">
-        <v>3393</v>
+        <v>9793</v>
       </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
@@ -959,7 +965,7 @@
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@hillsdale; 3393/15690 at last check</t>
+          <t>newspaper-scraper@hillsdale; 9793/15690 at 2026-09-28 15:48 UTC</t>
         </is>
       </c>
     </row>
@@ -991,11 +997,11 @@
       </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
-          <t>testing</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
@@ -1009,7 +1015,7 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t>200-test wrote 0: first 200 URLs were 1998 (pre-2000 skip). Wait for URL-skip fix before full run.</t>
+          <t>newspaper-scraper@swarthmore; 700/13251 at 2026-09-28 15:48 UTC; pre_2000 skip working (578 skipped)</t>
         </is>
       </c>
     </row>
@@ -1041,11 +1047,11 @@
       </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
-          <t>testing</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>183</v>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="n">
+        <v>783</v>
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
@@ -1059,7 +1065,7 @@
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t>200-test done: 183 articles. Ready for systemd full run.</t>
+          <t>newspaper-scraper@occidental; 783/10055 at 2026-09-28 15:48 UTC</t>
         </is>
       </c>
     </row>
@@ -1091,11 +1097,11 @@
       </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
-          <t>testing</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>186</v>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="n">
+        <v>682</v>
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
@@ -1109,7 +1115,191 @@
       </c>
       <c r="J14" s="0" t="inlineStr">
         <is>
-          <t>200-test done: 186 articles. Ready for systemd full run.</t>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>University of Michigan</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>The Michigan Daily</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>michigan</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>michigandaily.com</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Wave 4. Open WordPress. Probe + 200-test before full run. ~120k URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>University of California, Irvine</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>New University</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>uci</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>newuniversity.org</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="n"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Wave 4. Open WordPress. 200-test required: recon empty on 2003-04 URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>University of Miami</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>The Miami Hurricane</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>miami</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>themiamihurricane.com</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Wave 4. Open WordPress behind Sucuri. Probe + 200-test before full run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rochester Institute of Technology</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Reporter</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>rit</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>reporter.rit.edu</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Wave 4. Open SNO, Crawl-delay 6. Probe + 200-test before full run.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Point Loma and UC Santa Cruz after Chicago and RIT finished.
These two open WordPress papers refill the 12-scraper cap without more Cloudflare load, and the Status tab now records Chicago (22,117) and RIT (2,137) as done.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -9,19 +9,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Universities" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Christian Colleges" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status'!$A$1:$J$14</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -75,8 +74,18 @@
     <font>
       <b val="1"/>
     </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +98,11 @@
         <bgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F4F6F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -96,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -127,6 +141,38 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,909 +448,1052 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" style="19" min="1" max="1"/>
+    <col width="34" customWidth="1" style="19" min="1" max="1"/>
     <col width="26" customWidth="1" style="19" min="2" max="2"/>
     <col width="14" customWidth="1" style="19" min="3" max="3"/>
     <col width="28" customWidth="1" style="19" min="4" max="4"/>
-    <col width="42" customWidth="1" style="19" min="5" max="5"/>
+    <col width="44" customWidth="1" style="19" min="5" max="5"/>
     <col width="12" customWidth="1" style="19" min="6" max="6"/>
     <col width="12" customWidth="1" style="19" min="7" max="7"/>
     <col width="12" customWidth="1" style="19" min="8" max="8"/>
     <col width="12" customWidth="1" style="19" min="9" max="9"/>
-    <col width="64" customWidth="1" style="19" min="10" max="10"/>
+    <col width="80" customWidth="1" style="19" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>university</t>
         </is>
       </c>
-      <c r="B1" s="20" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>paper</t>
         </is>
       </c>
-      <c r="C1" s="20" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>site_key</t>
         </is>
       </c>
-      <c r="D1" s="20" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="E1" s="20" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" s="20" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="G1" s="20" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>articles</t>
         </is>
       </c>
-      <c r="H1" s="20" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>machine</t>
         </is>
       </c>
-      <c r="I1" s="20" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>started</t>
         </is>
       </c>
-      <c r="J1" s="20" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="0" t="inlineStr">
+      <c r="A2" s="32" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="B2" s="32" t="n"/>
+      <c r="C2" s="32" t="n"/>
+      <c r="D2" s="32" t="n"/>
+      <c r="E2" s="32" t="n"/>
+      <c r="F2" s="32" t="n"/>
+      <c r="G2" s="32" t="n"/>
+      <c r="H2" s="32" t="n"/>
+      <c r="I2" s="32" t="n"/>
+      <c r="J2" s="32" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Rochester Institute of Technology</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Reporter</t>
+        </is>
+      </c>
+      <c r="C3" s="33" t="inlineStr">
+        <is>
+          <t>rit</t>
+        </is>
+      </c>
+      <c r="D3" s="33" t="inlineStr">
+        <is>
+          <t>reporter.rit.edu</t>
+        </is>
+      </c>
+      <c r="E3" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F3" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G3" s="30" t="n">
+        <v>2137</v>
+      </c>
+      <c r="H3" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I3" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J3" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 2137 articles of 2140 URLs (99.9%); 5 empty_body. systemd inactive. File: ~/Downloads/rit.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>University of Chicago</t>
         </is>
       </c>
-      <c r="B2" s="0" t="inlineStr">
+      <c r="B4" s="33" t="inlineStr">
         <is>
           <t>The Chicago Maroon</t>
         </is>
       </c>
-      <c r="C2" s="0" t="inlineStr">
+      <c r="C4" s="33" t="inlineStr">
         <is>
           <t>chicago</t>
         </is>
       </c>
-      <c r="D2" s="0" t="inlineStr">
+      <c r="D4" s="33" t="inlineStr">
         <is>
           <t>chicagomaroon.com</t>
         </is>
       </c>
-      <c r="E2" s="0" t="inlineStr">
+      <c r="E4" s="33" t="inlineStr">
         <is>
           <t>National Universities</t>
         </is>
       </c>
-      <c r="F2" s="0" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="n">
+        <v>22117</v>
+      </c>
+      <c r="H4" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I4" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J4" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 22117 articles of 22493 URLs (98.3%); 371 empty_body, 2 http_301, 3 http_404. systemd inactive. File: ~/Downloads/chicago.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Northwestern University</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Northwestern</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>northwestern</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
+        <is>
+          <t>dailynorthwestern.com</t>
+        </is>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F5" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G2" s="21" t="n">
-        <v>20750</v>
-      </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="G5" s="33" t="n"/>
+      <c r="H5" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I2" s="0" t="inlineStr">
+      <c r="I5" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="J5" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@northwestern; 403s still present at last check</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>University of Miami</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>The Miami Hurricane</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>miami</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>themiamihurricane.com</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="n"/>
+      <c r="H6" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I6" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J6" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@miami; full run started 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>University of California, Santa Cruz</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>City on a Hill Press</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>ucsc</t>
+        </is>
+      </c>
+      <c r="D7" s="33" t="inlineStr">
+        <is>
+          <t>cityonahillpress.com</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F7" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="n"/>
+      <c r="H7" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I7" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J7" s="34" t="inlineStr">
+        <is>
+          <t>Wave 5. Open WordPress. Probe + 200-test before full run. ~7k URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>Public Universities</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="n"/>
+      <c r="C8" s="32" t="n"/>
+      <c r="D8" s="32" t="n"/>
+      <c r="E8" s="32" t="n"/>
+      <c r="F8" s="32" t="n"/>
+      <c r="G8" s="32" t="n"/>
+      <c r="H8" s="32" t="n"/>
+      <c r="I8" s="32" t="n"/>
+      <c r="J8" s="32" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>University of California, Irvine</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>New University</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>uci</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>newuniversity.org</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F9" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="n"/>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J9" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@uci; full run started 2026-09-28 after td-post-content fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>University of Michigan</t>
+        </is>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>The Michigan Daily</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>michigan</t>
+        </is>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>michigandaily.com</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="n"/>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I10" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J10" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@michigan; full run started 2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="n"/>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="32" t="n"/>
+      <c r="F11" s="32" t="n"/>
+      <c r="G11" s="32" t="n"/>
+      <c r="H11" s="32" t="n"/>
+      <c r="I11" s="32" t="n"/>
+      <c r="J11" s="32" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Connecticut College</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>The College Voice</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>conncoll</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>thecollegevoice.org</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="n">
+        <v>4039</v>
+      </c>
+      <c r="H12" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I12" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J12" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Franklin &amp; Marshall College</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>The College Reporter</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>fandm</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>the-college-reporter.com</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G13" s="30" t="n">
+        <v>3449</v>
+      </c>
+      <c r="H13" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I13" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J13" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I14" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Union College (NY)</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>Concordiensis</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>union</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>concordiensis.com</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G15" s="30" t="n">
+        <v>1604</v>
+      </c>
+      <c r="H15" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I15" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J15" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 1604 articles of 1626 URLs; 44 empty_body skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>Hillsdale College</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>The Collegian</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>hillsdale</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>hillsdalecollegian.com</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G16" s="33" t="n"/>
+      <c r="H16" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I16" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J16" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@hillsdale</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>Occidental College</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>The Occidental</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>occidental</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>theoccidentalnews.com</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="n"/>
+      <c r="H17" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I17" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J17" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@occidental</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D18" s="33" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F18" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G18" s="33" t="n"/>
+      <c r="H18" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I18" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J18" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@swarthmore; pre-2000 permalinks skipped without fetch</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="32" t="n"/>
+      <c r="H19" s="32" t="n"/>
+      <c r="I19" s="32" t="n"/>
+      <c r="J19" s="32" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Lipscomb University</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>Lipscomb Media</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>lipscomb</t>
+        </is>
+      </c>
+      <c r="D20" s="33" t="inlineStr">
+        <is>
+          <t>lipscombmedia.com</t>
+        </is>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G20" s="30" t="n">
+        <v>682</v>
+      </c>
+      <c r="H20" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I20" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J20" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Biola University</t>
+        </is>
+      </c>
+      <c r="B21" s="33" t="inlineStr">
+        <is>
+          <t>The Chimes</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>biola</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>chimesnewspaper.com</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I21" s="33" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J2" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@chicago; 20750/22493 at 2026-09-28 15:48 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="0" t="inlineStr">
-        <is>
-          <t>Northwestern University</t>
-        </is>
-      </c>
-      <c r="B3" s="0" t="inlineStr">
-        <is>
-          <t>The Daily Northwestern</t>
-        </is>
-      </c>
-      <c r="C3" s="0" t="inlineStr">
-        <is>
-          <t>northwestern</t>
-        </is>
-      </c>
-      <c r="D3" s="0" t="inlineStr">
-        <is>
-          <t>dailynorthwestern.com</t>
-        </is>
-      </c>
-      <c r="E3" s="0" t="inlineStr">
-        <is>
-          <t>National Universities</t>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
+      <c r="J21" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@biola; recovered after href fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>Southern Methodist University</t>
+        </is>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Campus</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>smu</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="inlineStr">
+        <is>
+          <t>smudailycampus.com</t>
+        </is>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F22" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G3" s="21" t="n">
-        <v>21000</v>
-      </c>
-      <c r="H3" s="0" t="inlineStr">
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I3" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="J3" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@northwestern; 21000/70720 at 2026-09-28 15:48 UTC; 403s still 32, network_error=1083</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="0" t="inlineStr">
-        <is>
-          <t>Southern Methodist University</t>
-        </is>
-      </c>
-      <c r="B4" s="0" t="inlineStr">
-        <is>
-          <t>The Daily Campus</t>
-        </is>
-      </c>
-      <c r="C4" s="0" t="inlineStr">
-        <is>
-          <t>smu</t>
-        </is>
-      </c>
-      <c r="D4" s="0" t="inlineStr">
-        <is>
-          <t>smudailycampus.com</t>
-        </is>
-      </c>
-      <c r="E4" s="0" t="inlineStr">
+      <c r="I22" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J22" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@smu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>Texas Christian University</t>
+        </is>
+      </c>
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t>TCU 360</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>tcu</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="inlineStr">
+        <is>
+          <t>tcu360.com</t>
+        </is>
+      </c>
+      <c r="E23" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F4" s="0" t="inlineStr">
+      <c r="F23" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G4" s="21" t="n">
-        <v>12650</v>
-      </c>
-      <c r="H4" s="0" t="inlineStr">
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I4" s="0" t="inlineStr">
+      <c r="I23" s="33" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J4" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@smu; 12650/26572 at 2026-09-28 15:48 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="0" t="inlineStr">
-        <is>
-          <t>Texas Christian University</t>
-        </is>
-      </c>
-      <c r="B5" s="0" t="inlineStr">
-        <is>
-          <t>TCU 360</t>
-        </is>
-      </c>
-      <c r="C5" s="0" t="inlineStr">
-        <is>
-          <t>tcu</t>
-        </is>
-      </c>
-      <c r="D5" s="0" t="inlineStr">
-        <is>
-          <t>tcu360.com</t>
-        </is>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
-        <is>
-          <t>Christian Colleges | National Universities</t>
-        </is>
-      </c>
-      <c r="F5" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G5" s="21" t="n">
-        <v>12296</v>
-      </c>
-      <c r="H5" s="0" t="inlineStr">
+      <c r="J23" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tcu</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>Point Loma Nazarene University</t>
+        </is>
+      </c>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>Loma Beat</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat.com</t>
+        </is>
+      </c>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F24" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="n"/>
+      <c r="H24" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I5" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J5" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@tcu; 12296/26172 at 2026-09-28 15:48 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="0" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B6" s="0" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C6" s="0" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D6" s="0" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E6" s="0" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F6" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G6" s="21" t="n">
-        <v>9000</v>
-      </c>
-      <c r="H6" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I6" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J6" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@biola; 9000/11390 at 2026-09-28 15:48 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="0" t="inlineStr">
-        <is>
-          <t>Union College (NY)</t>
-        </is>
-      </c>
-      <c r="B7" s="0" t="inlineStr">
-        <is>
-          <t>Concordiensis</t>
-        </is>
-      </c>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t>union</t>
-        </is>
-      </c>
-      <c r="D7" s="0" t="inlineStr">
-        <is>
-          <t>concordiensis.com</t>
-        </is>
-      </c>
-      <c r="E7" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F7" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G7" s="21" t="n">
-        <v>1604</v>
-      </c>
-      <c r="H7" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I7" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J7" s="0" t="inlineStr">
-        <is>
-          <t>Finished. 1604 articles of 1626 URLs; 44 empty_body skipped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="0" t="inlineStr">
-        <is>
-          <t>St. Olaf College</t>
-        </is>
-      </c>
-      <c r="B8" s="0" t="inlineStr">
-        <is>
-          <t>Manitou Messenger</t>
-        </is>
-      </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t>stolaf</t>
-        </is>
-      </c>
-      <c r="D8" s="0" t="inlineStr">
-        <is>
-          <t>olafmessenger.com</t>
-        </is>
-      </c>
-      <c r="E8" s="0" t="inlineStr">
-        <is>
-          <t>Christian Colleges | Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F8" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G8" s="21" t="n">
-        <v>5048</v>
-      </c>
-      <c r="H8" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I8" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J8" s="0" t="inlineStr">
-        <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="0" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B9" s="0" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C9" s="0" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D9" s="0" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E9" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F9" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G9" s="21" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H9" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I9" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J9" s="0" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="0" t="inlineStr">
-        <is>
-          <t>Franklin &amp; Marshall College</t>
-        </is>
-      </c>
-      <c r="B10" s="0" t="inlineStr">
-        <is>
-          <t>The College Reporter</t>
-        </is>
-      </c>
-      <c r="C10" s="0" t="inlineStr">
-        <is>
-          <t>fandm</t>
-        </is>
-      </c>
-      <c r="D10" s="0" t="inlineStr">
-        <is>
-          <t>the-college-reporter.com</t>
-        </is>
-      </c>
-      <c r="E10" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F10" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G10" s="21" t="n">
-        <v>3449</v>
-      </c>
-      <c r="H10" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I10" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J10" s="0" t="inlineStr">
-        <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0" t="inlineStr">
-        <is>
-          <t>Hillsdale College</t>
-        </is>
-      </c>
-      <c r="B11" s="0" t="inlineStr">
-        <is>
-          <t>The Collegian</t>
-        </is>
-      </c>
-      <c r="C11" s="0" t="inlineStr">
-        <is>
-          <t>hillsdale</t>
-        </is>
-      </c>
-      <c r="D11" s="0" t="inlineStr">
-        <is>
-          <t>hillsdalecollegian.com</t>
-        </is>
-      </c>
-      <c r="E11" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F11" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G11" s="21" t="n">
-        <v>9793</v>
-      </c>
-      <c r="H11" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I11" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J11" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@hillsdale; 9793/15690 at 2026-09-28 15:48 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="0" t="inlineStr">
-        <is>
-          <t>Swarthmore College</t>
-        </is>
-      </c>
-      <c r="B12" s="0" t="inlineStr">
-        <is>
-          <t>The Phoenix</t>
-        </is>
-      </c>
-      <c r="C12" s="0" t="inlineStr">
-        <is>
-          <t>swarthmore</t>
-        </is>
-      </c>
-      <c r="D12" s="0" t="inlineStr">
-        <is>
-          <t>swarthmorephoenix.com</t>
-        </is>
-      </c>
-      <c r="E12" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F12" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G12" s="22" t="n">
-        <v>700</v>
-      </c>
-      <c r="H12" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I12" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J12" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@swarthmore; 700/13251 at 2026-09-28 15:48 UTC; pre_2000 skip working (578 skipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="0" t="inlineStr">
-        <is>
-          <t>Occidental College</t>
-        </is>
-      </c>
-      <c r="B13" s="0" t="inlineStr">
-        <is>
-          <t>The Occidental</t>
-        </is>
-      </c>
-      <c r="C13" s="0" t="inlineStr">
-        <is>
-          <t>occidental</t>
-        </is>
-      </c>
-      <c r="D13" s="0" t="inlineStr">
-        <is>
-          <t>theoccidentalnews.com</t>
-        </is>
-      </c>
-      <c r="E13" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F13" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G13" s="22" t="n">
-        <v>783</v>
-      </c>
-      <c r="H13" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I13" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J13" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@occidental; 783/10055 at 2026-09-28 15:48 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="0" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B14" s="0" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C14" s="0" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D14" s="0" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E14" s="0" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F14" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G14" s="22" t="n">
-        <v>682</v>
-      </c>
-      <c r="H14" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I14" s="0" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J14" s="0" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>University of Michigan</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>The Michigan Daily</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>michigan</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>michigandaily.com</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G15" s="21" t="n"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I15" s="23" t="n">
+      <c r="I24" s="35" t="n">
         <v>46293</v>
       </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Wave 4. Open WordPress. Probe + 200-test before full run. ~120k URLs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>University of California, Irvine</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>New University</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>uci</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>newuniversity.org</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G16" s="21" t="n"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I16" s="23" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Wave 4. Open WordPress. 200-test required: recon empty on 2003-04 URLs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>University of Miami</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>The Miami Hurricane</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>miami</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>themiamihurricane.com</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>National Universities</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="n"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I17" s="23" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Wave 4. Open WordPress behind Sucuri. Probe + 200-test before full run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Rochester Institute of Technology</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Reporter</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>rit</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>reporter.rit.edu</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>National Universities</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="n"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I18" s="23" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Wave 4. Open SNO, Crawl-delay 6. Probe + 200-test before full run.</t>
+      <c r="J24" s="34" t="inlineStr">
+        <is>
+          <t>Wave 5. Open WordPress. Probe + 200-test before full run. ~4k URLs.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add USF Oracle to refill the scraper slot Biola freed.
Open WordPress, no Cloudflare, about 32k URLs. Probe and a 200-test come before any full run.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -680,22 +680,22 @@
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
         <is>
-          <t>University of Miami</t>
+          <t>University of California, Santa Cruz</t>
         </is>
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>The Miami Hurricane</t>
+          <t>City on a Hill Press</t>
         </is>
       </c>
       <c r="C6" s="33" t="inlineStr">
         <is>
-          <t>miami</t>
+          <t>ucsc</t>
         </is>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
-          <t>themiamihurricane.com</t>
+          <t>cityonahillpress.com</t>
         </is>
       </c>
       <c r="E6" s="33" t="inlineStr">
@@ -719,29 +719,29 @@
       </c>
       <c r="J6" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@miami; full run started 2026-09-28</t>
+          <t>newspaper-scraper@ucsc; full run started 2026-09-28 after 200-row 200-test</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="33" t="inlineStr">
         <is>
-          <t>University of California, Santa Cruz</t>
+          <t>University of Miami</t>
         </is>
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>City on a Hill Press</t>
+          <t>The Miami Hurricane</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
         <is>
-          <t>ucsc</t>
+          <t>miami</t>
         </is>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>cityonahillpress.com</t>
+          <t>themiamihurricane.com</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="F7" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G7" s="33" t="n"/>
@@ -765,91 +765,91 @@
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
-          <t>Wave 5. Open WordPress. Probe + 200-test before full run. ~7k URLs.</t>
+          <t>newspaper-scraper@miami; full run started 2026-09-28</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>University of South Florida</t>
+        </is>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>The Oracle</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>usf</t>
+        </is>
+      </c>
+      <c r="D8" s="33" t="inlineStr">
+        <is>
+          <t>usforacle.com</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F8" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="n"/>
+      <c r="H8" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I8" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J8" s="34" t="inlineStr">
+        <is>
+          <t>Wave 5. Open WordPress. Probe + 200-test before full run. ~32k URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Public Universities</t>
         </is>
       </c>
-      <c r="B8" s="32" t="n"/>
-      <c r="C8" s="32" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="32" t="n"/>
-      <c r="F8" s="32" t="n"/>
-      <c r="G8" s="32" t="n"/>
-      <c r="H8" s="32" t="n"/>
-      <c r="I8" s="32" t="n"/>
-      <c r="J8" s="32" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>University of California, Irvine</t>
-        </is>
-      </c>
-      <c r="B9" s="33" t="inlineStr">
-        <is>
-          <t>New University</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="inlineStr">
-        <is>
-          <t>uci</t>
-        </is>
-      </c>
-      <c r="D9" s="33" t="inlineStr">
-        <is>
-          <t>newuniversity.org</t>
-        </is>
-      </c>
-      <c r="E9" s="33" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G9" s="33" t="n"/>
-      <c r="H9" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I9" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J9" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@uci; full run started 2026-09-28 after td-post-content fix</t>
-        </is>
-      </c>
+      <c r="B9" s="32" t="n"/>
+      <c r="C9" s="32" t="n"/>
+      <c r="D9" s="32" t="n"/>
+      <c r="E9" s="32" t="n"/>
+      <c r="F9" s="32" t="n"/>
+      <c r="G9" s="32" t="n"/>
+      <c r="H9" s="32" t="n"/>
+      <c r="I9" s="32" t="n"/>
+      <c r="J9" s="32" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="33" t="inlineStr">
         <is>
-          <t>University of Michigan</t>
+          <t>University of California, Irvine</t>
         </is>
       </c>
       <c r="B10" s="33" t="inlineStr">
         <is>
-          <t>The Michigan Daily</t>
+          <t>New University</t>
         </is>
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>michigan</t>
+          <t>uci</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
         <is>
-          <t>michigandaily.com</t>
+          <t>newuniversity.org</t>
         </is>
       </c>
       <c r="E10" s="33" t="inlineStr">
@@ -873,95 +873,91 @@
       </c>
       <c r="J10" s="34" t="inlineStr">
         <is>
+          <t>newspaper-scraper@uci; full run started 2026-09-28 after td-post-content fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>University of Michigan</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>The Michigan Daily</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>michigan</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>michigandaily.com</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="n"/>
+      <c r="H11" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I11" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J11" s="34" t="inlineStr">
+        <is>
           <t>newspaper-scraper@michigan; full run started 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B11" s="32" t="n"/>
-      <c r="C11" s="32" t="n"/>
-      <c r="D11" s="32" t="n"/>
-      <c r="E11" s="32" t="n"/>
-      <c r="F11" s="32" t="n"/>
-      <c r="G11" s="32" t="n"/>
-      <c r="H11" s="32" t="n"/>
-      <c r="I11" s="32" t="n"/>
-      <c r="J11" s="32" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E12" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F12" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G12" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H12" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I12" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J12" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
-        </is>
-      </c>
+      <c r="B12" s="32" t="n"/>
+      <c r="C12" s="32" t="n"/>
+      <c r="D12" s="32" t="n"/>
+      <c r="E12" s="32" t="n"/>
+      <c r="F12" s="32" t="n"/>
+      <c r="G12" s="32" t="n"/>
+      <c r="H12" s="32" t="n"/>
+      <c r="I12" s="32" t="n"/>
+      <c r="J12" s="32" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>Franklin &amp; Marshall College</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>The College Reporter</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>fandm</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D13" s="33" t="inlineStr">
         <is>
-          <t>the-college-reporter.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E13" s="33" t="inlineStr">
@@ -975,7 +971,7 @@
         </is>
       </c>
       <c r="G13" s="30" t="n">
-        <v>3449</v>
+        <v>4039</v>
       </c>
       <c r="H13" s="33" t="inlineStr">
         <is>
@@ -989,34 +985,34 @@
       </c>
       <c r="J13" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B14" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D14" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Liberal Arts</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
@@ -1025,7 +1021,7 @@
         </is>
       </c>
       <c r="G14" s="30" t="n">
-        <v>5048</v>
+        <v>3449</v>
       </c>
       <c r="H14" s="33" t="inlineStr">
         <is>
@@ -1039,127 +1035,129 @@
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G15" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H15" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I15" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J15" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
           <t>Union College (NY)</t>
         </is>
       </c>
-      <c r="B15" s="33" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>Concordiensis</t>
         </is>
       </c>
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>union</t>
         </is>
       </c>
-      <c r="D15" s="33" t="inlineStr">
+      <c r="D16" s="33" t="inlineStr">
         <is>
           <t>concordiensis.com</t>
         </is>
       </c>
-      <c r="E15" s="33" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F15" s="24" t="inlineStr">
+      <c r="F16" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G15" s="30" t="n">
+      <c r="G16" s="30" t="n">
         <v>1604</v>
       </c>
-      <c r="H15" s="33" t="inlineStr">
+      <c r="H16" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I15" s="33" t="inlineStr">
+      <c r="I16" s="33" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J15" s="34" t="inlineStr">
+      <c r="J16" s="34" t="inlineStr">
         <is>
           <t>Finished. 1604 articles of 1626 URLs; 44 empty_body skipped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>Hillsdale College</t>
-        </is>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>The Collegian</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>hillsdale</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>hillsdalecollegian.com</t>
-        </is>
-      </c>
-      <c r="E16" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F16" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G16" s="33" t="n"/>
-      <c r="H16" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I16" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J16" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@hillsdale</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="33" t="inlineStr">
         <is>
-          <t>Occidental College</t>
+          <t>Hillsdale College</t>
         </is>
       </c>
       <c r="B17" s="33" t="inlineStr">
         <is>
-          <t>The Occidental</t>
+          <t>The Collegian</t>
         </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>occidental</t>
+          <t>hillsdale</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>theoccidentalnews.com</t>
+          <t>hillsdalecollegian.com</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
@@ -1185,29 +1183,29 @@
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@occidental</t>
+          <t>newspaper-scraper@hillsdale</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="33" t="inlineStr">
         <is>
-          <t>Swarthmore College</t>
+          <t>Occidental College</t>
         </is>
       </c>
       <c r="B18" s="33" t="inlineStr">
         <is>
-          <t>The Phoenix</t>
+          <t>The Occidental</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>swarthmore</t>
+          <t>occidental</t>
         </is>
       </c>
       <c r="D18" s="33" t="inlineStr">
         <is>
-          <t>swarthmorephoenix.com</t>
+          <t>theoccidentalnews.com</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
@@ -1233,196 +1231,198 @@
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
+          <t>newspaper-scraper@occidental</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D19" s="33" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F19" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="n"/>
+      <c r="H19" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I19" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J19" s="34" t="inlineStr">
+        <is>
           <t>newspaper-scraper@swarthmore; pre-2000 permalinks skipped without fetch</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B19" s="32" t="n"/>
-      <c r="C19" s="32" t="n"/>
-      <c r="D19" s="32" t="n"/>
-      <c r="E19" s="32" t="n"/>
-      <c r="F19" s="32" t="n"/>
-      <c r="G19" s="32" t="n"/>
-      <c r="H19" s="32" t="n"/>
-      <c r="I19" s="32" t="n"/>
-      <c r="J19" s="32" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="32" t="n"/>
+      <c r="I20" s="32" t="n"/>
+      <c r="J20" s="32" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>Biola University</t>
+        </is>
+      </c>
+      <c r="B21" s="33" t="inlineStr">
+        <is>
+          <t>The Chimes</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>biola</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>chimesnewspaper.com</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F21" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G21" s="30" t="n">
+        <v>11331</v>
+      </c>
+      <c r="H21" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I21" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J21" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>Lipscomb University</t>
         </is>
       </c>
-      <c r="B20" s="33" t="inlineStr">
+      <c r="B22" s="33" t="inlineStr">
         <is>
           <t>Lipscomb Media</t>
         </is>
       </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="C22" s="33" t="inlineStr">
         <is>
           <t>lipscomb</t>
         </is>
       </c>
-      <c r="D20" s="33" t="inlineStr">
+      <c r="D22" s="33" t="inlineStr">
         <is>
           <t>lipscombmedia.com</t>
         </is>
       </c>
-      <c r="E20" s="33" t="inlineStr">
+      <c r="E22" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="F20" s="24" t="inlineStr">
+      <c r="F22" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G20" s="30" t="n">
+      <c r="G22" s="30" t="n">
         <v>682</v>
       </c>
-      <c r="H20" s="33" t="inlineStr">
+      <c r="H22" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I20" s="33" t="inlineStr">
+      <c r="I22" s="33" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J20" s="34" t="inlineStr">
+      <c r="J22" s="34" t="inlineStr">
         <is>
           <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D21" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E21" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F21" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G21" s="33" t="n"/>
-      <c r="H21" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I21" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J21" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@biola; recovered after href fix</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>Southern Methodist University</t>
-        </is>
-      </c>
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t>The Daily Campus</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>smu</t>
-        </is>
-      </c>
-      <c r="D22" s="33" t="inlineStr">
-        <is>
-          <t>smudailycampus.com</t>
-        </is>
-      </c>
-      <c r="E22" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges | National Universities</t>
-        </is>
-      </c>
-      <c r="F22" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G22" s="33" t="n"/>
-      <c r="H22" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I22" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J22" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@smu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="33" t="inlineStr">
         <is>
-          <t>Texas Christian University</t>
+          <t>Point Loma Nazarene University</t>
         </is>
       </c>
       <c r="B23" s="33" t="inlineStr">
         <is>
-          <t>TCU 360</t>
+          <t>Loma Beat</t>
         </is>
       </c>
       <c r="C23" s="33" t="inlineStr">
         <is>
-          <t>tcu</t>
+          <t>lomabeat</t>
         </is>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
-          <t>tcu360.com</t>
+          <t>lomabeat.com</t>
         </is>
       </c>
       <c r="E23" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | National Universities</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F23" s="33" t="inlineStr">
@@ -1436,46 +1436,44 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I23" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
+      <c r="I23" s="35" t="n">
+        <v>46293</v>
       </c>
       <c r="J23" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tcu</t>
+          <t>newspaper-scraper@lomabeat; full run started 2026-09-28 after 196-row 200-test</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="33" t="inlineStr">
         <is>
-          <t>Point Loma Nazarene University</t>
+          <t>Southern Methodist University</t>
         </is>
       </c>
       <c r="B24" s="33" t="inlineStr">
         <is>
-          <t>Loma Beat</t>
+          <t>The Daily Campus</t>
         </is>
       </c>
       <c r="C24" s="33" t="inlineStr">
         <is>
-          <t>lomabeat</t>
+          <t>smu</t>
         </is>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
-          <t>lomabeat.com</t>
+          <t>smudailycampus.com</t>
         </is>
       </c>
       <c r="E24" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges</t>
+          <t>Christian Colleges | National Universities</t>
         </is>
       </c>
       <c r="F24" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G24" s="33" t="n"/>
@@ -1484,12 +1482,62 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I24" s="35" t="n">
-        <v>46293</v>
+      <c r="I24" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
       </c>
       <c r="J24" s="34" t="inlineStr">
         <is>
-          <t>Wave 5. Open WordPress. Probe + 200-test before full run. ~4k URLs.</t>
+          <t>newspaper-scraper@smu</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>Texas Christian University</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>TCU 360</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>tcu</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>tcu360.com</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F25" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G25" s="33" t="n"/>
+      <c r="H25" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I25" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J25" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tcu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Denison, Wesleyan, and Yeshiva to refill three scraper slots.
Open WordPress only: two Liberal Arts papers and one National, with no extra Cloudflare load.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -797,7 +797,7 @@
       </c>
       <c r="F8" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G8" s="33" t="n"/>
@@ -811,91 +811,91 @@
       </c>
       <c r="J8" s="34" t="inlineStr">
         <is>
-          <t>Wave 5. Open WordPress. Probe + 200-test before full run. ~32k URLs.</t>
+          <t>newspaper-scraper@usf; full run started 2026-09-28 after 199-row 200-test</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Yeshiva University</t>
+        </is>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>The Commentator</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>yu</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>yucommentator.org</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F9" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="n"/>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="J9" s="34" t="inlineStr">
+        <is>
+          <t>Wave 6. Open WordPress. Probe + 200-test before full run. ~4.7k URLs; Crawl-delay 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Public Universities</t>
         </is>
       </c>
-      <c r="B9" s="32" t="n"/>
-      <c r="C9" s="32" t="n"/>
-      <c r="D9" s="32" t="n"/>
-      <c r="E9" s="32" t="n"/>
-      <c r="F9" s="32" t="n"/>
-      <c r="G9" s="32" t="n"/>
-      <c r="H9" s="32" t="n"/>
-      <c r="I9" s="32" t="n"/>
-      <c r="J9" s="32" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>University of California, Irvine</t>
-        </is>
-      </c>
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>New University</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>uci</t>
-        </is>
-      </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>newuniversity.org</t>
-        </is>
-      </c>
-      <c r="E10" s="33" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F10" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G10" s="33" t="n"/>
-      <c r="H10" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I10" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J10" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@uci; full run started 2026-09-28 after td-post-content fix</t>
-        </is>
-      </c>
+      <c r="B10" s="32" t="n"/>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="32" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="n"/>
+      <c r="H10" s="32" t="n"/>
+      <c r="I10" s="32" t="n"/>
+      <c r="J10" s="32" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="33" t="inlineStr">
         <is>
-          <t>University of Michigan</t>
+          <t>University of California, Irvine</t>
         </is>
       </c>
       <c r="B11" s="33" t="inlineStr">
         <is>
-          <t>The Michigan Daily</t>
+          <t>New University</t>
         </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
         <is>
-          <t>michigan</t>
+          <t>uci</t>
         </is>
       </c>
       <c r="D11" s="33" t="inlineStr">
         <is>
-          <t>michigandaily.com</t>
+          <t>newuniversity.org</t>
         </is>
       </c>
       <c r="E11" s="33" t="inlineStr">
@@ -919,95 +919,91 @@
       </c>
       <c r="J11" s="34" t="inlineStr">
         <is>
+          <t>newspaper-scraper@uci; full run started 2026-09-28 after td-post-content fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>University of Michigan</t>
+        </is>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>The Michigan Daily</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>michigan</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>michigandaily.com</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F12" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="n"/>
+      <c r="H12" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I12" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J12" s="34" t="inlineStr">
+        <is>
           <t>newspaper-scraper@michigan; full run started 2026-09-28</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B12" s="32" t="n"/>
-      <c r="C12" s="32" t="n"/>
-      <c r="D12" s="32" t="n"/>
-      <c r="E12" s="32" t="n"/>
-      <c r="F12" s="32" t="n"/>
-      <c r="G12" s="32" t="n"/>
-      <c r="H12" s="32" t="n"/>
-      <c r="I12" s="32" t="n"/>
-      <c r="J12" s="32" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C13" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D13" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E13" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F13" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G13" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H13" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I13" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J13" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
-        </is>
-      </c>
+      <c r="B13" s="32" t="n"/>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="32" t="n"/>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="32" t="n"/>
+      <c r="H13" s="32" t="n"/>
+      <c r="I13" s="32" t="n"/>
+      <c r="J13" s="32" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
-          <t>Franklin &amp; Marshall College</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B14" s="33" t="inlineStr">
         <is>
-          <t>The College Reporter</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>fandm</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D14" s="33" t="inlineStr">
         <is>
-          <t>the-college-reporter.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr">
@@ -1021,7 +1017,7 @@
         </is>
       </c>
       <c r="G14" s="30" t="n">
-        <v>3449</v>
+        <v>4039</v>
       </c>
       <c r="H14" s="33" t="inlineStr">
         <is>
@@ -1035,34 +1031,34 @@
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B15" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Liberal Arts</t>
         </is>
       </c>
       <c r="F15" s="24" t="inlineStr">
@@ -1071,7 +1067,7 @@
         </is>
       </c>
       <c r="G15" s="30" t="n">
-        <v>5048</v>
+        <v>3449</v>
       </c>
       <c r="H15" s="33" t="inlineStr">
         <is>
@@ -1085,457 +1081,605 @@
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
+          <t>Hillsdale College</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>The Collegian</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>hillsdale</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>hillsdalecollegian.com</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G16" s="30" t="n">
+        <v>15573</v>
+      </c>
+      <c r="H16" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I16" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J16" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Occidental College</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>The Occidental</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>occidental</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>theoccidentalnews.com</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G17" s="30" t="n">
+        <v>9892</v>
+      </c>
+      <c r="H17" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I17" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J17" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D18" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G18" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H18" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I18" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J18" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
           <t>Union College (NY)</t>
         </is>
       </c>
-      <c r="B16" s="33" t="inlineStr">
+      <c r="B19" s="33" t="inlineStr">
         <is>
           <t>Concordiensis</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C19" s="33" t="inlineStr">
         <is>
           <t>union</t>
         </is>
       </c>
-      <c r="D16" s="33" t="inlineStr">
+      <c r="D19" s="33" t="inlineStr">
         <is>
           <t>concordiensis.com</t>
         </is>
       </c>
-      <c r="E16" s="33" t="inlineStr">
+      <c r="E19" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F16" s="24" t="inlineStr">
+      <c r="F19" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G16" s="30" t="n">
+      <c r="G19" s="30" t="n">
         <v>1604</v>
       </c>
-      <c r="H16" s="33" t="inlineStr">
+      <c r="H19" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I16" s="33" t="inlineStr">
+      <c r="I19" s="33" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J16" s="34" t="inlineStr">
+      <c r="J19" s="34" t="inlineStr">
         <is>
           <t>Finished. 1604 articles of 1626 URLs; 44 empty_body skipped.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>Hillsdale College</t>
-        </is>
-      </c>
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>The Collegian</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>hillsdale</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
-        <is>
-          <t>hillsdalecollegian.com</t>
-        </is>
-      </c>
-      <c r="E17" s="33" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D20" s="33" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F17" s="33" t="inlineStr">
+      <c r="F20" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G17" s="33" t="n"/>
-      <c r="H17" s="33" t="inlineStr">
+      <c r="G20" s="33" t="n"/>
+      <c r="H20" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I17" s="33" t="inlineStr">
+      <c r="I20" s="33" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="J17" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@hillsdale</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="33" t="inlineStr">
-        <is>
-          <t>Occidental College</t>
-        </is>
-      </c>
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>The Occidental</t>
-        </is>
-      </c>
-      <c r="C18" s="33" t="inlineStr">
-        <is>
-          <t>occidental</t>
-        </is>
-      </c>
-      <c r="D18" s="33" t="inlineStr">
-        <is>
-          <t>theoccidentalnews.com</t>
-        </is>
-      </c>
-      <c r="E18" s="33" t="inlineStr">
+      <c r="J20" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@swarthmore; pre-2000 permalinks skipped without fetch</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Denison University</t>
+        </is>
+      </c>
+      <c r="B21" s="33" t="inlineStr">
+        <is>
+          <t>The Denisonian</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>denison</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>denisonian.com</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F18" s="33" t="inlineStr">
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="n"/>
+      <c r="H21" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I21" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="J21" s="34" t="inlineStr">
+        <is>
+          <t>Wave 6. Open WordPress. Probe + 200-test before full run. ~3.7k URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>Wesleyan University</t>
+        </is>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>The Wesleyan Argus</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>wesleyan</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="inlineStr">
+        <is>
+          <t>wesleyanargus.com</t>
+        </is>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F22" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G22" s="33" t="n"/>
+      <c r="H22" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I22" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="J22" s="34" t="inlineStr">
+        <is>
+          <t>Wave 6. Open WordPress. Probe + 200-test before full run. ~22k URLs; titles/authors may be thin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="n"/>
+      <c r="C23" s="32" t="n"/>
+      <c r="D23" s="32" t="n"/>
+      <c r="E23" s="32" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="32" t="n"/>
+      <c r="H23" s="32" t="n"/>
+      <c r="I23" s="32" t="n"/>
+      <c r="J23" s="32" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Biola University</t>
+        </is>
+      </c>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>The Chimes</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>biola</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="inlineStr">
+        <is>
+          <t>chimesnewspaper.com</t>
+        </is>
+      </c>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G24" s="30" t="n">
+        <v>11331</v>
+      </c>
+      <c r="H24" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I24" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J24" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Lipscomb University</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>Lipscomb Media</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>lipscomb</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>lipscombmedia.com</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G25" s="30" t="n">
+        <v>682</v>
+      </c>
+      <c r="H25" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I25" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="J25" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Point Loma Nazarene University</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>Loma Beat</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat.com</t>
+        </is>
+      </c>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F26" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G26" s="30" t="n">
+        <v>3950</v>
+      </c>
+      <c r="H26" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I26" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J26" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="inlineStr">
+        <is>
+          <t>Southern Methodist University</t>
+        </is>
+      </c>
+      <c r="B27" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Campus</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>smu</t>
+        </is>
+      </c>
+      <c r="D27" s="33" t="inlineStr">
+        <is>
+          <t>smudailycampus.com</t>
+        </is>
+      </c>
+      <c r="E27" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F27" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G18" s="33" t="n"/>
-      <c r="H18" s="33" t="inlineStr">
+      <c r="G27" s="33" t="n"/>
+      <c r="H27" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I18" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J18" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@occidental</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>Swarthmore College</t>
-        </is>
-      </c>
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>The Phoenix</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="inlineStr">
-        <is>
-          <t>swarthmore</t>
-        </is>
-      </c>
-      <c r="D19" s="33" t="inlineStr">
-        <is>
-          <t>swarthmorephoenix.com</t>
-        </is>
-      </c>
-      <c r="E19" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F19" s="33" t="inlineStr">
+      <c r="I27" s="33" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="J27" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@smu</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="33" t="inlineStr">
+        <is>
+          <t>Texas Christian University</t>
+        </is>
+      </c>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>TCU 360</t>
+        </is>
+      </c>
+      <c r="C28" s="33" t="inlineStr">
+        <is>
+          <t>tcu</t>
+        </is>
+      </c>
+      <c r="D28" s="33" t="inlineStr">
+        <is>
+          <t>tcu360.com</t>
+        </is>
+      </c>
+      <c r="E28" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F28" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G19" s="33" t="n"/>
-      <c r="H19" s="33" t="inlineStr">
+      <c r="G28" s="33" t="n"/>
+      <c r="H28" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I19" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J19" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@swarthmore; pre-2000 permalinks skipped without fetch</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="32" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="B20" s="32" t="n"/>
-      <c r="C20" s="32" t="n"/>
-      <c r="D20" s="32" t="n"/>
-      <c r="E20" s="32" t="n"/>
-      <c r="F20" s="32" t="n"/>
-      <c r="G20" s="32" t="n"/>
-      <c r="H20" s="32" t="n"/>
-      <c r="I20" s="32" t="n"/>
-      <c r="J20" s="32" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D21" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E21" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F21" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G21" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H21" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I21" s="33" t="inlineStr">
+      <c r="I28" s="33" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="J21" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D22" s="33" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E22" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F22" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G22" s="30" t="n">
-        <v>682</v>
-      </c>
-      <c r="H22" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I22" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J22" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>Point Loma Nazarene University</t>
-        </is>
-      </c>
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t>Loma Beat</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat</t>
-        </is>
-      </c>
-      <c r="D23" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat.com</t>
-        </is>
-      </c>
-      <c r="E23" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F23" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G23" s="33" t="n"/>
-      <c r="H23" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I23" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J23" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@lomabeat; full run started 2026-09-28 after 196-row 200-test</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="33" t="inlineStr">
-        <is>
-          <t>Southern Methodist University</t>
-        </is>
-      </c>
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t>The Daily Campus</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="inlineStr">
-        <is>
-          <t>smu</t>
-        </is>
-      </c>
-      <c r="D24" s="33" t="inlineStr">
-        <is>
-          <t>smudailycampus.com</t>
-        </is>
-      </c>
-      <c r="E24" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges | National Universities</t>
-        </is>
-      </c>
-      <c r="F24" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G24" s="33" t="n"/>
-      <c r="H24" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I24" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J24" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@smu</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="33" t="inlineStr">
-        <is>
-          <t>Texas Christian University</t>
-        </is>
-      </c>
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t>TCU 360</t>
-        </is>
-      </c>
-      <c r="C25" s="33" t="inlineStr">
-        <is>
-          <t>tcu</t>
-        </is>
-      </c>
-      <c r="D25" s="33" t="inlineStr">
-        <is>
-          <t>tcu360.com</t>
-        </is>
-      </c>
-      <c r="E25" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges | National Universities</t>
-        </is>
-      </c>
-      <c r="F25" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G25" s="33" t="n"/>
-      <c r="H25" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I25" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J25" s="34" t="inlineStr">
+      <c r="J28" s="34" t="inlineStr">
         <is>
           <t>newspaper-scraper@tcu</t>
         </is>

</xml_diff>

<commit_message>
Add The Student Life and The Hilltop; keep long articles in one CSV.
Two open Yoast WordPress papers refill empty slots without Cloudflare. St. Olaf now groups under Christian Colleges on the Status tab, and oversized bodies log a warning instead of splitting the file.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -460,7 +460,7 @@
     <col width="12" customWidth="1" style="19" min="7" max="7"/>
     <col width="12" customWidth="1" style="19" min="8" max="8"/>
     <col width="12" customWidth="1" style="19" min="9" max="9"/>
-    <col width="80" customWidth="1" style="19" min="10" max="10"/>
+    <col width="90" customWidth="1" style="19" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -575,173 +575,173 @@
       </c>
       <c r="J3" s="34" t="inlineStr">
         <is>
-          <t>Finished. 2137 articles of 2140 URLs (99.9%); 5 empty_body. systemd inactive. File: ~/Downloads/rit.csv</t>
+          <t>Finished. 2137 articles of 2140 URLs (99.9%); 5 empty_body. systemd inactive. File: repo output/rit.csv</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="24" t="inlineStr">
         <is>
+          <t>University of California, Santa Cruz</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>City on a Hill Press</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>ucsc</t>
+        </is>
+      </c>
+      <c r="D4" s="33" t="inlineStr">
+        <is>
+          <t>cityonahillpress.com</t>
+        </is>
+      </c>
+      <c r="E4" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="n">
+        <v>6899</v>
+      </c>
+      <c r="H4" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I4" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J4" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 6899 articles of 6992 URLs (98.7%); 67 empty_body, 26 pre_2000. systemd inactive. File: ~/Downloads/ucsc.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
           <t>University of Chicago</t>
         </is>
       </c>
-      <c r="B4" s="33" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>The Chicago Maroon</t>
         </is>
       </c>
-      <c r="C4" s="33" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>chicago</t>
         </is>
       </c>
-      <c r="D4" s="33" t="inlineStr">
+      <c r="D5" s="33" t="inlineStr">
         <is>
           <t>chicagomaroon.com</t>
         </is>
       </c>
-      <c r="E4" s="33" t="inlineStr">
+      <c r="E5" s="33" t="inlineStr">
         <is>
           <t>National Universities</t>
         </is>
       </c>
-      <c r="F4" s="24" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G4" s="30" t="n">
+      <c r="G5" s="30" t="n">
         <v>22117</v>
       </c>
-      <c r="H4" s="33" t="inlineStr">
+      <c r="H5" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I4" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J4" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 22117 articles of 22493 URLs (98.3%); 371 empty_body, 2 http_301, 3 http_404. systemd inactive. File: ~/Downloads/chicago.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="33" t="inlineStr">
-        <is>
-          <t>Northwestern University</t>
-        </is>
-      </c>
-      <c r="B5" s="33" t="inlineStr">
-        <is>
-          <t>The Daily Northwestern</t>
-        </is>
-      </c>
-      <c r="C5" s="33" t="inlineStr">
-        <is>
-          <t>northwestern</t>
-        </is>
-      </c>
-      <c r="D5" s="33" t="inlineStr">
-        <is>
-          <t>dailynorthwestern.com</t>
-        </is>
-      </c>
-      <c r="E5" s="33" t="inlineStr">
+      <c r="I5" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J5" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 22117 articles of 22493 URLs (98.3%); 371 empty_body, 2 http_301, 3 http_404. systemd inactive. File: repo output/chicago.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Yeshiva University</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>The Commentator</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>yu</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>yucommentator.org</t>
+        </is>
+      </c>
+      <c r="E6" s="33" t="inlineStr">
         <is>
           <t>National Universities</t>
         </is>
       </c>
-      <c r="F5" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G5" s="33" t="n"/>
-      <c r="H5" s="33" t="inlineStr">
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G6" s="30" t="n">
+        <v>4175</v>
+      </c>
+      <c r="H6" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I5" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="J5" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@northwestern; 403s still present at last check</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>University of California, Santa Cruz</t>
-        </is>
-      </c>
-      <c r="B6" s="33" t="inlineStr">
-        <is>
-          <t>City on a Hill Press</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>ucsc</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
-        <is>
-          <t>cityonahillpress.com</t>
-        </is>
-      </c>
-      <c r="E6" s="33" t="inlineStr">
-        <is>
-          <t>National Universities</t>
-        </is>
-      </c>
-      <c r="F6" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G6" s="33" t="n"/>
-      <c r="H6" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
       <c r="I6" s="35" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="J6" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@ucsc; full run started 2026-09-28 after 200-row 200-test</t>
+          <t>Finished. 4175 articles of 4678 URLs (89.2%); 41 empty_body, 464 pre_2000. systemd inactive. File: ~/Downloads/yu.csv</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="33" t="inlineStr">
         <is>
-          <t>University of Miami</t>
+          <t>Northwestern University</t>
         </is>
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>The Miami Hurricane</t>
+          <t>The Daily Northwestern</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
         <is>
-          <t>miami</t>
+          <t>northwestern</t>
         </is>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
-          <t>themiamihurricane.com</t>
+          <t>dailynorthwestern.com</t>
         </is>
       </c>
       <c r="E7" s="33" t="inlineStr">
@@ -761,33 +761,33 @@
         </is>
       </c>
       <c r="I7" s="35" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@miami; full run started 2026-09-28</t>
+          <t>newspaper-scraper@northwestern; 32750 of 70720 (46.3%). 403s still 32; network_error 1083.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
         <is>
-          <t>University of South Florida</t>
+          <t>University of Miami</t>
         </is>
       </c>
       <c r="B8" s="33" t="inlineStr">
         <is>
-          <t>The Oracle</t>
+          <t>The Miami Hurricane</t>
         </is>
       </c>
       <c r="C8" s="33" t="inlineStr">
         <is>
-          <t>usf</t>
+          <t>miami</t>
         </is>
       </c>
       <c r="D8" s="33" t="inlineStr">
         <is>
-          <t>usforacle.com</t>
+          <t>themiamihurricane.com</t>
         </is>
       </c>
       <c r="E8" s="33" t="inlineStr">
@@ -811,29 +811,29 @@
       </c>
       <c r="J8" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@usf; full run started 2026-09-28 after 199-row 200-test</t>
+          <t>newspaper-scraper@miami; 15050 of 25641 (58.7%). Watch http_403=2.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="33" t="inlineStr">
         <is>
-          <t>Yeshiva University</t>
+          <t>University of South Florida</t>
         </is>
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>The Commentator</t>
+          <t>The Oracle</t>
         </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
-          <t>yu</t>
+          <t>usf</t>
         </is>
       </c>
       <c r="D9" s="33" t="inlineStr">
         <is>
-          <t>yucommentator.org</t>
+          <t>usforacle.com</t>
         </is>
       </c>
       <c r="E9" s="33" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="F9" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G9" s="33" t="n"/>
@@ -853,108 +853,110 @@
         </is>
       </c>
       <c r="I9" s="35" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="J9" s="34" t="inlineStr">
         <is>
-          <t>Wave 6. Open WordPress. Probe + 200-test before full run. ~4.7k URLs; Crawl-delay 10.</t>
+          <t>newspaper-scraper@usf; 18099 of 32243 (56.1%).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Howard University</t>
+        </is>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>The Hilltop</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>hilltop</t>
+        </is>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>thehilltoponline.com</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="n"/>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I10" s="35" t="n">
+        <v>46295</v>
+      </c>
+      <c r="J10" s="34" t="inlineStr">
+        <is>
+          <t>Wave 7. Open WordPress Yoast. Probe + 200-test before full run. Crawl-delay 30; ~8.2k URLs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Public Universities</t>
         </is>
       </c>
-      <c r="B10" s="32" t="n"/>
-      <c r="C10" s="32" t="n"/>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="32" t="n"/>
-      <c r="F10" s="32" t="n"/>
-      <c r="G10" s="32" t="n"/>
-      <c r="H10" s="32" t="n"/>
-      <c r="I10" s="32" t="n"/>
-      <c r="J10" s="32" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="B11" s="32" t="n"/>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="32" t="n"/>
+      <c r="F11" s="32" t="n"/>
+      <c r="G11" s="32" t="n"/>
+      <c r="H11" s="32" t="n"/>
+      <c r="I11" s="32" t="n"/>
+      <c r="J11" s="32" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>University of California, Irvine</t>
         </is>
       </c>
-      <c r="B11" s="33" t="inlineStr">
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>New University</t>
         </is>
       </c>
-      <c r="C11" s="33" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>uci</t>
         </is>
       </c>
-      <c r="D11" s="33" t="inlineStr">
+      <c r="D12" s="33" t="inlineStr">
         <is>
           <t>newuniversity.org</t>
         </is>
       </c>
-      <c r="E11" s="33" t="inlineStr">
+      <c r="E12" s="33" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F11" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G11" s="33" t="n"/>
-      <c r="H11" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I11" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J11" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@uci; full run started 2026-09-28 after td-post-content fix</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>University of Michigan</t>
-        </is>
-      </c>
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>The Michigan Daily</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="inlineStr">
-        <is>
-          <t>michigan</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>michigandaily.com</t>
-        </is>
-      </c>
-      <c r="E12" s="33" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F12" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G12" s="33" t="n"/>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="n">
+        <v>17411</v>
+      </c>
       <c r="H12" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -965,95 +967,91 @@
       </c>
       <c r="J12" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan; full run started 2026-09-28</t>
+          <t>Finished. 17411 articles of 17447 URLs (99.8%); 165 empty_body. systemd inactive. File: ~/Downloads/uci.csv</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>University of Michigan</t>
+        </is>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>The Michigan Daily</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>michigan</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>michigandaily.com</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F13" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="n"/>
+      <c r="H13" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I13" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J13" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@michigan resumed after 168 KB field-limit crash. 16443 of 119764 (13.7%). http_301=440.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B13" s="32" t="n"/>
-      <c r="C13" s="32" t="n"/>
-      <c r="D13" s="32" t="n"/>
-      <c r="E13" s="32" t="n"/>
-      <c r="F13" s="32" t="n"/>
-      <c r="G13" s="32" t="n"/>
-      <c r="H13" s="32" t="n"/>
-      <c r="I13" s="32" t="n"/>
-      <c r="J13" s="32" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E14" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F14" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G14" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H14" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I14" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J14" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive.</t>
-        </is>
-      </c>
+      <c r="B14" s="32" t="n"/>
+      <c r="C14" s="32" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="32" t="n"/>
+      <c r="F14" s="32" t="n"/>
+      <c r="G14" s="32" t="n"/>
+      <c r="H14" s="32" t="n"/>
+      <c r="I14" s="32" t="n"/>
+      <c r="J14" s="32" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>Franklin &amp; Marshall College</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B15" s="33" t="inlineStr">
         <is>
-          <t>The College Reporter</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
-          <t>fandm</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>the-college-reporter.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr">
@@ -1067,43 +1065,41 @@
         </is>
       </c>
       <c r="G15" s="30" t="n">
-        <v>3449</v>
+        <v>4039</v>
       </c>
       <c r="H15" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I15" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
+      <c r="I15" s="35" t="n">
+        <v>46292</v>
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive.</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>Hillsdale College</t>
+          <t>Denison University</t>
         </is>
       </c>
       <c r="B16" s="33" t="inlineStr">
         <is>
-          <t>The Collegian</t>
+          <t>The Denisonian</t>
         </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
-          <t>hillsdale</t>
+          <t>denison</t>
         </is>
       </c>
       <c r="D16" s="33" t="inlineStr">
         <is>
-          <t>hillsdalecollegian.com</t>
+          <t>denisonian.com</t>
         </is>
       </c>
       <c r="E16" s="33" t="inlineStr">
@@ -1117,43 +1113,41 @@
         </is>
       </c>
       <c r="G16" s="30" t="n">
-        <v>15573</v>
+        <v>3671</v>
       </c>
       <c r="H16" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I16" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
+      <c r="I16" s="35" t="n">
+        <v>46294</v>
       </c>
       <c r="J16" s="34" t="inlineStr">
         <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive.</t>
+          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>Occidental College</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B17" s="33" t="inlineStr">
         <is>
-          <t>The Occidental</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>occidental</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>theoccidentalnews.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
@@ -1167,48 +1161,46 @@
         </is>
       </c>
       <c r="G17" s="30" t="n">
-        <v>9892</v>
+        <v>3449</v>
       </c>
       <c r="H17" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I17" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
+      <c r="I17" s="35" t="n">
+        <v>46292</v>
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive.</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Hillsdale College</t>
         </is>
       </c>
       <c r="B18" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>The Collegian</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>hillsdale</t>
         </is>
       </c>
       <c r="D18" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>hillsdalecollegian.com</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Liberal Arts</t>
         </is>
       </c>
       <c r="F18" s="24" t="inlineStr">
@@ -1217,165 +1209,163 @@
         </is>
       </c>
       <c r="G18" s="30" t="n">
-        <v>5048</v>
+        <v>15573</v>
       </c>
       <c r="H18" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I18" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
+      <c r="I18" s="35" t="n">
+        <v>46292</v>
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%). File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
+          <t>Occidental College</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>The Occidental</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>occidental</t>
+        </is>
+      </c>
+      <c r="D19" s="33" t="inlineStr">
+        <is>
+          <t>theoccidentalnews.com</t>
+        </is>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F19" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G19" s="30" t="n">
+        <v>9892</v>
+      </c>
+      <c r="H19" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I19" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J19" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D20" s="33" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G20" s="30" t="n">
+        <v>12798</v>
+      </c>
+      <c r="H20" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I20" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J20" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
           <t>Union College (NY)</t>
         </is>
       </c>
-      <c r="B19" s="33" t="inlineStr">
+      <c r="B21" s="33" t="inlineStr">
         <is>
           <t>Concordiensis</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C21" s="33" t="inlineStr">
         <is>
           <t>union</t>
         </is>
       </c>
-      <c r="D19" s="33" t="inlineStr">
+      <c r="D21" s="33" t="inlineStr">
         <is>
           <t>concordiensis.com</t>
         </is>
       </c>
-      <c r="E19" s="33" t="inlineStr">
+      <c r="E21" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F19" s="24" t="inlineStr">
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G19" s="30" t="n">
+      <c r="G21" s="30" t="n">
         <v>1604</v>
       </c>
-      <c r="H19" s="33" t="inlineStr">
+      <c r="H21" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I19" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J19" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 1604 articles of 1626 URLs; 44 empty_body skipped.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="33" t="inlineStr">
-        <is>
-          <t>Swarthmore College</t>
-        </is>
-      </c>
-      <c r="B20" s="33" t="inlineStr">
-        <is>
-          <t>The Phoenix</t>
-        </is>
-      </c>
-      <c r="C20" s="33" t="inlineStr">
-        <is>
-          <t>swarthmore</t>
-        </is>
-      </c>
-      <c r="D20" s="33" t="inlineStr">
-        <is>
-          <t>swarthmorephoenix.com</t>
-        </is>
-      </c>
-      <c r="E20" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F20" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G20" s="33" t="n"/>
-      <c r="H20" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I20" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
-      </c>
-      <c r="J20" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@swarthmore; pre-2000 permalinks skipped without fetch</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>Denison University</t>
-        </is>
-      </c>
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>The Denisonian</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="inlineStr">
-        <is>
-          <t>denison</t>
-        </is>
-      </c>
-      <c r="D21" s="33" t="inlineStr">
-        <is>
-          <t>denisonian.com</t>
-        </is>
-      </c>
-      <c r="E21" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F21" s="33" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G21" s="33" t="n"/>
-      <c r="H21" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
       <c r="I21" s="35" t="n">
-        <v>46294</v>
+        <v>46292</v>
       </c>
       <c r="J21" s="34" t="inlineStr">
         <is>
-          <t>Wave 6. Open WordPress. Probe + 200-test before full run. ~3.7k URLs.</t>
+          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1397,7 @@
       </c>
       <c r="F22" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G22" s="33" t="n"/>
@@ -1421,95 +1411,91 @@
       </c>
       <c r="J22" s="34" t="inlineStr">
         <is>
-          <t>Wave 6. Open WordPress. Probe + 200-test before full run. ~22k URLs; titles/authors may be thin.</t>
+          <t>newspaper-scraper@wesleyan; 13300 of 21917 (60.7%). Titles present, authors empty.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>Claremont Colleges</t>
+        </is>
+      </c>
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t>The Student Life</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>tsl</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="inlineStr">
+        <is>
+          <t>tsl.news</t>
+        </is>
+      </c>
+      <c r="E23" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F23" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="n"/>
+      <c r="H23" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I23" s="35" t="n">
+        <v>46295</v>
+      </c>
+      <c r="J23" s="34" t="inlineStr">
+        <is>
+          <t>Wave 7. Open WordPress Yoast. Probe + 200-test before full run. ~22.7k URLs; five Claremont colleges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n"/>
-      <c r="C23" s="32" t="n"/>
-      <c r="D23" s="32" t="n"/>
-      <c r="E23" s="32" t="n"/>
-      <c r="F23" s="32" t="n"/>
-      <c r="G23" s="32" t="n"/>
-      <c r="H23" s="32" t="n"/>
-      <c r="I23" s="32" t="n"/>
-      <c r="J23" s="32" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D24" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E24" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F24" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G24" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H24" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I24" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J24" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive.</t>
-        </is>
-      </c>
+      <c r="B24" s="32" t="n"/>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="32" t="n"/>
+      <c r="E24" s="32" t="n"/>
+      <c r="F24" s="32" t="n"/>
+      <c r="G24" s="32" t="n"/>
+      <c r="H24" s="32" t="n"/>
+      <c r="I24" s="32" t="n"/>
+      <c r="J24" s="32" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>Lipscomb University</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B25" s="33" t="inlineStr">
         <is>
-          <t>Lipscomb Media</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C25" s="33" t="inlineStr">
         <is>
-          <t>lipscomb</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
-          <t>lipscombmedia.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E25" s="33" t="inlineStr">
@@ -1523,165 +1509,259 @@
         </is>
       </c>
       <c r="G25" s="30" t="n">
-        <v>682</v>
+        <v>11331</v>
       </c>
       <c r="H25" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I25" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-27</t>
-        </is>
+      <c r="I25" s="35" t="n">
+        <v>46291</v>
       </c>
       <c r="J25" s="34" t="inlineStr">
         <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive.</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
+          <t>Lipscomb University</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>Lipscomb Media</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>lipscomb</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>lipscombmedia.com</t>
+        </is>
+      </c>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F26" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G26" s="30" t="n">
+        <v>682</v>
+      </c>
+      <c r="H26" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I26" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J26" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
           <t>Point Loma Nazarene University</t>
         </is>
       </c>
-      <c r="B26" s="33" t="inlineStr">
+      <c r="B27" s="33" t="inlineStr">
         <is>
           <t>Loma Beat</t>
         </is>
       </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C27" s="33" t="inlineStr">
         <is>
           <t>lomabeat</t>
         </is>
       </c>
-      <c r="D26" s="33" t="inlineStr">
+      <c r="D27" s="33" t="inlineStr">
         <is>
           <t>lomabeat.com</t>
         </is>
       </c>
-      <c r="E26" s="33" t="inlineStr">
+      <c r="E27" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="F26" s="24" t="inlineStr">
+      <c r="F27" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G26" s="30" t="n">
+      <c r="G27" s="30" t="n">
         <v>3950</v>
       </c>
-      <c r="H26" s="33" t="inlineStr">
+      <c r="H27" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I26" s="35" t="n">
+      <c r="I27" s="35" t="n">
         <v>46293</v>
       </c>
-      <c r="J26" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="33" t="inlineStr">
+      <c r="J27" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Southern Methodist University</t>
         </is>
       </c>
-      <c r="B27" s="33" t="inlineStr">
+      <c r="B28" s="33" t="inlineStr">
         <is>
           <t>The Daily Campus</t>
         </is>
       </c>
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C28" s="33" t="inlineStr">
         <is>
           <t>smu</t>
         </is>
       </c>
-      <c r="D27" s="33" t="inlineStr">
+      <c r="D28" s="33" t="inlineStr">
         <is>
           <t>smudailycampus.com</t>
         </is>
       </c>
-      <c r="E27" s="33" t="inlineStr">
+      <c r="E28" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F27" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G27" s="33" t="n"/>
-      <c r="H27" s="33" t="inlineStr">
+      <c r="F28" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G28" s="30" t="n">
+        <v>26208</v>
+      </c>
+      <c r="H28" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I27" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J27" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@smu</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="33" t="inlineStr">
+      <c r="I28" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J28" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B29" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D29" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E29" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G29" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H29" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I29" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J29" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="24" t="inlineStr">
         <is>
           <t>Texas Christian University</t>
         </is>
       </c>
-      <c r="B28" s="33" t="inlineStr">
+      <c r="B30" s="33" t="inlineStr">
         <is>
           <t>TCU 360</t>
         </is>
       </c>
-      <c r="C28" s="33" t="inlineStr">
+      <c r="C30" s="33" t="inlineStr">
         <is>
           <t>tcu</t>
         </is>
       </c>
-      <c r="D28" s="33" t="inlineStr">
+      <c r="D30" s="33" t="inlineStr">
         <is>
           <t>tcu360.com</t>
         </is>
       </c>
-      <c r="E28" s="33" t="inlineStr">
+      <c r="E30" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F28" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G28" s="33" t="n"/>
-      <c r="H28" s="33" t="inlineStr">
+      <c r="F30" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G30" s="30" t="n">
+        <v>25690</v>
+      </c>
+      <c r="H30" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I28" s="33" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="J28" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@tcu</t>
+      <c r="I30" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J30" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add UCSD Guardian as a Cloudflare canary and allow browser UA when a site refuses the honest bot.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -16,9 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -110,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -171,6 +172,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -448,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -765,7 +769,7 @@
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@northwestern; 32750 of 70720 (46.3%). 403s still 32; network_error 1083.</t>
+          <t>newspaper-scraper@northwestern; 38600 of 70720 (54.6%). 403s still 32; network_error 1083.</t>
         </is>
       </c>
     </row>
@@ -811,7 +815,7 @@
       </c>
       <c r="J8" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@miami; 15050 of 25641 (58.7%). Watch http_403=2.</t>
+          <t>newspaper-scraper@miami; 21700 of 25641 (84.6%). Watch http_403=2.</t>
         </is>
       </c>
     </row>
@@ -857,7 +861,7 @@
       </c>
       <c r="J9" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@usf; 18099 of 32243 (56.1%).</t>
+          <t>newspaper-scraper@usf; 28449 of 32243 (88.2%).</t>
         </is>
       </c>
     </row>
@@ -1013,93 +1017,91 @@
       </c>
       <c r="J13" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan resumed after 168 KB field-limit crash. 16443 of 119764 (13.7%). http_301=440.</t>
+          <t>newspaper-scraper@michigan resumed after 168 KB field-limit crash. 25693 of 119764 (21.4%). http_301=440.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>University of California San Diego</t>
+        </is>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>The UCSD Guardian</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>ucsd</t>
+        </is>
+      </c>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>ucsdguardian.org</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F14" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="n"/>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I14" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>Wave 8 Cloudflare canary. SNO. Probe + 200-test before full run. Pace 10-14 s (~22.6k URLs). Honest UA first; browser UA allowed if refused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B14" s="32" t="n"/>
-      <c r="C14" s="32" t="n"/>
-      <c r="D14" s="32" t="n"/>
-      <c r="E14" s="32" t="n"/>
-      <c r="F14" s="32" t="n"/>
-      <c r="G14" s="32" t="n"/>
-      <c r="H14" s="32" t="n"/>
-      <c r="I14" s="32" t="n"/>
-      <c r="J14" s="32" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B15" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E15" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F15" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G15" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H15" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I15" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J15" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
-        </is>
-      </c>
+      <c r="B15" s="32" t="n"/>
+      <c r="C15" s="32" t="n"/>
+      <c r="D15" s="32" t="n"/>
+      <c r="E15" s="32" t="n"/>
+      <c r="F15" s="32" t="n"/>
+      <c r="G15" s="32" t="n"/>
+      <c r="H15" s="32" t="n"/>
+      <c r="I15" s="32" t="n"/>
+      <c r="J15" s="32" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>Denison University</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B16" s="33" t="inlineStr">
         <is>
-          <t>The Denisonian</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C16" s="33" t="inlineStr">
         <is>
-          <t>denison</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D16" s="33" t="inlineStr">
         <is>
-          <t>denisonian.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E16" s="33" t="inlineStr">
@@ -1113,7 +1115,7 @@
         </is>
       </c>
       <c r="G16" s="30" t="n">
-        <v>3671</v>
+        <v>4039</v>
       </c>
       <c r="H16" s="33" t="inlineStr">
         <is>
@@ -1121,33 +1123,33 @@
         </is>
       </c>
       <c r="I16" s="35" t="n">
-        <v>46294</v>
+        <v>46292</v>
       </c>
       <c r="J16" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>Franklin &amp; Marshall College</t>
+          <t>Denison University</t>
         </is>
       </c>
       <c r="B17" s="33" t="inlineStr">
         <is>
-          <t>The College Reporter</t>
+          <t>The Denisonian</t>
         </is>
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>fandm</t>
+          <t>denison</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>the-college-reporter.com</t>
+          <t>denisonian.com</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
@@ -1161,7 +1163,7 @@
         </is>
       </c>
       <c r="G17" s="30" t="n">
-        <v>3449</v>
+        <v>3671</v>
       </c>
       <c r="H17" s="33" t="inlineStr">
         <is>
@@ -1169,33 +1171,33 @@
         </is>
       </c>
       <c r="I17" s="35" t="n">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
+          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>Hillsdale College</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B18" s="33" t="inlineStr">
         <is>
-          <t>The Collegian</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>hillsdale</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D18" s="33" t="inlineStr">
         <is>
-          <t>hillsdalecollegian.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
@@ -1209,7 +1211,7 @@
         </is>
       </c>
       <c r="G18" s="30" t="n">
-        <v>15573</v>
+        <v>3449</v>
       </c>
       <c r="H18" s="33" t="inlineStr">
         <is>
@@ -1221,29 +1223,29 @@
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>Occidental College</t>
+          <t>Hillsdale College</t>
         </is>
       </c>
       <c r="B19" s="33" t="inlineStr">
         <is>
-          <t>The Occidental</t>
+          <t>The Collegian</t>
         </is>
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>occidental</t>
+          <t>hillsdale</t>
         </is>
       </c>
       <c r="D19" s="33" t="inlineStr">
         <is>
-          <t>theoccidentalnews.com</t>
+          <t>hillsdalecollegian.com</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
@@ -1257,7 +1259,7 @@
         </is>
       </c>
       <c r="G19" s="30" t="n">
-        <v>9892</v>
+        <v>15573</v>
       </c>
       <c r="H19" s="33" t="inlineStr">
         <is>
@@ -1269,29 +1271,29 @@
       </c>
       <c r="J19" s="34" t="inlineStr">
         <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>Swarthmore College</t>
+          <t>Occidental College</t>
         </is>
       </c>
       <c r="B20" s="33" t="inlineStr">
         <is>
-          <t>The Phoenix</t>
+          <t>The Occidental</t>
         </is>
       </c>
       <c r="C20" s="33" t="inlineStr">
         <is>
-          <t>swarthmore</t>
+          <t>occidental</t>
         </is>
       </c>
       <c r="D20" s="33" t="inlineStr">
         <is>
-          <t>swarthmorephoenix.com</t>
+          <t>theoccidentalnews.com</t>
         </is>
       </c>
       <c r="E20" s="33" t="inlineStr">
@@ -1305,7 +1307,7 @@
         </is>
       </c>
       <c r="G20" s="30" t="n">
-        <v>12798</v>
+        <v>9892</v>
       </c>
       <c r="H20" s="33" t="inlineStr">
         <is>
@@ -1317,29 +1319,29 @@
       </c>
       <c r="J20" s="34" t="inlineStr">
         <is>
-          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="24" t="inlineStr">
         <is>
-          <t>Union College (NY)</t>
+          <t>Swarthmore College</t>
         </is>
       </c>
       <c r="B21" s="33" t="inlineStr">
         <is>
-          <t>Concordiensis</t>
+          <t>The Phoenix</t>
         </is>
       </c>
       <c r="C21" s="33" t="inlineStr">
         <is>
-          <t>union</t>
+          <t>swarthmore</t>
         </is>
       </c>
       <c r="D21" s="33" t="inlineStr">
         <is>
-          <t>concordiensis.com</t>
+          <t>swarthmorephoenix.com</t>
         </is>
       </c>
       <c r="E21" s="33" t="inlineStr">
@@ -1353,7 +1355,7 @@
         </is>
       </c>
       <c r="G21" s="30" t="n">
-        <v>1604</v>
+        <v>12798</v>
       </c>
       <c r="H21" s="33" t="inlineStr">
         <is>
@@ -1365,185 +1367,187 @@
       </c>
       <c r="J21" s="34" t="inlineStr">
         <is>
+          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>Union College (NY)</t>
+        </is>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>Concordiensis</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>union</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="inlineStr">
+        <is>
+          <t>concordiensis.com</t>
+        </is>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F22" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G22" s="30" t="n">
+        <v>1604</v>
+      </c>
+      <c r="H22" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I22" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J22" s="34" t="inlineStr">
+        <is>
           <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="33" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>Wesleyan University</t>
         </is>
       </c>
-      <c r="B22" s="33" t="inlineStr">
+      <c r="B23" s="33" t="inlineStr">
         <is>
           <t>The Wesleyan Argus</t>
         </is>
       </c>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C23" s="33" t="inlineStr">
         <is>
           <t>wesleyan</t>
         </is>
       </c>
-      <c r="D22" s="33" t="inlineStr">
+      <c r="D23" s="33" t="inlineStr">
         <is>
           <t>wesleyanargus.com</t>
         </is>
       </c>
-      <c r="E22" s="33" t="inlineStr">
+      <c r="E23" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F22" s="33" t="inlineStr">
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G23" s="24" t="n">
+        <v>21881</v>
+      </c>
+      <c r="H23" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I23" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="J23" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>Claremont Colleges</t>
+        </is>
+      </c>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>The Student Life</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>tsl</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="inlineStr">
+        <is>
+          <t>tsl.news</t>
+        </is>
+      </c>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F24" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G22" s="33" t="n"/>
-      <c r="H22" s="33" t="inlineStr">
+      <c r="G24" s="33" t="n"/>
+      <c r="H24" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I22" s="35" t="n">
-        <v>46294</v>
-      </c>
-      <c r="J22" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@wesleyan; 13300 of 21917 (60.7%). Titles present, authors empty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>Claremont Colleges</t>
-        </is>
-      </c>
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t>The Student Life</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="inlineStr">
-        <is>
-          <t>tsl</t>
-        </is>
-      </c>
-      <c r="D23" s="33" t="inlineStr">
-        <is>
-          <t>tsl.news</t>
-        </is>
-      </c>
-      <c r="E23" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F23" s="33" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G23" s="33" t="n"/>
-      <c r="H23" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I23" s="35" t="n">
+      <c r="I24" s="35" t="n">
         <v>46295</v>
       </c>
-      <c r="J23" s="34" t="inlineStr">
-        <is>
-          <t>Wave 7. Open WordPress Yoast. Probe + 200-test before full run. ~22.7k URLs; five Claremont colleges.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="J24" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tsl full run after 200-test OK. Resuming 200 of 11437 (1.7%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n"/>
-      <c r="C24" s="32" t="n"/>
-      <c r="D24" s="32" t="n"/>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="32" t="n"/>
-      <c r="G24" s="32" t="n"/>
-      <c r="H24" s="32" t="n"/>
-      <c r="I24" s="32" t="n"/>
-      <c r="J24" s="32" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C25" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D25" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E25" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F25" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G25" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H25" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I25" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J25" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
-        </is>
-      </c>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="32" t="n"/>
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="32" t="n"/>
+      <c r="I25" s="32" t="n"/>
+      <c r="J25" s="32" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>Lipscomb University</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B26" s="33" t="inlineStr">
         <is>
-          <t>Lipscomb Media</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C26" s="33" t="inlineStr">
         <is>
-          <t>lipscomb</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D26" s="33" t="inlineStr">
         <is>
-          <t>lipscombmedia.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E26" s="33" t="inlineStr">
@@ -1557,7 +1561,7 @@
         </is>
       </c>
       <c r="G26" s="30" t="n">
-        <v>682</v>
+        <v>11331</v>
       </c>
       <c r="H26" s="33" t="inlineStr">
         <is>
@@ -1565,33 +1569,33 @@
         </is>
       </c>
       <c r="I26" s="35" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="J26" s="34" t="inlineStr">
         <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>Point Loma Nazarene University</t>
+          <t>Lipscomb University</t>
         </is>
       </c>
       <c r="B27" s="33" t="inlineStr">
         <is>
-          <t>Loma Beat</t>
+          <t>Lipscomb Media</t>
         </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
-          <t>lomabeat</t>
+          <t>lipscomb</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>lomabeat.com</t>
+          <t>lipscombmedia.com</t>
         </is>
       </c>
       <c r="E27" s="33" t="inlineStr">
@@ -1605,7 +1609,7 @@
         </is>
       </c>
       <c r="G27" s="30" t="n">
-        <v>3950</v>
+        <v>682</v>
       </c>
       <c r="H27" s="33" t="inlineStr">
         <is>
@@ -1613,38 +1617,38 @@
         </is>
       </c>
       <c r="I27" s="35" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="J27" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>Southern Methodist University</t>
+          <t>Point Loma Nazarene University</t>
         </is>
       </c>
       <c r="B28" s="33" t="inlineStr">
         <is>
-          <t>The Daily Campus</t>
+          <t>Loma Beat</t>
         </is>
       </c>
       <c r="C28" s="33" t="inlineStr">
         <is>
-          <t>smu</t>
+          <t>lomabeat</t>
         </is>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
-          <t>smudailycampus.com</t>
+          <t>lomabeat.com</t>
         </is>
       </c>
       <c r="E28" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | National Universities</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F28" s="24" t="inlineStr">
@@ -1653,7 +1657,7 @@
         </is>
       </c>
       <c r="G28" s="30" t="n">
-        <v>26208</v>
+        <v>3950</v>
       </c>
       <c r="H28" s="33" t="inlineStr">
         <is>
@@ -1661,38 +1665,38 @@
         </is>
       </c>
       <c r="I28" s="35" t="n">
-        <v>46291</v>
+        <v>46293</v>
       </c>
       <c r="J28" s="34" t="inlineStr">
         <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Southern Methodist University</t>
         </is>
       </c>
       <c r="B29" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>The Daily Campus</t>
         </is>
       </c>
       <c r="C29" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>smu</t>
         </is>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>smudailycampus.com</t>
         </is>
       </c>
       <c r="E29" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Christian Colleges | National Universities</t>
         </is>
       </c>
       <c r="F29" s="24" t="inlineStr">
@@ -1701,7 +1705,7 @@
         </is>
       </c>
       <c r="G29" s="30" t="n">
-        <v>5048</v>
+        <v>26208</v>
       </c>
       <c r="H29" s="33" t="inlineStr">
         <is>
@@ -1709,57 +1713,105 @@
         </is>
       </c>
       <c r="I29" s="35" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="J29" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F30" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G30" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H30" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I30" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J30" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
           <t>Texas Christian University</t>
         </is>
       </c>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B31" s="33" t="inlineStr">
         <is>
           <t>TCU 360</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C31" s="33" t="inlineStr">
         <is>
           <t>tcu</t>
         </is>
       </c>
-      <c r="D30" s="33" t="inlineStr">
+      <c r="D31" s="33" t="inlineStr">
         <is>
           <t>tcu360.com</t>
         </is>
       </c>
-      <c r="E30" s="33" t="inlineStr">
+      <c r="E31" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F30" s="24" t="inlineStr">
+      <c r="F31" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G30" s="30" t="n">
+      <c r="G31" s="30" t="n">
         <v>25690</v>
       </c>
-      <c r="H30" s="33" t="inlineStr">
+      <c r="H31" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I30" s="35" t="n">
+      <c r="I31" s="35" t="n">
         <v>46291</v>
       </c>
-      <c r="J30" s="34" t="inlineStr">
+      <c r="J31" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>

</xml_diff>

<commit_message>
Enable Duke full mode on the VM and add five Public Cloudflare papers to fill the 12-scraper cap.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -912,101 +912,101 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>Duke University</t>
+        </is>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>The Chronicle</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>duke</t>
+        </is>
+      </c>
+      <c r="D11" s="33" t="inlineStr">
+        <is>
+          <t>dukechronicle.com</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F11" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="n"/>
+      <c r="H11" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I11" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J11" s="34" t="inlineStr">
+        <is>
+          <t>VM probe OK with browser UA. Full mode is News-section listings only. 200-test before systemd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>Public Universities</t>
         </is>
       </c>
-      <c r="B11" s="32" t="n"/>
-      <c r="C11" s="32" t="n"/>
-      <c r="D11" s="32" t="n"/>
-      <c r="E11" s="32" t="n"/>
-      <c r="F11" s="32" t="n"/>
-      <c r="G11" s="32" t="n"/>
-      <c r="H11" s="32" t="n"/>
-      <c r="I11" s="32" t="n"/>
-      <c r="J11" s="32" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+      <c r="B12" s="32" t="n"/>
+      <c r="C12" s="32" t="n"/>
+      <c r="D12" s="32" t="n"/>
+      <c r="E12" s="32" t="n"/>
+      <c r="F12" s="32" t="n"/>
+      <c r="G12" s="32" t="n"/>
+      <c r="H12" s="32" t="n"/>
+      <c r="I12" s="32" t="n"/>
+      <c r="J12" s="32" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>University of California, Irvine</t>
         </is>
       </c>
-      <c r="B12" s="33" t="inlineStr">
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>New University</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>uci</t>
         </is>
       </c>
-      <c r="D12" s="33" t="inlineStr">
+      <c r="D13" s="33" t="inlineStr">
         <is>
           <t>newuniversity.org</t>
         </is>
       </c>
-      <c r="E12" s="33" t="inlineStr">
+      <c r="E13" s="33" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F12" s="24" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G12" s="30" t="n">
+      <c r="G13" s="30" t="n">
         <v>17411</v>
       </c>
-      <c r="H12" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I12" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J12" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 17411 articles of 17447 URLs (99.8%); 165 empty_body. systemd inactive. File: ~/Downloads/uci.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>University of Michigan</t>
-        </is>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>The Michigan Daily</t>
-        </is>
-      </c>
-      <c r="C13" s="33" t="inlineStr">
-        <is>
-          <t>michigan</t>
-        </is>
-      </c>
-      <c r="D13" s="33" t="inlineStr">
-        <is>
-          <t>michigandaily.com</t>
-        </is>
-      </c>
-      <c r="E13" s="33" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F13" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G13" s="33" t="n"/>
       <c r="H13" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1017,29 +1017,29 @@
       </c>
       <c r="J13" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan resumed after 168 KB field-limit crash. 25693 of 119764 (21.4%). http_301=440.</t>
+          <t>Finished. 17411 articles of 17447 URLs (99.8%); 165 empty_body. systemd inactive. File: ~/Downloads/uci.csv</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="33" t="inlineStr">
         <is>
-          <t>University of California San Diego</t>
+          <t>University of Michigan</t>
         </is>
       </c>
       <c r="B14" s="33" t="inlineStr">
         <is>
-          <t>The UCSD Guardian</t>
+          <t>The Michigan Daily</t>
         </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>ucsd</t>
+          <t>michigan</t>
         </is>
       </c>
       <c r="D14" s="33" t="inlineStr">
         <is>
-          <t>ucsdguardian.org</t>
+          <t>michigandaily.com</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F14" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G14" s="33" t="n"/>
@@ -1058,338 +1058,326 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I14" s="36" t="n">
+      <c r="I14" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@michigan resumed after 168 KB field-limit crash. 25693 of 119764 (21.4%). http_301=440.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>University of California San Diego</t>
+        </is>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>The UCSD Guardian</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>ucsd</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>ucsdguardian.org</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="n"/>
+      <c r="H15" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I15" s="36" t="n">
         <v>46296</v>
       </c>
-      <c r="J14" s="34" t="inlineStr">
-        <is>
-          <t>Wave 8 Cloudflare canary. SNO. Probe + 200-test before full run. Pace 10-14 s (~22.6k URLs). Honest UA first; browser UA allowed if refused.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="J15" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@ucsd full run after 200-test 200/200 OK on honest UA. Resuming 200 of 22,605.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>University of Texas at Austin</t>
+        </is>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Texan</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>texan</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>thedailytexan.com</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G16" s="33" t="n"/>
+      <c r="H16" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I16" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J16" s="34" t="inlineStr">
+        <is>
+          <t>Wave 9 Cloudflare SNO. Probe + 200-test. Pace 10-14 s (~51.6k URLs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>University of California, Santa Barbara</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>Daily Nexus</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>nexus</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>dailynexus.com</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="n"/>
+      <c r="H17" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I17" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J17" s="34" t="inlineStr">
+        <is>
+          <t>Wave 9 Cloudflare WordPress Yoast. Probe + 200-test. Pace 10-14 s (~40.5k URLs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>University of Illinois Urbana-Champaign</t>
+        </is>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Illini</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>illini</t>
+        </is>
+      </c>
+      <c r="D18" s="33" t="inlineStr">
+        <is>
+          <t>dailyillini.com</t>
+        </is>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F18" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G18" s="33" t="n"/>
+      <c r="H18" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I18" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J18" s="34" t="inlineStr">
+        <is>
+          <t>Wave 9 Cloudflare SNO Yoast. Probe + 200-test. Pace 10-14 s (~100k URLs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>North Carolina State University</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>Technician</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+      <c r="D19" s="33" t="inlineStr">
+        <is>
+          <t>technicianonline.com</t>
+        </is>
+      </c>
+      <c r="E19" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F19" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="n"/>
+      <c r="H19" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I19" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J19" s="34" t="inlineStr">
+        <is>
+          <t>Wave 9 Cloudflare SNO. Public flagship. Probe + 200-test. Pace 10-14 s (~41k URLs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>Stony Brook University</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>The Statesman</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>statesman</t>
+        </is>
+      </c>
+      <c r="D20" s="33" t="inlineStr">
+        <is>
+          <t>sbstatesman.com</t>
+        </is>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F20" s="33" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G20" s="33" t="n"/>
+      <c r="H20" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I20" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J20" s="34" t="inlineStr">
+        <is>
+          <t>Wave 9 Cloudflare SNO. Public flagship. Probe + 200-test. Pace 10-14 s (~13.6k URLs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B15" s="32" t="n"/>
-      <c r="C15" s="32" t="n"/>
-      <c r="D15" s="32" t="n"/>
-      <c r="E15" s="32" t="n"/>
-      <c r="F15" s="32" t="n"/>
-      <c r="G15" s="32" t="n"/>
-      <c r="H15" s="32" t="n"/>
-      <c r="I15" s="32" t="n"/>
-      <c r="J15" s="32" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E16" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F16" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G16" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H16" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I16" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J16" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="24" t="inlineStr">
-        <is>
-          <t>Denison University</t>
-        </is>
-      </c>
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>The Denisonian</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>denison</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
-        <is>
-          <t>denisonian.com</t>
-        </is>
-      </c>
-      <c r="E17" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F17" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G17" s="30" t="n">
-        <v>3671</v>
-      </c>
-      <c r="H17" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I17" s="35" t="n">
-        <v>46294</v>
-      </c>
-      <c r="J17" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="inlineStr">
-        <is>
-          <t>Franklin &amp; Marshall College</t>
-        </is>
-      </c>
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>The College Reporter</t>
-        </is>
-      </c>
-      <c r="C18" s="33" t="inlineStr">
-        <is>
-          <t>fandm</t>
-        </is>
-      </c>
-      <c r="D18" s="33" t="inlineStr">
-        <is>
-          <t>the-college-reporter.com</t>
-        </is>
-      </c>
-      <c r="E18" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F18" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G18" s="30" t="n">
-        <v>3449</v>
-      </c>
-      <c r="H18" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I18" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J18" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="24" t="inlineStr">
-        <is>
-          <t>Hillsdale College</t>
-        </is>
-      </c>
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>The Collegian</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="inlineStr">
-        <is>
-          <t>hillsdale</t>
-        </is>
-      </c>
-      <c r="D19" s="33" t="inlineStr">
-        <is>
-          <t>hillsdalecollegian.com</t>
-        </is>
-      </c>
-      <c r="E19" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F19" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G19" s="30" t="n">
-        <v>15573</v>
-      </c>
-      <c r="H19" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I19" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J19" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>Occidental College</t>
-        </is>
-      </c>
-      <c r="B20" s="33" t="inlineStr">
-        <is>
-          <t>The Occidental</t>
-        </is>
-      </c>
-      <c r="C20" s="33" t="inlineStr">
-        <is>
-          <t>occidental</t>
-        </is>
-      </c>
-      <c r="D20" s="33" t="inlineStr">
-        <is>
-          <t>theoccidentalnews.com</t>
-        </is>
-      </c>
-      <c r="E20" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F20" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G20" s="30" t="n">
-        <v>9892</v>
-      </c>
-      <c r="H20" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I20" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J20" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="24" t="inlineStr">
-        <is>
-          <t>Swarthmore College</t>
-        </is>
-      </c>
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>The Phoenix</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="inlineStr">
-        <is>
-          <t>swarthmore</t>
-        </is>
-      </c>
-      <c r="D21" s="33" t="inlineStr">
-        <is>
-          <t>swarthmorephoenix.com</t>
-        </is>
-      </c>
-      <c r="E21" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F21" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G21" s="30" t="n">
-        <v>12798</v>
-      </c>
-      <c r="H21" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I21" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J21" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
-        </is>
-      </c>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="32" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="32" t="n"/>
+      <c r="H21" s="32" t="n"/>
+      <c r="I21" s="32" t="n"/>
+      <c r="J21" s="32" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="24" t="inlineStr">
         <is>
-          <t>Union College (NY)</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B22" s="33" t="inlineStr">
         <is>
-          <t>Concordiensis</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C22" s="33" t="inlineStr">
         <is>
-          <t>union</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D22" s="33" t="inlineStr">
         <is>
-          <t>concordiensis.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E22" s="33" t="inlineStr">
@@ -1403,7 +1391,7 @@
         </is>
       </c>
       <c r="G22" s="30" t="n">
-        <v>1604</v>
+        <v>4039</v>
       </c>
       <c r="H22" s="33" t="inlineStr">
         <is>
@@ -1415,29 +1403,29 @@
       </c>
       <c r="J22" s="34" t="inlineStr">
         <is>
-          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
-          <t>Wesleyan University</t>
+          <t>Denison University</t>
         </is>
       </c>
       <c r="B23" s="33" t="inlineStr">
         <is>
-          <t>The Wesleyan Argus</t>
+          <t>The Denisonian</t>
         </is>
       </c>
       <c r="C23" s="33" t="inlineStr">
         <is>
-          <t>wesleyan</t>
+          <t>denison</t>
         </is>
       </c>
       <c r="D23" s="33" t="inlineStr">
         <is>
-          <t>wesleyanargus.com</t>
+          <t>denisonian.com</t>
         </is>
       </c>
       <c r="E23" s="33" t="inlineStr">
@@ -1450,8 +1438,8 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G23" s="24" t="n">
-        <v>21881</v>
+      <c r="G23" s="30" t="n">
+        <v>3671</v>
       </c>
       <c r="H23" s="33" t="inlineStr">
         <is>
@@ -1463,29 +1451,29 @@
       </c>
       <c r="J23" s="34" t="inlineStr">
         <is>
-          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="33" t="inlineStr">
-        <is>
-          <t>Claremont Colleges</t>
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B24" s="33" t="inlineStr">
         <is>
-          <t>The Student Life</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C24" s="33" t="inlineStr">
         <is>
-          <t>tsl</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
-          <t>tsl.news</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E24" s="33" t="inlineStr">
@@ -1493,66 +1481,100 @@
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F24" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G24" s="33" t="n"/>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G24" s="30" t="n">
+        <v>3449</v>
+      </c>
       <c r="H24" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
       <c r="I24" s="35" t="n">
-        <v>46295</v>
+        <v>46292</v>
       </c>
       <c r="J24" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tsl full run after 200-test OK. Resuming 200 of 11437 (1.7%).</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="32" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="B25" s="32" t="n"/>
-      <c r="C25" s="32" t="n"/>
-      <c r="D25" s="32" t="n"/>
-      <c r="E25" s="32" t="n"/>
-      <c r="F25" s="32" t="n"/>
-      <c r="G25" s="32" t="n"/>
-      <c r="H25" s="32" t="n"/>
-      <c r="I25" s="32" t="n"/>
-      <c r="J25" s="32" t="n"/>
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>Hillsdale College</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>The Collegian</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>hillsdale</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>hillsdalecollegian.com</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G25" s="30" t="n">
+        <v>15573</v>
+      </c>
+      <c r="H25" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I25" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J25" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>Biola University</t>
+          <t>Occidental College</t>
         </is>
       </c>
       <c r="B26" s="33" t="inlineStr">
         <is>
-          <t>The Chimes</t>
+          <t>The Occidental</t>
         </is>
       </c>
       <c r="C26" s="33" t="inlineStr">
         <is>
-          <t>biola</t>
+          <t>occidental</t>
         </is>
       </c>
       <c r="D26" s="33" t="inlineStr">
         <is>
-          <t>chimesnewspaper.com</t>
+          <t>theoccidentalnews.com</t>
         </is>
       </c>
       <c r="E26" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges</t>
+          <t>Liberal Arts</t>
         </is>
       </c>
       <c r="F26" s="24" t="inlineStr">
@@ -1561,7 +1583,7 @@
         </is>
       </c>
       <c r="G26" s="30" t="n">
-        <v>11331</v>
+        <v>9892</v>
       </c>
       <c r="H26" s="33" t="inlineStr">
         <is>
@@ -1569,38 +1591,38 @@
         </is>
       </c>
       <c r="I26" s="35" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="J26" s="34" t="inlineStr">
         <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>Lipscomb University</t>
+          <t>Swarthmore College</t>
         </is>
       </c>
       <c r="B27" s="33" t="inlineStr">
         <is>
-          <t>Lipscomb Media</t>
+          <t>The Phoenix</t>
         </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
-          <t>lipscomb</t>
+          <t>swarthmore</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>lipscombmedia.com</t>
+          <t>swarthmorephoenix.com</t>
         </is>
       </c>
       <c r="E27" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges</t>
+          <t>Liberal Arts</t>
         </is>
       </c>
       <c r="F27" s="24" t="inlineStr">
@@ -1609,7 +1631,7 @@
         </is>
       </c>
       <c r="G27" s="30" t="n">
-        <v>682</v>
+        <v>12798</v>
       </c>
       <c r="H27" s="33" t="inlineStr">
         <is>
@@ -1621,34 +1643,34 @@
       </c>
       <c r="J27" s="34" t="inlineStr">
         <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
+          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>Point Loma Nazarene University</t>
+          <t>Union College (NY)</t>
         </is>
       </c>
       <c r="B28" s="33" t="inlineStr">
         <is>
-          <t>Loma Beat</t>
+          <t>Concordiensis</t>
         </is>
       </c>
       <c r="C28" s="33" t="inlineStr">
         <is>
-          <t>lomabeat</t>
+          <t>union</t>
         </is>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
-          <t>lomabeat.com</t>
+          <t>concordiensis.com</t>
         </is>
       </c>
       <c r="E28" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges</t>
+          <t>Liberal Arts</t>
         </is>
       </c>
       <c r="F28" s="24" t="inlineStr">
@@ -1657,7 +1679,7 @@
         </is>
       </c>
       <c r="G28" s="30" t="n">
-        <v>3950</v>
+        <v>1604</v>
       </c>
       <c r="H28" s="33" t="inlineStr">
         <is>
@@ -1665,153 +1687,407 @@
         </is>
       </c>
       <c r="I28" s="35" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="J28" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
+          <t>Wesleyan University</t>
+        </is>
+      </c>
+      <c r="B29" s="33" t="inlineStr">
+        <is>
+          <t>The Wesleyan Argus</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>wesleyan</t>
+        </is>
+      </c>
+      <c r="D29" s="33" t="inlineStr">
+        <is>
+          <t>wesleyanargus.com</t>
+        </is>
+      </c>
+      <c r="E29" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>21881</v>
+      </c>
+      <c r="H29" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I29" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="J29" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="33" t="inlineStr">
+        <is>
+          <t>Claremont Colleges</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>The Student Life</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>tsl</t>
+        </is>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
+        <is>
+          <t>tsl.news</t>
+        </is>
+      </c>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F30" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G30" s="33" t="n"/>
+      <c r="H30" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I30" s="35" t="n">
+        <v>46295</v>
+      </c>
+      <c r="J30" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tsl full run after 200-test OK. Resuming 200 of 11437 (1.7%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="B31" s="32" t="n"/>
+      <c r="C31" s="32" t="n"/>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="32" t="n"/>
+      <c r="F31" s="32" t="n"/>
+      <c r="G31" s="32" t="n"/>
+      <c r="H31" s="32" t="n"/>
+      <c r="I31" s="32" t="n"/>
+      <c r="J31" s="32" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>Biola University</t>
+        </is>
+      </c>
+      <c r="B32" s="33" t="inlineStr">
+        <is>
+          <t>The Chimes</t>
+        </is>
+      </c>
+      <c r="C32" s="33" t="inlineStr">
+        <is>
+          <t>biola</t>
+        </is>
+      </c>
+      <c r="D32" s="33" t="inlineStr">
+        <is>
+          <t>chimesnewspaper.com</t>
+        </is>
+      </c>
+      <c r="E32" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F32" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G32" s="30" t="n">
+        <v>11331</v>
+      </c>
+      <c r="H32" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I32" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J32" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="24" t="inlineStr">
+        <is>
+          <t>Lipscomb University</t>
+        </is>
+      </c>
+      <c r="B33" s="33" t="inlineStr">
+        <is>
+          <t>Lipscomb Media</t>
+        </is>
+      </c>
+      <c r="C33" s="33" t="inlineStr">
+        <is>
+          <t>lipscomb</t>
+        </is>
+      </c>
+      <c r="D33" s="33" t="inlineStr">
+        <is>
+          <t>lipscombmedia.com</t>
+        </is>
+      </c>
+      <c r="E33" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G33" s="30" t="n">
+        <v>682</v>
+      </c>
+      <c r="H33" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I33" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J33" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>Point Loma Nazarene University</t>
+        </is>
+      </c>
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>Loma Beat</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat</t>
+        </is>
+      </c>
+      <c r="D34" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat.com</t>
+        </is>
+      </c>
+      <c r="E34" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G34" s="30" t="n">
+        <v>3950</v>
+      </c>
+      <c r="H34" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I34" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J34" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
           <t>Southern Methodist University</t>
         </is>
       </c>
-      <c r="B29" s="33" t="inlineStr">
+      <c r="B35" s="33" t="inlineStr">
         <is>
           <t>The Daily Campus</t>
         </is>
       </c>
-      <c r="C29" s="33" t="inlineStr">
+      <c r="C35" s="33" t="inlineStr">
         <is>
           <t>smu</t>
         </is>
       </c>
-      <c r="D29" s="33" t="inlineStr">
+      <c r="D35" s="33" t="inlineStr">
         <is>
           <t>smudailycampus.com</t>
         </is>
       </c>
-      <c r="E29" s="33" t="inlineStr">
+      <c r="E35" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F29" s="24" t="inlineStr">
+      <c r="F35" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G29" s="30" t="n">
+      <c r="G35" s="30" t="n">
         <v>26208</v>
       </c>
-      <c r="H29" s="33" t="inlineStr">
+      <c r="H35" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I29" s="35" t="n">
+      <c r="I35" s="35" t="n">
         <v>46291</v>
       </c>
-      <c r="J29" s="34" t="inlineStr">
+      <c r="J35" s="34" t="inlineStr">
         <is>
           <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="24" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
         <is>
           <t>St. Olaf College</t>
         </is>
       </c>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B36" s="33" t="inlineStr">
         <is>
           <t>Manitou Messenger</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C36" s="33" t="inlineStr">
         <is>
           <t>stolaf</t>
         </is>
       </c>
-      <c r="D30" s="33" t="inlineStr">
+      <c r="D36" s="33" t="inlineStr">
         <is>
           <t>olafmessenger.com</t>
         </is>
       </c>
-      <c r="E30" s="33" t="inlineStr">
+      <c r="E36" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | Liberal Arts</t>
         </is>
       </c>
-      <c r="F30" s="24" t="inlineStr">
+      <c r="F36" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G30" s="30" t="n">
+      <c r="G36" s="30" t="n">
         <v>5048</v>
       </c>
-      <c r="H30" s="33" t="inlineStr">
+      <c r="H36" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I30" s="35" t="n">
+      <c r="I36" s="35" t="n">
         <v>46292</v>
       </c>
-      <c r="J30" s="34" t="inlineStr">
+      <c r="J36" s="34" t="inlineStr">
         <is>
           <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="24" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="24" t="inlineStr">
         <is>
           <t>Texas Christian University</t>
         </is>
       </c>
-      <c r="B31" s="33" t="inlineStr">
+      <c r="B37" s="33" t="inlineStr">
         <is>
           <t>TCU 360</t>
         </is>
       </c>
-      <c r="C31" s="33" t="inlineStr">
+      <c r="C37" s="33" t="inlineStr">
         <is>
           <t>tcu</t>
         </is>
       </c>
-      <c r="D31" s="33" t="inlineStr">
+      <c r="D37" s="33" t="inlineStr">
         <is>
           <t>tcu360.com</t>
         </is>
       </c>
-      <c r="E31" s="33" t="inlineStr">
+      <c r="E37" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F31" s="24" t="inlineStr">
+      <c r="F37" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G31" s="30" t="n">
+      <c r="G37" s="30" t="n">
         <v>25690</v>
       </c>
-      <c r="H31" s="33" t="inlineStr">
+      <c r="H37" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I31" s="35" t="n">
+      <c r="I37" s="35" t="n">
         <v>46291</v>
       </c>
-      <c r="J31" s="34" t="inlineStr">
+      <c r="J37" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>

</xml_diff>

<commit_message>
Add Daily Tar Heel and The Highlander to refill two Public scraper slots.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -177,6 +177,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -769,17 +770,17 @@
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@northwestern; 38600 of 70720 (54.6%). 403s still 32; network_error 1083.</t>
+          <t>newspaper-scraper@northwestern; 44850 of 70720 (63.4%) as of 2026-10-02 13:50 UTC. empty_body=1790, http_301=3, http_403=32 (stable), network_error=1083, pre_2000=37.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>University of Miami</t>
         </is>
       </c>
-      <c r="B8" s="33" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>The Miami Hurricane</t>
         </is>
@@ -799,12 +800,14 @@
           <t>National Universities</t>
         </is>
       </c>
-      <c r="F8" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G8" s="33" t="n"/>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="n">
+        <v>25622</v>
+      </c>
       <c r="H8" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -815,17 +818,17 @@
       </c>
       <c r="J8" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@miami; 21700 of 25641 (84.6%). Watch http_403=2.</t>
+          <t>Finished 2026-10-02. 25622 articles of 25641 URLs (99.9%); 8 empty_body, 2 http_403, 9 http_500, 5 network_error. systemd inactive. File: ~/Downloads/miami.csv</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>University of South Florida</t>
         </is>
       </c>
-      <c r="B9" s="33" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>The Oracle</t>
         </is>
@@ -845,12 +848,14 @@
           <t>National Universities</t>
         </is>
       </c>
-      <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G9" s="33" t="n"/>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="n">
+        <v>31894</v>
+      </c>
       <c r="H9" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -861,7 +866,7 @@
       </c>
       <c r="J9" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@usf; 28449 of 32243 (88.2%).</t>
+          <t>Finished 2026-10-01. 31894 articles of 32243 URLs (98.9%); 501 empty_body, 2 network_error, 9 pre_2000. systemd inactive. File: ~/Downloads/usf.csv</t>
         </is>
       </c>
     </row>
@@ -907,7 +912,7 @@
       </c>
       <c r="J10" s="34" t="inlineStr">
         <is>
-          <t>Wave 7. Open WordPress Yoast. Probe + 200-test before full run. Crawl-delay 30; ~8.2k URLs.</t>
+          <t>Not cleared on the VM: homepage timeout, article pages HTTP 508. Crawl-delay 30; ~8.2k URLs. Retry from Mac, wait, or skip.</t>
         </is>
       </c>
     </row>
@@ -939,7 +944,7 @@
       </c>
       <c r="F11" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G11" s="33" t="n"/>
@@ -953,7 +958,7 @@
       </c>
       <c r="J11" s="34" t="inlineStr">
         <is>
-          <t>VM probe OK with browser UA. Full mode is News-section listings only. 200-test before systemd.</t>
+          <t>newspaper-scraper@duke News-section listings only. 4600 rows as of 2026-10-02 13:50 UTC (no sitemap inventory). empty_body=17. Browser UA.</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1068,7 @@
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan resumed after 168 KB field-limit crash. 25693 of 119764 (21.4%). http_301=440.</t>
+          <t>newspaper-scraper@michigan; 35593 of 119764 (29.7%) as of 2026-10-02 13:50 UTC. empty_body=14, http_301=1130, http_429=3, network_error=2. Watch 429s.</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1114,7 @@
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@ucsd full run after 200-test 200/200 OK on honest UA. Resuming 200 of 22,605.</t>
+          <t>newspaper-scraper@ucsd Cloudflare canary 10-14s. 5450 of 22605 (24.1%) as of 2026-10-02 13:50 UTC. empty_body=3, http_500=2.</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1146,7 @@
       </c>
       <c r="F16" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G16" s="33" t="n"/>
@@ -1155,7 +1160,7 @@
       </c>
       <c r="J16" s="34" t="inlineStr">
         <is>
-          <t>Wave 9 Cloudflare SNO. Probe + 200-test. Pace 10-14 s (~51.6k URLs).</t>
+          <t>newspaper-scraper@texan Cloudflare SNO 10-14s. 4747 of 51636 (9.2%) as of 2026-10-02 13:50 UTC. empty_body=74, http_500=3.</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1192,7 @@
       </c>
       <c r="F17" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G17" s="33" t="n"/>
@@ -1201,7 +1206,7 @@
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>Wave 9 Cloudflare WordPress Yoast. Probe + 200-test. Pace 10-14 s (~40.5k URLs).</t>
+          <t>newspaper-scraper@nexus Cloudflare WP 10-14s. 4637 of 40465 (11.5%) as of 2026-10-02 13:50 UTC. empty_body=453 (high; photo features). Watch.</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1238,7 @@
       </c>
       <c r="F18" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G18" s="33" t="n"/>
@@ -1247,7 +1252,7 @@
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
-          <t>Wave 9 Cloudflare SNO Yoast. Probe + 200-test. Pace 10-14 s (~100k URLs).</t>
+          <t>newspaper-scraper@illini Cloudflare SNO 10-14s. 4900 of 100022 (4.9%) as of 2026-10-02 13:50 UTC. http_500=1, pre_2000=10.</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1284,7 @@
       </c>
       <c r="F19" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G19" s="33" t="n"/>
@@ -1293,7 +1298,7 @@
       </c>
       <c r="J19" s="34" t="inlineStr">
         <is>
-          <t>Wave 9 Cloudflare SNO. Public flagship. Probe + 200-test. Pace 10-14 s (~41k URLs).</t>
+          <t>newspaper-scraper@technician Cloudflare SNO 10-14s. 5083 of 41051 (12.4%) as of 2026-10-02 13:50 UTC. empty_body=82.</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1330,7 @@
       </c>
       <c r="F20" s="33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="G20" s="33" t="n"/>
@@ -1339,141 +1344,135 @@
       </c>
       <c r="J20" s="34" t="inlineStr">
         <is>
-          <t>Wave 9 Cloudflare SNO. Public flagship. Probe + 200-test. Pace 10-14 s (~13.6k URLs).</t>
+          <t>newspaper-scraper@statesman Cloudflare SNO 10-14s. 5047 of 13650 (37.0%) as of 2026-10-02 13:50 UTC. empty_body=106.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>University of North Carolina, Chapel Hill</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>The Daily Tar Heel</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>tarheel</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>dailytarheel.com</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I21" s="37" t="n">
+        <v>46297</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Wave 10. Cloudflare SNO. wp-sitemap.xml (~82k URLs). Pace 10-14 s. Probe + 200-test before systemd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>University of California, Riverside</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>The Highlander</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>highlander</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>highlandernews.org</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I22" s="37" t="n">
+        <v>46297</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Wave 10. Public campus listed only on the National tab. Cloudflare Yoast WP (~10k URLs). Pace 10-14 s. Probe + 200-test before systemd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B21" s="32" t="n"/>
-      <c r="C21" s="32" t="n"/>
-      <c r="D21" s="32" t="n"/>
-      <c r="E21" s="32" t="n"/>
-      <c r="F21" s="32" t="n"/>
-      <c r="G21" s="32" t="n"/>
-      <c r="H21" s="32" t="n"/>
-      <c r="I21" s="32" t="n"/>
-      <c r="J21" s="32" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B22" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D22" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E22" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F22" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G22" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H22" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I22" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J22" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="24" t="inlineStr">
-        <is>
-          <t>Denison University</t>
-        </is>
-      </c>
-      <c r="B23" s="33" t="inlineStr">
-        <is>
-          <t>The Denisonian</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="inlineStr">
-        <is>
-          <t>denison</t>
-        </is>
-      </c>
-      <c r="D23" s="33" t="inlineStr">
-        <is>
-          <t>denisonian.com</t>
-        </is>
-      </c>
-      <c r="E23" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F23" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G23" s="30" t="n">
-        <v>3671</v>
-      </c>
-      <c r="H23" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I23" s="35" t="n">
-        <v>46294</v>
-      </c>
-      <c r="J23" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
-        </is>
-      </c>
+      <c r="B23" s="32" t="n"/>
+      <c r="C23" s="32" t="n"/>
+      <c r="D23" s="32" t="n"/>
+      <c r="E23" s="32" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="32" t="n"/>
+      <c r="H23" s="32" t="n"/>
+      <c r="I23" s="32" t="n"/>
+      <c r="J23" s="32" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
         <is>
-          <t>Franklin &amp; Marshall College</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B24" s="33" t="inlineStr">
         <is>
-          <t>The College Reporter</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C24" s="33" t="inlineStr">
         <is>
-          <t>fandm</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D24" s="33" t="inlineStr">
         <is>
-          <t>the-college-reporter.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E24" s="33" t="inlineStr">
@@ -1487,7 +1486,7 @@
         </is>
       </c>
       <c r="G24" s="30" t="n">
-        <v>3449</v>
+        <v>4039</v>
       </c>
       <c r="H24" s="33" t="inlineStr">
         <is>
@@ -1499,29 +1498,29 @@
       </c>
       <c r="J24" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="24" t="inlineStr">
         <is>
-          <t>Hillsdale College</t>
+          <t>Denison University</t>
         </is>
       </c>
       <c r="B25" s="33" t="inlineStr">
         <is>
-          <t>The Collegian</t>
+          <t>The Denisonian</t>
         </is>
       </c>
       <c r="C25" s="33" t="inlineStr">
         <is>
-          <t>hillsdale</t>
+          <t>denison</t>
         </is>
       </c>
       <c r="D25" s="33" t="inlineStr">
         <is>
-          <t>hillsdalecollegian.com</t>
+          <t>denisonian.com</t>
         </is>
       </c>
       <c r="E25" s="33" t="inlineStr">
@@ -1535,7 +1534,7 @@
         </is>
       </c>
       <c r="G25" s="30" t="n">
-        <v>15573</v>
+        <v>3671</v>
       </c>
       <c r="H25" s="33" t="inlineStr">
         <is>
@@ -1543,33 +1542,33 @@
         </is>
       </c>
       <c r="I25" s="35" t="n">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="J25" s="34" t="inlineStr">
         <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
+          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="24" t="inlineStr">
         <is>
-          <t>Occidental College</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B26" s="33" t="inlineStr">
         <is>
-          <t>The Occidental</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C26" s="33" t="inlineStr">
         <is>
-          <t>occidental</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D26" s="33" t="inlineStr">
         <is>
-          <t>theoccidentalnews.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E26" s="33" t="inlineStr">
@@ -1583,7 +1582,7 @@
         </is>
       </c>
       <c r="G26" s="30" t="n">
-        <v>9892</v>
+        <v>3449</v>
       </c>
       <c r="H26" s="33" t="inlineStr">
         <is>
@@ -1595,29 +1594,29 @@
       </c>
       <c r="J26" s="34" t="inlineStr">
         <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>Swarthmore College</t>
+          <t>Hillsdale College</t>
         </is>
       </c>
       <c r="B27" s="33" t="inlineStr">
         <is>
-          <t>The Phoenix</t>
+          <t>The Collegian</t>
         </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
-          <t>swarthmore</t>
+          <t>hillsdale</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>swarthmorephoenix.com</t>
+          <t>hillsdalecollegian.com</t>
         </is>
       </c>
       <c r="E27" s="33" t="inlineStr">
@@ -1631,7 +1630,7 @@
         </is>
       </c>
       <c r="G27" s="30" t="n">
-        <v>12798</v>
+        <v>15573</v>
       </c>
       <c r="H27" s="33" t="inlineStr">
         <is>
@@ -1643,29 +1642,29 @@
       </c>
       <c r="J27" s="34" t="inlineStr">
         <is>
-          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>Union College (NY)</t>
+          <t>Occidental College</t>
         </is>
       </c>
       <c r="B28" s="33" t="inlineStr">
         <is>
-          <t>Concordiensis</t>
+          <t>The Occidental</t>
         </is>
       </c>
       <c r="C28" s="33" t="inlineStr">
         <is>
-          <t>union</t>
+          <t>occidental</t>
         </is>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
-          <t>concordiensis.com</t>
+          <t>theoccidentalnews.com</t>
         </is>
       </c>
       <c r="E28" s="33" t="inlineStr">
@@ -1679,7 +1678,7 @@
         </is>
       </c>
       <c r="G28" s="30" t="n">
-        <v>1604</v>
+        <v>9892</v>
       </c>
       <c r="H28" s="33" t="inlineStr">
         <is>
@@ -1691,235 +1690,235 @@
       </c>
       <c r="J28" s="34" t="inlineStr">
         <is>
-          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B29" s="33" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D29" s="33" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E29" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G29" s="30" t="n">
+        <v>12798</v>
+      </c>
+      <c r="H29" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I29" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J29" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="24" t="inlineStr">
+        <is>
+          <t>Union College (NY)</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>Concordiensis</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>union</t>
+        </is>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
+        <is>
+          <t>concordiensis.com</t>
+        </is>
+      </c>
+      <c r="E30" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F30" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G30" s="30" t="n">
+        <v>1604</v>
+      </c>
+      <c r="H30" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I30" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J30" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="24" t="inlineStr">
+        <is>
           <t>Wesleyan University</t>
         </is>
       </c>
-      <c r="B29" s="33" t="inlineStr">
+      <c r="B31" s="33" t="inlineStr">
         <is>
           <t>The Wesleyan Argus</t>
         </is>
       </c>
-      <c r="C29" s="33" t="inlineStr">
+      <c r="C31" s="33" t="inlineStr">
         <is>
           <t>wesleyan</t>
         </is>
       </c>
-      <c r="D29" s="33" t="inlineStr">
+      <c r="D31" s="33" t="inlineStr">
         <is>
           <t>wesleyanargus.com</t>
         </is>
       </c>
-      <c r="E29" s="33" t="inlineStr">
+      <c r="E31" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F29" s="24" t="inlineStr">
+      <c r="F31" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G29" s="24" t="n">
+      <c r="G31" s="24" t="n">
         <v>21881</v>
       </c>
-      <c r="H29" s="33" t="inlineStr">
+      <c r="H31" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I29" s="35" t="n">
+      <c r="I31" s="35" t="n">
         <v>46294</v>
       </c>
-      <c r="J29" s="34" t="inlineStr">
+      <c r="J31" s="34" t="inlineStr">
         <is>
           <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="33" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>Claremont Colleges</t>
         </is>
       </c>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B32" s="33" t="inlineStr">
         <is>
           <t>The Student Life</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C32" s="33" t="inlineStr">
         <is>
           <t>tsl</t>
         </is>
       </c>
-      <c r="D30" s="33" t="inlineStr">
+      <c r="D32" s="33" t="inlineStr">
         <is>
           <t>tsl.news</t>
         </is>
       </c>
-      <c r="E30" s="33" t="inlineStr">
+      <c r="E32" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F30" s="33" t="inlineStr">
+      <c r="F32" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G30" s="33" t="n"/>
-      <c r="H30" s="33" t="inlineStr">
+      <c r="G32" s="33" t="n"/>
+      <c r="H32" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I30" s="35" t="n">
+      <c r="I32" s="35" t="n">
         <v>46295</v>
       </c>
-      <c r="J30" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@tsl full run after 200-test OK. Resuming 200 of 11437 (1.7%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="32" t="inlineStr">
+      <c r="J32" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tsl; 9600 of 11437 (83.9%) as of 2026-10-02 13:50 UTC. empty_body=14, http_403=15. Closest to finishing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B31" s="32" t="n"/>
-      <c r="C31" s="32" t="n"/>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="32" t="n"/>
-      <c r="F31" s="32" t="n"/>
-      <c r="G31" s="32" t="n"/>
-      <c r="H31" s="32" t="n"/>
-      <c r="I31" s="32" t="n"/>
-      <c r="J31" s="32" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B32" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C32" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D32" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E32" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F32" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G32" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H32" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I32" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J32" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C33" s="33" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D33" s="33" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E33" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F33" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G33" s="30" t="n">
-        <v>682</v>
-      </c>
-      <c r="H33" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I33" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J33" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
-        </is>
-      </c>
+      <c r="B33" s="32" t="n"/>
+      <c r="C33" s="32" t="n"/>
+      <c r="D33" s="32" t="n"/>
+      <c r="E33" s="32" t="n"/>
+      <c r="F33" s="32" t="n"/>
+      <c r="G33" s="32" t="n"/>
+      <c r="H33" s="32" t="n"/>
+      <c r="I33" s="32" t="n"/>
+      <c r="J33" s="32" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>Point Loma Nazarene University</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B34" s="33" t="inlineStr">
         <is>
-          <t>Loma Beat</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
-          <t>lomabeat</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
-          <t>lomabeat.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E34" s="33" t="inlineStr">
@@ -1933,7 +1932,7 @@
         </is>
       </c>
       <c r="G34" s="30" t="n">
-        <v>3950</v>
+        <v>11331</v>
       </c>
       <c r="H34" s="33" t="inlineStr">
         <is>
@@ -1941,38 +1940,38 @@
         </is>
       </c>
       <c r="I34" s="35" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="J34" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>Southern Methodist University</t>
+          <t>Lipscomb University</t>
         </is>
       </c>
       <c r="B35" s="33" t="inlineStr">
         <is>
-          <t>The Daily Campus</t>
+          <t>Lipscomb Media</t>
         </is>
       </c>
       <c r="C35" s="33" t="inlineStr">
         <is>
-          <t>smu</t>
+          <t>lipscomb</t>
         </is>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
-          <t>smudailycampus.com</t>
+          <t>lipscombmedia.com</t>
         </is>
       </c>
       <c r="E35" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | National Universities</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F35" s="24" t="inlineStr">
@@ -1981,7 +1980,7 @@
         </is>
       </c>
       <c r="G35" s="30" t="n">
-        <v>26208</v>
+        <v>682</v>
       </c>
       <c r="H35" s="33" t="inlineStr">
         <is>
@@ -1989,38 +1988,38 @@
         </is>
       </c>
       <c r="I35" s="35" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="J35" s="34" t="inlineStr">
         <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Point Loma Nazarene University</t>
         </is>
       </c>
       <c r="B36" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>Loma Beat</t>
         </is>
       </c>
       <c r="C36" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>lomabeat</t>
         </is>
       </c>
       <c r="D36" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>lomabeat.com</t>
         </is>
       </c>
       <c r="E36" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F36" s="24" t="inlineStr">
@@ -2029,7 +2028,7 @@
         </is>
       </c>
       <c r="G36" s="30" t="n">
-        <v>5048</v>
+        <v>3950</v>
       </c>
       <c r="H36" s="33" t="inlineStr">
         <is>
@@ -2037,33 +2036,33 @@
         </is>
       </c>
       <c r="I36" s="35" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="J36" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>Texas Christian University</t>
+          <t>Southern Methodist University</t>
         </is>
       </c>
       <c r="B37" s="33" t="inlineStr">
         <is>
-          <t>TCU 360</t>
+          <t>The Daily Campus</t>
         </is>
       </c>
       <c r="C37" s="33" t="inlineStr">
         <is>
-          <t>tcu</t>
+          <t>smu</t>
         </is>
       </c>
       <c r="D37" s="33" t="inlineStr">
         <is>
-          <t>tcu360.com</t>
+          <t>smudailycampus.com</t>
         </is>
       </c>
       <c r="E37" s="33" t="inlineStr">
@@ -2077,7 +2076,7 @@
         </is>
       </c>
       <c r="G37" s="30" t="n">
-        <v>25690</v>
+        <v>26208</v>
       </c>
       <c r="H37" s="33" t="inlineStr">
         <is>
@@ -2088,6 +2087,102 @@
         <v>46291</v>
       </c>
       <c r="J37" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B38" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C38" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D38" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G38" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H38" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I38" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J38" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>Texas Christian University</t>
+        </is>
+      </c>
+      <c r="B39" s="33" t="inlineStr">
+        <is>
+          <t>TCU 360</t>
+        </is>
+      </c>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>tcu</t>
+        </is>
+      </c>
+      <c r="D39" s="33" t="inlineStr">
+        <is>
+          <t>tcu360.com</t>
+        </is>
+      </c>
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G39" s="30" t="n">
+        <v>25690</v>
+      </c>
+      <c r="H39" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I39" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J39" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>

</xml_diff>

<commit_message>
Skip Daily Tar Heel multimedia galleries and videos on the full run.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -1349,37 +1349,37 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>University of North Carolina, Chapel Hill</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>The Daily Tar Heel</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>tarheel</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>dailytarheel.com</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="F21" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H21" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -1387,44 +1387,44 @@
       <c r="I21" s="37" t="n">
         <v>46297</v>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Wave 10. Cloudflare SNO. wp-sitemap.xml (~82k URLs). Pace 10-14 s. Probe + 200-test before systemd.</t>
+      <c r="J21" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tarheel full run after 129/200 (71 empty_body, almost all /multimedia/ galleries and videos; those URLs now excluded). Resuming 129 of ~82k. Cloudflare SNO 10-14 s.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>University of California, Riverside</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>The Highlander</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>highlander</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>highlandernews.org</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
+      <c r="F22" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H22" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -1432,9 +1432,9 @@
       <c r="I22" s="37" t="n">
         <v>46297</v>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Wave 10. Public campus listed only on the National tab. Cloudflare Yoast WP (~10k URLs). Pace 10-14 s. Probe + 200-test before systemd.</t>
+      <c r="J22" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@highlander full run after 176/200 (24 empty_body). Resuming 176 of ~10144. Cloudflare Yoast WP 10-14 s. Public campus listed only on the National tab.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add UMass Collegian, Minnesota Daily, and Pitt News to refill three Public slots.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -178,6 +178,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -770,7 +773,7 @@
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@northwestern; 44850 of 70720 (63.4%) as of 2026-10-02 13:50 UTC. empty_body=1790, http_301=3, http_403=32 (stable), network_error=1083, pre_2000=37.</t>
+          <t>newspaper-scraper@northwestern; 59500 of 70720 (84.1%) as of 2026-10-04 23:44 UTC. empty_body=3420, http_403=32 (stable), network_error=1083.</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1071,7 @@
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan; 35593 of 119764 (29.7%) as of 2026-10-02 13:50 UTC. empty_body=14, http_301=1130, http_429=3, network_error=2. Watch 429s.</t>
+          <t>newspaper-scraper@michigan; 61043 of 119764 (51.0%) as of 2026-10-04 23:44 UTC. http_301=1821, http_429=15. Watch 429s.</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1117,7 @@
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@ucsd Cloudflare canary 10-14s. 5450 of 22605 (24.1%) as of 2026-10-02 13:50 UTC. empty_body=3, http_500=2.</t>
+          <t>newspaper-scraper@ucsd; 19850 of 22605 (87.8%) as of 2026-10-04 23:44 UTC. empty_body=1603, http_500=2. Closest Public finish after TSL.</t>
         </is>
       </c>
     </row>
@@ -1303,12 +1306,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="33" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>Stony Brook University</t>
         </is>
       </c>
-      <c r="B20" s="33" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>The Statesman</t>
         </is>
@@ -1328,12 +1331,14 @@
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F20" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G20" s="33" t="n"/>
+      <c r="F20" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G20" s="33" t="n">
+        <v>13354</v>
+      </c>
       <c r="H20" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1344,7 +1349,7 @@
       </c>
       <c r="J20" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@statesman Cloudflare SNO 10-14s. 5047 of 13650 (37.0%) as of 2026-10-02 13:50 UTC. empty_body=106.</t>
+          <t>Finished 2026-10-04. 13354 articles of 13650 URLs (97.8%); 517 empty_body, 32 pre_2000. systemd inactive. File: ~/Downloads/statesman.csv</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1399,12 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="0" t="inlineStr">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>University of California, Riverside</t>
         </is>
       </c>
-      <c r="B22" s="0" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>The Highlander</t>
         </is>
@@ -1419,10 +1424,13 @@
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F22" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
+      <c r="F22" s="38" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>9791</v>
       </c>
       <c r="H22" s="0" t="inlineStr">
         <is>
@@ -1434,189 +1442,180 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@highlander full run after 176/200 (24 empty_body). Resuming 176 of ~10144. Cloudflare Yoast WP 10-14 s. Public campus listed only on the National tab.</t>
+          <t>Finished 2026-10-04. 9791 articles of 10144 URLs (96.5%); 550 empty_body, 1 http_520, 1 http_525. systemd inactive. File: ~/Downloads/highlander.csv</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>University of Massachusetts, Amherst</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>The Massachusetts Daily Collegian</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>collegian</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>dailycollegian.com</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I23" s="37" t="n">
+        <v>46299</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Wave 11. Cloudflare SNO. wp-sitemap.xml (~52k URLs). Pace 10-14 s. Public flagship listed only on the National tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>University of Minnesota, Twin Cities</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>The Minnesota Daily</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>mndaily</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>mndaily.com</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I24" s="37" t="n">
+        <v>46299</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Wave 11. Cloudflare SNO Yoast (~81k URLs). Pace 10-14 s. Public flagship listed only on the National tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>University of Pittsburgh</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>The Pitt News</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>pitt</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>pittnews.com</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I25" s="37" t="n">
+        <v>46299</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Wave 11. Cloudflare SNO Yoast (~56k URLs). Pace 10-14 s. Public university listed only on the National tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n"/>
-      <c r="C23" s="32" t="n"/>
-      <c r="D23" s="32" t="n"/>
-      <c r="E23" s="32" t="n"/>
-      <c r="F23" s="32" t="n"/>
-      <c r="G23" s="32" t="n"/>
-      <c r="H23" s="32" t="n"/>
-      <c r="I23" s="32" t="n"/>
-      <c r="J23" s="32" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D24" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E24" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F24" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G24" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H24" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I24" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J24" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="24" t="inlineStr">
-        <is>
-          <t>Denison University</t>
-        </is>
-      </c>
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t>The Denisonian</t>
-        </is>
-      </c>
-      <c r="C25" s="33" t="inlineStr">
-        <is>
-          <t>denison</t>
-        </is>
-      </c>
-      <c r="D25" s="33" t="inlineStr">
-        <is>
-          <t>denisonian.com</t>
-        </is>
-      </c>
-      <c r="E25" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F25" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G25" s="30" t="n">
-        <v>3671</v>
-      </c>
-      <c r="H25" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I25" s="35" t="n">
-        <v>46294</v>
-      </c>
-      <c r="J25" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="24" t="inlineStr">
-        <is>
-          <t>Franklin &amp; Marshall College</t>
-        </is>
-      </c>
-      <c r="B26" s="33" t="inlineStr">
-        <is>
-          <t>The College Reporter</t>
-        </is>
-      </c>
-      <c r="C26" s="33" t="inlineStr">
-        <is>
-          <t>fandm</t>
-        </is>
-      </c>
-      <c r="D26" s="33" t="inlineStr">
-        <is>
-          <t>the-college-reporter.com</t>
-        </is>
-      </c>
-      <c r="E26" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F26" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G26" s="30" t="n">
-        <v>3449</v>
-      </c>
-      <c r="H26" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I26" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J26" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
-        </is>
-      </c>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="32" t="n"/>
+      <c r="F26" s="32" t="n"/>
+      <c r="G26" s="32" t="n"/>
+      <c r="H26" s="32" t="n"/>
+      <c r="I26" s="32" t="n"/>
+      <c r="J26" s="32" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>Hillsdale College</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B27" s="33" t="inlineStr">
         <is>
-          <t>The Collegian</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C27" s="33" t="inlineStr">
         <is>
-          <t>hillsdale</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D27" s="33" t="inlineStr">
         <is>
-          <t>hillsdalecollegian.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E27" s="33" t="inlineStr">
@@ -1630,7 +1629,7 @@
         </is>
       </c>
       <c r="G27" s="30" t="n">
-        <v>15573</v>
+        <v>4039</v>
       </c>
       <c r="H27" s="33" t="inlineStr">
         <is>
@@ -1642,29 +1641,29 @@
       </c>
       <c r="J27" s="34" t="inlineStr">
         <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="24" t="inlineStr">
         <is>
-          <t>Occidental College</t>
+          <t>Denison University</t>
         </is>
       </c>
       <c r="B28" s="33" t="inlineStr">
         <is>
-          <t>The Occidental</t>
+          <t>The Denisonian</t>
         </is>
       </c>
       <c r="C28" s="33" t="inlineStr">
         <is>
-          <t>occidental</t>
+          <t>denison</t>
         </is>
       </c>
       <c r="D28" s="33" t="inlineStr">
         <is>
-          <t>theoccidentalnews.com</t>
+          <t>denisonian.com</t>
         </is>
       </c>
       <c r="E28" s="33" t="inlineStr">
@@ -1678,7 +1677,7 @@
         </is>
       </c>
       <c r="G28" s="30" t="n">
-        <v>9892</v>
+        <v>3671</v>
       </c>
       <c r="H28" s="33" t="inlineStr">
         <is>
@@ -1686,33 +1685,33 @@
         </is>
       </c>
       <c r="I28" s="35" t="n">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="J28" s="34" t="inlineStr">
         <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>Swarthmore College</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B29" s="33" t="inlineStr">
         <is>
-          <t>The Phoenix</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C29" s="33" t="inlineStr">
         <is>
-          <t>swarthmore</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
-          <t>swarthmorephoenix.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E29" s="33" t="inlineStr">
@@ -1726,7 +1725,7 @@
         </is>
       </c>
       <c r="G29" s="30" t="n">
-        <v>12798</v>
+        <v>3449</v>
       </c>
       <c r="H29" s="33" t="inlineStr">
         <is>
@@ -1738,29 +1737,29 @@
       </c>
       <c r="J29" s="34" t="inlineStr">
         <is>
-          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>Union College (NY)</t>
+          <t>Hillsdale College</t>
         </is>
       </c>
       <c r="B30" s="33" t="inlineStr">
         <is>
-          <t>Concordiensis</t>
+          <t>The Collegian</t>
         </is>
       </c>
       <c r="C30" s="33" t="inlineStr">
         <is>
-          <t>union</t>
+          <t>hillsdale</t>
         </is>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
-          <t>concordiensis.com</t>
+          <t>hillsdalecollegian.com</t>
         </is>
       </c>
       <c r="E30" s="33" t="inlineStr">
@@ -1774,7 +1773,7 @@
         </is>
       </c>
       <c r="G30" s="30" t="n">
-        <v>1604</v>
+        <v>15573</v>
       </c>
       <c r="H30" s="33" t="inlineStr">
         <is>
@@ -1786,29 +1785,29 @@
       </c>
       <c r="J30" s="34" t="inlineStr">
         <is>
-          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>Wesleyan University</t>
+          <t>Occidental College</t>
         </is>
       </c>
       <c r="B31" s="33" t="inlineStr">
         <is>
-          <t>The Wesleyan Argus</t>
+          <t>The Occidental</t>
         </is>
       </c>
       <c r="C31" s="33" t="inlineStr">
         <is>
-          <t>wesleyan</t>
+          <t>occidental</t>
         </is>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
-          <t>wesleyanargus.com</t>
+          <t>theoccidentalnews.com</t>
         </is>
       </c>
       <c r="E31" s="33" t="inlineStr">
@@ -1821,8 +1820,8 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G31" s="24" t="n">
-        <v>21881</v>
+      <c r="G31" s="30" t="n">
+        <v>9892</v>
       </c>
       <c r="H31" s="33" t="inlineStr">
         <is>
@@ -1830,33 +1829,33 @@
         </is>
       </c>
       <c r="I31" s="35" t="n">
-        <v>46294</v>
+        <v>46292</v>
       </c>
       <c r="J31" s="34" t="inlineStr">
         <is>
-          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="33" t="inlineStr">
-        <is>
-          <t>Claremont Colleges</t>
+      <c r="A32" s="24" t="inlineStr">
+        <is>
+          <t>Swarthmore College</t>
         </is>
       </c>
       <c r="B32" s="33" t="inlineStr">
         <is>
-          <t>The Student Life</t>
+          <t>The Phoenix</t>
         </is>
       </c>
       <c r="C32" s="33" t="inlineStr">
         <is>
-          <t>tsl</t>
+          <t>swarthmore</t>
         </is>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
-          <t>tsl.news</t>
+          <t>swarthmorephoenix.com</t>
         </is>
       </c>
       <c r="E32" s="33" t="inlineStr">
@@ -1864,210 +1863,210 @@
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F32" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G32" s="33" t="n"/>
+      <c r="F32" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G32" s="30" t="n">
+        <v>12798</v>
+      </c>
       <c r="H32" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
       <c r="I32" s="35" t="n">
-        <v>46295</v>
+        <v>46292</v>
       </c>
       <c r="J32" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tsl; 9600 of 11437 (83.9%) as of 2026-10-02 13:50 UTC. empty_body=14, http_403=15. Closest to finishing.</t>
+          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="32" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="B33" s="32" t="n"/>
-      <c r="C33" s="32" t="n"/>
-      <c r="D33" s="32" t="n"/>
-      <c r="E33" s="32" t="n"/>
-      <c r="F33" s="32" t="n"/>
-      <c r="G33" s="32" t="n"/>
-      <c r="H33" s="32" t="n"/>
-      <c r="I33" s="32" t="n"/>
-      <c r="J33" s="32" t="n"/>
+      <c r="A33" s="24" t="inlineStr">
+        <is>
+          <t>Union College (NY)</t>
+        </is>
+      </c>
+      <c r="B33" s="33" t="inlineStr">
+        <is>
+          <t>Concordiensis</t>
+        </is>
+      </c>
+      <c r="C33" s="33" t="inlineStr">
+        <is>
+          <t>union</t>
+        </is>
+      </c>
+      <c r="D33" s="33" t="inlineStr">
+        <is>
+          <t>concordiensis.com</t>
+        </is>
+      </c>
+      <c r="E33" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F33" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G33" s="30" t="n">
+        <v>1604</v>
+      </c>
+      <c r="H33" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I33" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J33" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>Biola University</t>
+          <t>Wesleyan University</t>
         </is>
       </c>
       <c r="B34" s="33" t="inlineStr">
         <is>
-          <t>The Chimes</t>
+          <t>The Wesleyan Argus</t>
         </is>
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
-          <t>biola</t>
+          <t>wesleyan</t>
         </is>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
-          <t>chimesnewspaper.com</t>
+          <t>wesleyanargus.com</t>
         </is>
       </c>
       <c r="E34" s="33" t="inlineStr">
         <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>21881</v>
+      </c>
+      <c r="H34" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I34" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="J34" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>Claremont Colleges</t>
+        </is>
+      </c>
+      <c r="B35" s="33" t="inlineStr">
+        <is>
+          <t>The Student Life</t>
+        </is>
+      </c>
+      <c r="C35" s="33" t="inlineStr">
+        <is>
+          <t>tsl</t>
+        </is>
+      </c>
+      <c r="D35" s="33" t="inlineStr">
+        <is>
+          <t>tsl.news</t>
+        </is>
+      </c>
+      <c r="E35" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F35" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G35" s="33" t="n"/>
+      <c r="H35" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I35" s="35" t="n">
+        <v>46295</v>
+      </c>
+      <c r="J35" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tsl; 9600 of 11437 (83.9%) as of 2026-10-02 13:50 UTC. empty_body=14, http_403=15. Closest to finishing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="F34" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G34" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H34" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I34" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J34" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C35" s="33" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D35" s="33" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E35" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F35" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G35" s="30" t="n">
-        <v>682</v>
-      </c>
-      <c r="H35" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I35" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J35" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>Point Loma Nazarene University</t>
-        </is>
-      </c>
-      <c r="B36" s="33" t="inlineStr">
-        <is>
-          <t>Loma Beat</t>
-        </is>
-      </c>
-      <c r="C36" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat</t>
-        </is>
-      </c>
-      <c r="D36" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat.com</t>
-        </is>
-      </c>
-      <c r="E36" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F36" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G36" s="30" t="n">
-        <v>3950</v>
-      </c>
-      <c r="H36" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I36" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J36" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
-        </is>
-      </c>
+      <c r="B36" s="32" t="n"/>
+      <c r="C36" s="32" t="n"/>
+      <c r="D36" s="32" t="n"/>
+      <c r="E36" s="32" t="n"/>
+      <c r="F36" s="32" t="n"/>
+      <c r="G36" s="32" t="n"/>
+      <c r="H36" s="32" t="n"/>
+      <c r="I36" s="32" t="n"/>
+      <c r="J36" s="32" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>Southern Methodist University</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B37" s="33" t="inlineStr">
         <is>
-          <t>The Daily Campus</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C37" s="33" t="inlineStr">
         <is>
-          <t>smu</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D37" s="33" t="inlineStr">
         <is>
-          <t>smudailycampus.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E37" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | National Universities</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F37" s="24" t="inlineStr">
@@ -2076,7 +2075,7 @@
         </is>
       </c>
       <c r="G37" s="30" t="n">
-        <v>26208</v>
+        <v>11331</v>
       </c>
       <c r="H37" s="33" t="inlineStr">
         <is>
@@ -2088,34 +2087,34 @@
       </c>
       <c r="J37" s="34" t="inlineStr">
         <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Lipscomb University</t>
         </is>
       </c>
       <c r="B38" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>Lipscomb Media</t>
         </is>
       </c>
       <c r="C38" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>lipscomb</t>
         </is>
       </c>
       <c r="D38" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>lipscombmedia.com</t>
         </is>
       </c>
       <c r="E38" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F38" s="24" t="inlineStr">
@@ -2124,7 +2123,7 @@
         </is>
       </c>
       <c r="G38" s="30" t="n">
-        <v>5048</v>
+        <v>682</v>
       </c>
       <c r="H38" s="33" t="inlineStr">
         <is>
@@ -2136,53 +2135,197 @@
       </c>
       <c r="J38" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="24" t="inlineStr">
         <is>
+          <t>Point Loma Nazarene University</t>
+        </is>
+      </c>
+      <c r="B39" s="33" t="inlineStr">
+        <is>
+          <t>Loma Beat</t>
+        </is>
+      </c>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat</t>
+        </is>
+      </c>
+      <c r="D39" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat.com</t>
+        </is>
+      </c>
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G39" s="30" t="n">
+        <v>3950</v>
+      </c>
+      <c r="H39" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I39" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J39" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>Southern Methodist University</t>
+        </is>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Campus</t>
+        </is>
+      </c>
+      <c r="C40" s="33" t="inlineStr">
+        <is>
+          <t>smu</t>
+        </is>
+      </c>
+      <c r="D40" s="33" t="inlineStr">
+        <is>
+          <t>smudailycampus.com</t>
+        </is>
+      </c>
+      <c r="E40" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G40" s="30" t="n">
+        <v>26208</v>
+      </c>
+      <c r="H40" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I40" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J40" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B41" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C41" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D41" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E41" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F41" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G41" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H41" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I41" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J41" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="24" t="inlineStr">
+        <is>
           <t>Texas Christian University</t>
         </is>
       </c>
-      <c r="B39" s="33" t="inlineStr">
+      <c r="B42" s="33" t="inlineStr">
         <is>
           <t>TCU 360</t>
         </is>
       </c>
-      <c r="C39" s="33" t="inlineStr">
+      <c r="C42" s="33" t="inlineStr">
         <is>
           <t>tcu</t>
         </is>
       </c>
-      <c r="D39" s="33" t="inlineStr">
+      <c r="D42" s="33" t="inlineStr">
         <is>
           <t>tcu360.com</t>
         </is>
       </c>
-      <c r="E39" s="33" t="inlineStr">
+      <c r="E42" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F39" s="24" t="inlineStr">
+      <c r="F42" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G39" s="30" t="n">
+      <c r="G42" s="30" t="n">
         <v>25690</v>
       </c>
-      <c r="H39" s="33" t="inlineStr">
+      <c r="H42" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I39" s="35" t="n">
+      <c r="I42" s="35" t="n">
         <v>46291</v>
       </c>
-      <c r="J39" s="34" t="inlineStr">
+      <c r="J42" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>

</xml_diff>

<commit_message>
Add Clemson, NJIT, and Carleton, and skip Minnesota Daily 1990s URLs without fetching.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -920,12 +920,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>Duke University</t>
         </is>
       </c>
-      <c r="B11" s="33" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>The Chronicle</t>
         </is>
@@ -945,12 +945,14 @@
           <t>National Universities</t>
         </is>
       </c>
-      <c r="F11" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G11" s="33" t="n"/>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="n">
+        <v>22155</v>
+      </c>
       <c r="H11" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -961,7 +963,7 @@
       </c>
       <c r="J11" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@duke News-section listings only. 4600 rows as of 2026-10-02 13:50 UTC (no sitemap inventory). empty_body=17. Browser UA.</t>
+          <t>Finished 2026-10-05. News-section listings only, 22155 articles; 217 empty_body, 3 pre_2000. systemd inactive. Other Chronicle sections later. File: ~/Downloads/duke.csv</t>
         </is>
       </c>
     </row>
@@ -1076,12 +1078,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>University of California San Diego</t>
         </is>
       </c>
-      <c r="B15" s="33" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>The UCSD Guardian</t>
         </is>
@@ -1101,12 +1103,14 @@
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F15" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G15" s="33" t="n"/>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="n">
+        <v>21079</v>
+      </c>
       <c r="H15" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1117,7 +1121,7 @@
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@ucsd; 19850 of 22605 (87.8%) as of 2026-10-04 23:44 UTC. empty_body=1603, http_500=2. Closest Public finish after TSL.</t>
+          <t>Finished 2026-10-05. 21079 articles of 22605 URLs (93.2%); 1660 empty_body, 2 http_500. systemd inactive. File: ~/Downloads/ucsd.csv</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1433,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" s="0" t="n">
         <v>9791</v>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1447,37 +1451,37 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>University of Massachusetts, Amherst</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>The Massachusetts Daily Collegian</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>collegian</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>dailycollegian.com</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
+      <c r="F23" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H23" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -1485,44 +1489,44 @@
       <c r="I23" s="37" t="n">
         <v>46299</v>
       </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Wave 11. Cloudflare SNO. wp-sitemap.xml (~52k URLs). Pace 10-14 s. Public flagship listed only on the National tab.</t>
+      <c r="J23" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@collegian full run after 187/200 (2024 lastmod bucket). Resuming 187 of ~52k. Cloudflare SNO 10-14 s. /YYYY/MM/ pre-2000 skipped without fetch.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>University of Minnesota, Twin Cities</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>The Minnesota Daily</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>mndaily</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>mndaily.com</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
+      <c r="F24" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H24" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -1530,44 +1534,44 @@
       <c r="I24" s="37" t="n">
         <v>46299</v>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Wave 11. Cloudflare SNO Yoast (~81k URLs). Pace 10-14 s. Public flagship listed only on the National tab.</t>
+      <c r="J24" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@mndaily; 190 of 80516 after 200-test. Was fetching 1996 /MM/DD/YYYY/ URLs; permalink skip added 2026-10-05 so pre-2000 does not consume fetches. Restart after deploy.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>University of Pittsburgh</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>The Pitt News</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>pitt</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>pittnews.com</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="0" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -1575,143 +1579,137 @@
       <c r="I25" s="37" t="n">
         <v>46299</v>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Wave 11. Cloudflare SNO Yoast (~56k URLs). Pace 10-14 s. Public university listed only on the National tab.</t>
+      <c r="J25" s="0" t="inlineStr">
+        <is>
+          <t>Not cleared. VM 200-test hit HTTP 403 on /opinions/satire/ and entered block cooldown. Probe of two news articles was OK. Do not start full until a later 200-test passes.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Clemson University</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>The Tiger</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>tiger</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>thetigercu.com</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I26" s="37" t="n">
+        <v>46300</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Wave 12. Cloudflare SNO Yoast (~7.4k URLs). Pace 10-14 s. Public university listed only on the National tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>New Jersey Institute of Technology</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>The Vector</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>njitvector.com</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I27" s="37" t="n">
+        <v>46300</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Wave 12. Cloudflare SNO (~336 URLs). Pace 10-14 s. Public university listed only on the National tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="32" t="n"/>
-      <c r="G26" s="32" t="n"/>
-      <c r="H26" s="32" t="n"/>
-      <c r="I26" s="32" t="n"/>
-      <c r="J26" s="32" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B27" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C27" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D27" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E27" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F27" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G27" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H27" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I27" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J27" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="24" t="inlineStr">
-        <is>
-          <t>Denison University</t>
-        </is>
-      </c>
-      <c r="B28" s="33" t="inlineStr">
-        <is>
-          <t>The Denisonian</t>
-        </is>
-      </c>
-      <c r="C28" s="33" t="inlineStr">
-        <is>
-          <t>denison</t>
-        </is>
-      </c>
-      <c r="D28" s="33" t="inlineStr">
-        <is>
-          <t>denisonian.com</t>
-        </is>
-      </c>
-      <c r="E28" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F28" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G28" s="30" t="n">
-        <v>3671</v>
-      </c>
-      <c r="H28" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I28" s="35" t="n">
-        <v>46294</v>
-      </c>
-      <c r="J28" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
-        </is>
-      </c>
+      <c r="B28" s="32" t="n"/>
+      <c r="C28" s="32" t="n"/>
+      <c r="D28" s="32" t="n"/>
+      <c r="E28" s="32" t="n"/>
+      <c r="F28" s="32" t="n"/>
+      <c r="G28" s="32" t="n"/>
+      <c r="H28" s="32" t="n"/>
+      <c r="I28" s="32" t="n"/>
+      <c r="J28" s="32" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="24" t="inlineStr">
         <is>
-          <t>Franklin &amp; Marshall College</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B29" s="33" t="inlineStr">
         <is>
-          <t>The College Reporter</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C29" s="33" t="inlineStr">
         <is>
-          <t>fandm</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D29" s="33" t="inlineStr">
         <is>
-          <t>the-college-reporter.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E29" s="33" t="inlineStr">
@@ -1725,7 +1723,7 @@
         </is>
       </c>
       <c r="G29" s="30" t="n">
-        <v>3449</v>
+        <v>4039</v>
       </c>
       <c r="H29" s="33" t="inlineStr">
         <is>
@@ -1737,29 +1735,29 @@
       </c>
       <c r="J29" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="24" t="inlineStr">
         <is>
-          <t>Hillsdale College</t>
+          <t>Denison University</t>
         </is>
       </c>
       <c r="B30" s="33" t="inlineStr">
         <is>
-          <t>The Collegian</t>
+          <t>The Denisonian</t>
         </is>
       </c>
       <c r="C30" s="33" t="inlineStr">
         <is>
-          <t>hillsdale</t>
+          <t>denison</t>
         </is>
       </c>
       <c r="D30" s="33" t="inlineStr">
         <is>
-          <t>hillsdalecollegian.com</t>
+          <t>denisonian.com</t>
         </is>
       </c>
       <c r="E30" s="33" t="inlineStr">
@@ -1773,7 +1771,7 @@
         </is>
       </c>
       <c r="G30" s="30" t="n">
-        <v>15573</v>
+        <v>3671</v>
       </c>
       <c r="H30" s="33" t="inlineStr">
         <is>
@@ -1781,33 +1779,33 @@
         </is>
       </c>
       <c r="I30" s="35" t="n">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="J30" s="34" t="inlineStr">
         <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
+          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
         <is>
-          <t>Occidental College</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B31" s="33" t="inlineStr">
         <is>
-          <t>The Occidental</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C31" s="33" t="inlineStr">
         <is>
-          <t>occidental</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D31" s="33" t="inlineStr">
         <is>
-          <t>theoccidentalnews.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E31" s="33" t="inlineStr">
@@ -1821,7 +1819,7 @@
         </is>
       </c>
       <c r="G31" s="30" t="n">
-        <v>9892</v>
+        <v>3449</v>
       </c>
       <c r="H31" s="33" t="inlineStr">
         <is>
@@ -1833,29 +1831,29 @@
       </c>
       <c r="J31" s="34" t="inlineStr">
         <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="24" t="inlineStr">
         <is>
-          <t>Swarthmore College</t>
+          <t>Hillsdale College</t>
         </is>
       </c>
       <c r="B32" s="33" t="inlineStr">
         <is>
-          <t>The Phoenix</t>
+          <t>The Collegian</t>
         </is>
       </c>
       <c r="C32" s="33" t="inlineStr">
         <is>
-          <t>swarthmore</t>
+          <t>hillsdale</t>
         </is>
       </c>
       <c r="D32" s="33" t="inlineStr">
         <is>
-          <t>swarthmorephoenix.com</t>
+          <t>hillsdalecollegian.com</t>
         </is>
       </c>
       <c r="E32" s="33" t="inlineStr">
@@ -1869,7 +1867,7 @@
         </is>
       </c>
       <c r="G32" s="30" t="n">
-        <v>12798</v>
+        <v>15573</v>
       </c>
       <c r="H32" s="33" t="inlineStr">
         <is>
@@ -1881,29 +1879,29 @@
       </c>
       <c r="J32" s="34" t="inlineStr">
         <is>
-          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>Union College (NY)</t>
+          <t>Occidental College</t>
         </is>
       </c>
       <c r="B33" s="33" t="inlineStr">
         <is>
-          <t>Concordiensis</t>
+          <t>The Occidental</t>
         </is>
       </c>
       <c r="C33" s="33" t="inlineStr">
         <is>
-          <t>union</t>
+          <t>occidental</t>
         </is>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
-          <t>concordiensis.com</t>
+          <t>theoccidentalnews.com</t>
         </is>
       </c>
       <c r="E33" s="33" t="inlineStr">
@@ -1917,7 +1915,7 @@
         </is>
       </c>
       <c r="G33" s="30" t="n">
-        <v>1604</v>
+        <v>9892</v>
       </c>
       <c r="H33" s="33" t="inlineStr">
         <is>
@@ -1929,288 +1927,285 @@
       </c>
       <c r="J33" s="34" t="inlineStr">
         <is>
-          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D34" s="33" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E34" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F34" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G34" s="30" t="n">
+        <v>12798</v>
+      </c>
+      <c r="H34" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I34" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J34" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>Union College (NY)</t>
+        </is>
+      </c>
+      <c r="B35" s="33" t="inlineStr">
+        <is>
+          <t>Concordiensis</t>
+        </is>
+      </c>
+      <c r="C35" s="33" t="inlineStr">
+        <is>
+          <t>union</t>
+        </is>
+      </c>
+      <c r="D35" s="33" t="inlineStr">
+        <is>
+          <t>concordiensis.com</t>
+        </is>
+      </c>
+      <c r="E35" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G35" s="30" t="n">
+        <v>1604</v>
+      </c>
+      <c r="H35" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I35" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J35" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
           <t>Wesleyan University</t>
         </is>
       </c>
-      <c r="B34" s="33" t="inlineStr">
+      <c r="B36" s="33" t="inlineStr">
         <is>
           <t>The Wesleyan Argus</t>
         </is>
       </c>
-      <c r="C34" s="33" t="inlineStr">
+      <c r="C36" s="33" t="inlineStr">
         <is>
           <t>wesleyan</t>
         </is>
       </c>
-      <c r="D34" s="33" t="inlineStr">
+      <c r="D36" s="33" t="inlineStr">
         <is>
           <t>wesleyanargus.com</t>
         </is>
       </c>
-      <c r="E34" s="33" t="inlineStr">
+      <c r="E36" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F34" s="24" t="inlineStr">
+      <c r="F36" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G34" s="24" t="n">
+      <c r="G36" s="24" t="n">
         <v>21881</v>
       </c>
-      <c r="H34" s="33" t="inlineStr">
+      <c r="H36" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I34" s="35" t="n">
+      <c r="I36" s="35" t="n">
         <v>46294</v>
       </c>
-      <c r="J34" s="34" t="inlineStr">
+      <c r="J36" s="34" t="inlineStr">
         <is>
           <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="33" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="33" t="inlineStr">
         <is>
           <t>Claremont Colleges</t>
         </is>
       </c>
-      <c r="B35" s="33" t="inlineStr">
+      <c r="B37" s="33" t="inlineStr">
         <is>
           <t>The Student Life</t>
         </is>
       </c>
-      <c r="C35" s="33" t="inlineStr">
+      <c r="C37" s="33" t="inlineStr">
         <is>
           <t>tsl</t>
         </is>
       </c>
-      <c r="D35" s="33" t="inlineStr">
+      <c r="D37" s="33" t="inlineStr">
         <is>
           <t>tsl.news</t>
         </is>
       </c>
-      <c r="E35" s="33" t="inlineStr">
+      <c r="E37" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F35" s="33" t="inlineStr">
+      <c r="F37" s="33" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G35" s="33" t="n"/>
-      <c r="H35" s="33" t="inlineStr">
+      <c r="G37" s="33" t="n"/>
+      <c r="H37" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I35" s="35" t="n">
+      <c r="I37" s="35" t="n">
         <v>46295</v>
       </c>
-      <c r="J35" s="34" t="inlineStr">
+      <c r="J37" s="34" t="inlineStr">
         <is>
           <t>newspaper-scraper@tsl; 9600 of 11437 (83.9%) as of 2026-10-02 13:50 UTC. empty_body=14, http_403=15. Closest to finishing.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="32" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Carleton College</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>The Carletonian</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>carleton</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>thecarletonian.com</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I38" s="37" t="n">
+        <v>46300</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Wave 12. Cloudflare SNO (~7.9k URLs). Pace 10-14 s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B36" s="32" t="n"/>
-      <c r="C36" s="32" t="n"/>
-      <c r="D36" s="32" t="n"/>
-      <c r="E36" s="32" t="n"/>
-      <c r="F36" s="32" t="n"/>
-      <c r="G36" s="32" t="n"/>
-      <c r="H36" s="32" t="n"/>
-      <c r="I36" s="32" t="n"/>
-      <c r="J36" s="32" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B37" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C37" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D37" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E37" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F37" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G37" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H37" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I37" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J37" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="24" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B38" s="33" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C38" s="33" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D38" s="33" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E38" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F38" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G38" s="30" t="n">
-        <v>682</v>
-      </c>
-      <c r="H38" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I38" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J38" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>Point Loma Nazarene University</t>
-        </is>
-      </c>
-      <c r="B39" s="33" t="inlineStr">
-        <is>
-          <t>Loma Beat</t>
-        </is>
-      </c>
-      <c r="C39" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat</t>
-        </is>
-      </c>
-      <c r="D39" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat.com</t>
-        </is>
-      </c>
-      <c r="E39" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F39" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G39" s="30" t="n">
-        <v>3950</v>
-      </c>
-      <c r="H39" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I39" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J39" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
-        </is>
-      </c>
+      <c r="B39" s="32" t="n"/>
+      <c r="C39" s="32" t="n"/>
+      <c r="D39" s="32" t="n"/>
+      <c r="E39" s="32" t="n"/>
+      <c r="F39" s="32" t="n"/>
+      <c r="G39" s="32" t="n"/>
+      <c r="H39" s="32" t="n"/>
+      <c r="I39" s="32" t="n"/>
+      <c r="J39" s="32" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="24" t="inlineStr">
         <is>
-          <t>Southern Methodist University</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B40" s="33" t="inlineStr">
         <is>
-          <t>The Daily Campus</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C40" s="33" t="inlineStr">
         <is>
-          <t>smu</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D40" s="33" t="inlineStr">
         <is>
-          <t>smudailycampus.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E40" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | National Universities</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F40" s="24" t="inlineStr">
@@ -2219,7 +2214,7 @@
         </is>
       </c>
       <c r="G40" s="30" t="n">
-        <v>26208</v>
+        <v>11331</v>
       </c>
       <c r="H40" s="33" t="inlineStr">
         <is>
@@ -2231,34 +2226,34 @@
       </c>
       <c r="J40" s="34" t="inlineStr">
         <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Lipscomb University</t>
         </is>
       </c>
       <c r="B41" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>Lipscomb Media</t>
         </is>
       </c>
       <c r="C41" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>lipscomb</t>
         </is>
       </c>
       <c r="D41" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>lipscombmedia.com</t>
         </is>
       </c>
       <c r="E41" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F41" s="24" t="inlineStr">
@@ -2267,7 +2262,7 @@
         </is>
       </c>
       <c r="G41" s="30" t="n">
-        <v>5048</v>
+        <v>682</v>
       </c>
       <c r="H41" s="33" t="inlineStr">
         <is>
@@ -2279,53 +2274,197 @@
       </c>
       <c r="J41" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="24" t="inlineStr">
         <is>
+          <t>Point Loma Nazarene University</t>
+        </is>
+      </c>
+      <c r="B42" s="33" t="inlineStr">
+        <is>
+          <t>Loma Beat</t>
+        </is>
+      </c>
+      <c r="C42" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat</t>
+        </is>
+      </c>
+      <c r="D42" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat.com</t>
+        </is>
+      </c>
+      <c r="E42" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F42" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G42" s="30" t="n">
+        <v>3950</v>
+      </c>
+      <c r="H42" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I42" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J42" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="24" t="inlineStr">
+        <is>
+          <t>Southern Methodist University</t>
+        </is>
+      </c>
+      <c r="B43" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Campus</t>
+        </is>
+      </c>
+      <c r="C43" s="33" t="inlineStr">
+        <is>
+          <t>smu</t>
+        </is>
+      </c>
+      <c r="D43" s="33" t="inlineStr">
+        <is>
+          <t>smudailycampus.com</t>
+        </is>
+      </c>
+      <c r="E43" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F43" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G43" s="30" t="n">
+        <v>26208</v>
+      </c>
+      <c r="H43" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I43" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J43" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B44" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C44" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E44" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F44" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G44" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H44" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I44" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J44" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="24" t="inlineStr">
+        <is>
           <t>Texas Christian University</t>
         </is>
       </c>
-      <c r="B42" s="33" t="inlineStr">
+      <c r="B45" s="33" t="inlineStr">
         <is>
           <t>TCU 360</t>
         </is>
       </c>
-      <c r="C42" s="33" t="inlineStr">
+      <c r="C45" s="33" t="inlineStr">
         <is>
           <t>tcu</t>
         </is>
       </c>
-      <c r="D42" s="33" t="inlineStr">
+      <c r="D45" s="33" t="inlineStr">
         <is>
           <t>tcu360.com</t>
         </is>
       </c>
-      <c r="E42" s="33" t="inlineStr">
+      <c r="E45" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F42" s="24" t="inlineStr">
+      <c r="F45" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G42" s="30" t="n">
+      <c r="G45" s="30" t="n">
         <v>25690</v>
       </c>
-      <c r="H42" s="33" t="inlineStr">
+      <c r="H45" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I42" s="35" t="n">
+      <c r="I45" s="35" t="n">
         <v>46291</v>
       </c>
-      <c r="J42" s="34" t="inlineStr">
+      <c r="J45" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>

</xml_diff>

<commit_message>
Add Mac Weekly and Scarlet & Black to refill two Liberal Arts slots.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -732,12 +732,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Northwestern University</t>
         </is>
       </c>
-      <c r="B7" s="33" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>The Daily Northwestern</t>
         </is>
@@ -757,12 +757,14 @@
           <t>National Universities</t>
         </is>
       </c>
-      <c r="F7" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G7" s="33" t="n"/>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="n">
+        <v>69041</v>
+      </c>
       <c r="H7" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -773,7 +775,7 @@
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@northwestern; 59500 of 70720 (84.1%) as of 2026-10-04 23:44 UTC. empty_body=3420, http_403=32 (stable), network_error=1083.</t>
+          <t>Finished 2026-10-06. 69041 articles of 70720 URLs (97.6%); empty_body=3558, http_301=11, http_403=32, network_error=1083, pre_2000=46. systemd inactive. File: ~/Downloads/northwestern.csv</t>
         </is>
       </c>
     </row>
@@ -963,7 +965,7 @@
       </c>
       <c r="J11" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-05. News-section listings only, 22155 articles; 217 empty_body, 3 pre_2000. systemd inactive. Other Chronicle sections later. File: ~/Downloads/duke.csv</t>
+          <t>Finished 2026-10-05. News-section listings only, 22155 articles; 217 empty_body, 3 pre_2000. Other Chronicle sections later. File: ~/Downloads/duke.csv</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1075,7 @@
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan; 61043 of 119764 (51.0%) as of 2026-10-04 23:44 UTC. http_301=1821, http_429=15. Watch 429s.</t>
+          <t>newspaper-scraper@michigan; 78143 of 119764 (65.2%) as of 2026-10-06 14:31 UTC. http_429=15 (stable).</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1123,7 @@
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-05. 21079 articles of 22605 URLs (93.2%); 1660 empty_body, 2 http_500. systemd inactive. File: ~/Downloads/ucsd.csv</t>
+          <t>Finished 2026-10-05 before later downloads. 21079 articles of 22605 URLs (93.2%); 1660 empty_body, 2 http_500. systemd inactive. File: ~/Downloads/ucsd.csv</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1169,7 @@
       </c>
       <c r="J16" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@texan Cloudflare SNO 10-14s. 4747 of 51636 (9.2%) as of 2026-10-02 13:50 UTC. empty_body=74, http_500=3.</t>
+          <t>newspaper-scraper@texan; 31397 of 51636 (60.8%) as of 2026-10-06 14:31 UTC.</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1215,7 @@
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@nexus Cloudflare WP 10-14s. 4637 of 40465 (11.5%) as of 2026-10-02 13:50 UTC. empty_body=453 (high; photo features). Watch.</t>
+          <t>newspaper-scraper@nexus; 28787 of 40465 (71.1%) as of 2026-10-06 14:31 UTC. empty_body=3838.</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1261,7 @@
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@illini Cloudflare SNO 10-14s. 4900 of 100022 (4.9%) as of 2026-10-02 13:50 UTC. http_500=1, pre_2000=10.</t>
+          <t>newspaper-scraper@illini; 31000 of 100022 (31.0%) as of 2026-10-06 14:31 UTC.</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1307,7 @@
       </c>
       <c r="J19" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@technician Cloudflare SNO 10-14s. 5083 of 41051 (12.4%) as of 2026-10-02 13:50 UTC. empty_body=82.</t>
+          <t>newspaper-scraper@technician; 32283 of 41051 (78.6%) as of 2026-10-06 14:31 UTC. empty_body=750.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1355,7 @@
       </c>
       <c r="J20" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-04. 13354 articles of 13650 URLs (97.8%); 517 empty_body, 32 pre_2000. systemd inactive. File: ~/Downloads/statesman.csv</t>
+          <t>Finished 2026-10-04. 13354 of 13650 (97.8%); 517 empty_body, 32 pre_2000. File: ~/Downloads/statesman.csv</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1400,7 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tarheel full run after 129/200 (71 empty_body, almost all /multimedia/ galleries and videos; those URLs now excluded). Resuming 129 of ~82k. Cloudflare SNO 10-14 s.</t>
+          <t>newspaper-scraper@tarheel; 23379 of 81683 (28.6%) as of 2026-10-06 14:31 UTC. empty_body=3581, http_403=19.</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1448,7 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t>Finished 2026-10-04. 9791 articles of 10144 URLs (96.5%); 550 empty_body, 1 http_520, 1 http_525. systemd inactive. File: ~/Downloads/highlander.csv</t>
+          <t>Finished 2026-10-04. 9791 of 10144 (96.5%); 550 empty_body, 1 http_520, 1 http_525. File: ~/Downloads/highlander.csv</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1493,7 @@
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@collegian full run after 187/200 (2024 lastmod bucket). Resuming 187 of ~52k. Cloudflare SNO 10-14 s. /YYYY/MM/ pre-2000 skipped without fetch.</t>
+          <t>newspaper-scraper@collegian; 10537 of 52185 (20.2%) as of 2026-10-06 14:31 UTC. empty_body=26, pre_2000=234.</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1538,7 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@mndaily; 190 of 80516 after 200-test. Was fetching 1996 /MM/DD/YYYY/ URLs; permalink skip added 2026-10-05 so pre-2000 does not consume fetches. Restart after deploy.</t>
+          <t>newspaper-scraper@mndaily; 7240 of 80516 (9.0%) as of 2026-10-06 14:31 UTC. pre_2000=14440 skipped.</t>
         </is>
       </c>
     </row>
@@ -1581,42 +1583,42 @@
       </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t>Not cleared. VM 200-test hit HTTP 403 on /opinions/satire/ and entered block cooldown. Probe of two news articles was OK. Do not start full until a later 200-test passes.</t>
+          <t>Not cleared. VM 200-test HTTP 403 on /opinions/satire/; block cooldown. Probe of two news articles OK. Do not start full until a later 200-test passes.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>Clemson University</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>The Tiger</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>tiger</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>thetigercu.com</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
+      <c r="F26" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H26" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -1624,44 +1626,47 @@
       <c r="I26" s="37" t="n">
         <v>46300</v>
       </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Wave 12. Cloudflare SNO Yoast (~7.4k URLs). Pace 10-14 s. Public university listed only on the National tab.</t>
+      <c r="J26" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tiger; 5688 of 7455 (76.3%) as of 2026-10-06 14:31 UTC. empty_body=125.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="38" t="inlineStr">
         <is>
           <t>New Jersey Institute of Technology</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="38" t="inlineStr">
         <is>
           <t>The Vector</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>vector</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>njitvector.com</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
+      <c r="F27" s="38" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G27" s="0" t="n">
+        <v>335</v>
+      </c>
+      <c r="H27" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -1669,9 +1674,9 @@
       <c r="I27" s="37" t="n">
         <v>46300</v>
       </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Wave 12. Cloudflare SNO (~336 URLs). Pace 10-14 s. Public university listed only on the National tab.</t>
+      <c r="J27" s="0" t="inlineStr">
+        <is>
+          <t>Finished 2026-10-05. 335 of 336 (99.7%); 1 empty_body. File: ~/Downloads/vector.csv</t>
         </is>
       </c>
     </row>
@@ -2076,12 +2081,12 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="33" t="inlineStr">
+      <c r="A37" s="24" t="inlineStr">
         <is>
           <t>Claremont Colleges</t>
         </is>
       </c>
-      <c r="B37" s="33" t="inlineStr">
+      <c r="B37" s="24" t="inlineStr">
         <is>
           <t>The Student Life</t>
         </is>
@@ -2101,12 +2106,14 @@
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F37" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G37" s="33" t="n"/>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G37" s="33" t="n">
+        <v>11405</v>
+      </c>
       <c r="H37" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -2117,42 +2124,42 @@
       </c>
       <c r="J37" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tsl; 9600 of 11437 (83.9%) as of 2026-10-02 13:50 UTC. empty_body=14, http_403=15. Closest to finishing.</t>
+          <t>Finished 2026-10-04. 11405 of 11437 (99.7%); 16 empty_body, 15 http_403, 1 http_404. File: ~/Downloads/tsl.csv</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="0" t="inlineStr">
         <is>
           <t>Carleton College</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>The Carletonian</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>carleton</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>thecarletonian.com</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="0" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
+      <c r="F38" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H38" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
@@ -2160,143 +2167,137 @@
       <c r="I38" s="37" t="n">
         <v>46300</v>
       </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>Wave 12. Cloudflare SNO (~7.9k URLs). Pace 10-14 s.</t>
+      <c r="J38" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@carleton; 5800 of 7941 (73.0%) as of 2026-10-06 14:31 UTC. empty_body=14.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="32" t="inlineStr">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>Macalester College</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>The Mac Weekly</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>macweekly</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>themacweekly.com</t>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F39" s="0" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H39" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I39" s="37" t="n">
+        <v>46301</v>
+      </c>
+      <c r="J39" s="0" t="inlineStr">
+        <is>
+          <t>Wave 13 Liberal Arts SNO (Yoast). ~9418 URLs, Cloudflare 10–14 s. Fills a slot after Northwestern. Probe + 200-test next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>Grinnell College</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>Scarlet &amp; Black</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>sandb</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>thesandb.com</t>
+        </is>
+      </c>
+      <c r="E40" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F40" s="0" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="H40" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I40" s="37" t="n">
+        <v>46301</v>
+      </c>
+      <c r="J40" s="0" t="inlineStr">
+        <is>
+          <t>Wave 13 Liberal Arts SNO. ~9196 URLs, Cloudflare 10–14 s. Use wp-sitemap.xml. Fills a slot after Vector. Probe + 200-test next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B39" s="32" t="n"/>
-      <c r="C39" s="32" t="n"/>
-      <c r="D39" s="32" t="n"/>
-      <c r="E39" s="32" t="n"/>
-      <c r="F39" s="32" t="n"/>
-      <c r="G39" s="32" t="n"/>
-      <c r="H39" s="32" t="n"/>
-      <c r="I39" s="32" t="n"/>
-      <c r="J39" s="32" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B40" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C40" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D40" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E40" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F40" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G40" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H40" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I40" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J40" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="24" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B41" s="33" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C41" s="33" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D41" s="33" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E41" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F41" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G41" s="30" t="n">
-        <v>682</v>
-      </c>
-      <c r="H41" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I41" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J41" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
-        </is>
-      </c>
+      <c r="B41" s="32" t="n"/>
+      <c r="C41" s="32" t="n"/>
+      <c r="D41" s="32" t="n"/>
+      <c r="E41" s="32" t="n"/>
+      <c r="F41" s="32" t="n"/>
+      <c r="G41" s="32" t="n"/>
+      <c r="H41" s="32" t="n"/>
+      <c r="I41" s="32" t="n"/>
+      <c r="J41" s="32" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="24" t="inlineStr">
         <is>
-          <t>Point Loma Nazarene University</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B42" s="33" t="inlineStr">
         <is>
-          <t>Loma Beat</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C42" s="33" t="inlineStr">
         <is>
-          <t>lomabeat</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D42" s="33" t="inlineStr">
         <is>
-          <t>lomabeat.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E42" s="33" t="inlineStr">
@@ -2310,7 +2311,7 @@
         </is>
       </c>
       <c r="G42" s="30" t="n">
-        <v>3950</v>
+        <v>11331</v>
       </c>
       <c r="H42" s="33" t="inlineStr">
         <is>
@@ -2318,38 +2319,38 @@
         </is>
       </c>
       <c r="I42" s="35" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="J42" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="24" t="inlineStr">
         <is>
-          <t>Southern Methodist University</t>
+          <t>Lipscomb University</t>
         </is>
       </c>
       <c r="B43" s="33" t="inlineStr">
         <is>
-          <t>The Daily Campus</t>
+          <t>Lipscomb Media</t>
         </is>
       </c>
       <c r="C43" s="33" t="inlineStr">
         <is>
-          <t>smu</t>
+          <t>lipscomb</t>
         </is>
       </c>
       <c r="D43" s="33" t="inlineStr">
         <is>
-          <t>smudailycampus.com</t>
+          <t>lipscombmedia.com</t>
         </is>
       </c>
       <c r="E43" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | National Universities</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F43" s="24" t="inlineStr">
@@ -2358,7 +2359,7 @@
         </is>
       </c>
       <c r="G43" s="30" t="n">
-        <v>26208</v>
+        <v>682</v>
       </c>
       <c r="H43" s="33" t="inlineStr">
         <is>
@@ -2366,38 +2367,38 @@
         </is>
       </c>
       <c r="I43" s="35" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="J43" s="34" t="inlineStr">
         <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Point Loma Nazarene University</t>
         </is>
       </c>
       <c r="B44" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>Loma Beat</t>
         </is>
       </c>
       <c r="C44" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>lomabeat</t>
         </is>
       </c>
       <c r="D44" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>lomabeat.com</t>
         </is>
       </c>
       <c r="E44" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F44" s="24" t="inlineStr">
@@ -2406,7 +2407,7 @@
         </is>
       </c>
       <c r="G44" s="30" t="n">
-        <v>5048</v>
+        <v>3950</v>
       </c>
       <c r="H44" s="33" t="inlineStr">
         <is>
@@ -2414,33 +2415,33 @@
         </is>
       </c>
       <c r="I44" s="35" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="J44" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>Texas Christian University</t>
+          <t>Southern Methodist University</t>
         </is>
       </c>
       <c r="B45" s="33" t="inlineStr">
         <is>
-          <t>TCU 360</t>
+          <t>The Daily Campus</t>
         </is>
       </c>
       <c r="C45" s="33" t="inlineStr">
         <is>
-          <t>tcu</t>
+          <t>smu</t>
         </is>
       </c>
       <c r="D45" s="33" t="inlineStr">
         <is>
-          <t>tcu360.com</t>
+          <t>smudailycampus.com</t>
         </is>
       </c>
       <c r="E45" s="33" t="inlineStr">
@@ -2454,7 +2455,7 @@
         </is>
       </c>
       <c r="G45" s="30" t="n">
-        <v>25690</v>
+        <v>26208</v>
       </c>
       <c r="H45" s="33" t="inlineStr">
         <is>
@@ -2465,6 +2466,102 @@
         <v>46291</v>
       </c>
       <c r="J45" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B46" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C46" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D46" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E46" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F46" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G46" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H46" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I46" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J46" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t>Texas Christian University</t>
+        </is>
+      </c>
+      <c r="B47" s="33" t="inlineStr">
+        <is>
+          <t>TCU 360</t>
+        </is>
+      </c>
+      <c r="C47" s="33" t="inlineStr">
+        <is>
+          <t>tcu</t>
+        </is>
+      </c>
+      <c r="D47" s="33" t="inlineStr">
+        <is>
+          <t>tcu360.com</t>
+        </is>
+      </c>
+      <c r="E47" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F47" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G47" s="30" t="n">
+        <v>25690</v>
+      </c>
+      <c r="H47" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I47" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J47" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>

</xml_diff>

<commit_message>
Mark Mac Weekly and Scarlet & Black running after their 200-tests passed.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -2201,8 +2201,11 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>191</v>
       </c>
       <c r="H39" s="0" t="inlineStr">
         <is>
@@ -2214,7 +2217,7 @@
       </c>
       <c r="J39" s="0" t="inlineStr">
         <is>
-          <t>Wave 13 Liberal Arts SNO (Yoast). ~9418 URLs, Cloudflare 10–14 s. Fills a slot after Northwestern. Probe + 200-test next.</t>
+          <t>newspaper-scraper@macweekly; 200-test OK (191/200, empty_body=9). systemd enabled 2026-10-06 16:28 UTC. Liberal Arts SNO Yoast, ~9420 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
         </is>
       </c>
     </row>
@@ -2246,8 +2249,11 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>190</v>
       </c>
       <c r="H40" s="0" t="inlineStr">
         <is>
@@ -2259,7 +2265,7 @@
       </c>
       <c r="J40" s="0" t="inlineStr">
         <is>
-          <t>Wave 13 Liberal Arts SNO. ~9196 URLs, Cloudflare 10–14 s. Use wp-sitemap.xml. Fills a slot after Vector. Probe + 200-test next.</t>
+          <t>newspaper-scraper@sandb; 200-test OK (190/200, empty_body=10, mostly comics/photos). systemd enabled 2026-10-06 16:28 UTC. Liberal Arts SNO, ~9228 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Colgate Maroon-News and The Bucknellian to refill two Liberal Arts slots.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -1615,8 +1615,11 @@
       </c>
       <c r="F26" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>7337</v>
       </c>
       <c r="H26" s="0" t="inlineStr">
         <is>
@@ -1628,7 +1631,7 @@
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tiger; 5688 of 7455 (76.3%) as of 2026-10-06 14:31 UTC. empty_body=125.</t>
+          <t>Finished 2026-10-06. 7337 of 7455 (98.4%); empty_body=130. systemd inactive. File: ~/Downloads/tiger.csv</t>
         </is>
       </c>
     </row>
@@ -2156,8 +2159,11 @@
       </c>
       <c r="F38" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>7805</v>
       </c>
       <c r="H38" s="0" t="inlineStr">
         <is>
@@ -2169,7 +2175,7 @@
       </c>
       <c r="J38" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@carleton; 5800 of 7941 (73.0%) as of 2026-10-06 14:31 UTC. empty_body=14.</t>
+          <t>Finished 2026-10-06. 7805 of 7941 (98.3%); empty_body=135, http_404=1. systemd inactive. File: ~/Downloads/carleton.csv</t>
         </is>
       </c>
     </row>
@@ -2204,8 +2210,8 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G39" t="n">
-        <v>191</v>
+      <c r="G39" s="0" t="n">
+        <v>6141</v>
       </c>
       <c r="H39" s="0" t="inlineStr">
         <is>
@@ -2217,7 +2223,7 @@
       </c>
       <c r="J39" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@macweekly; 200-test OK (191/200, empty_body=9). systemd enabled 2026-10-06 16:28 UTC. Liberal Arts SNO Yoast, ~9420 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
+          <t>newspaper-scraper@macweekly; 6141 of 9420 (65.2%) as of 2026-10-07 14:02 UTC. empty_body=218.</t>
         </is>
       </c>
     </row>
@@ -2252,8 +2258,8 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G40" t="n">
-        <v>190</v>
+      <c r="G40" s="0" t="n">
+        <v>6190</v>
       </c>
       <c r="H40" s="0" t="inlineStr">
         <is>
@@ -2265,141 +2271,137 @@
       </c>
       <c r="J40" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@sandb; 200-test OK (190/200, empty_body=10, mostly comics/photos). systemd enabled 2026-10-06 16:28 UTC. Liberal Arts SNO, ~9228 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
+          <t>newspaper-scraper@sandb; 6190 of 9228 (67.1%) as of 2026-10-07 14:02 UTC. empty_body=80.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="32" t="inlineStr">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>Colgate University</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>The Colgate Maroon-News</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>colgate</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>thecolgatemaroonnews.com</t>
+        </is>
+      </c>
+      <c r="E41" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F41" s="0" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G41" s="0" t="n"/>
+      <c r="H41" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I41" s="37" t="n">
+        <v>46302</v>
+      </c>
+      <c r="J41" s="0" t="inlineStr">
+        <is>
+          <t>Wave 14 Liberal Arts SNO. ~15458 URLs, Cloudflare 10–14 s. Use wp-sitemap.xml. Fills a slot after Carleton. Probe + 200-test next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>Bucknell University</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>The Bucknellian</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>bucknellian</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>bucknellian.net</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="n"/>
+      <c r="H42" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I42" s="37" t="n">
+        <v>46302</v>
+      </c>
+      <c r="J42" s="0" t="inlineStr">
+        <is>
+          <t>Wave 14 Liberal Arts SNO (Yoast). ~11585 URLs, Cloudflare 10–14 s. Fills a slot after Clemson. Probe + 200-test next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B41" s="32" t="n"/>
-      <c r="C41" s="32" t="n"/>
-      <c r="D41" s="32" t="n"/>
-      <c r="E41" s="32" t="n"/>
-      <c r="F41" s="32" t="n"/>
-      <c r="G41" s="32" t="n"/>
-      <c r="H41" s="32" t="n"/>
-      <c r="I41" s="32" t="n"/>
-      <c r="J41" s="32" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B42" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C42" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D42" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E42" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F42" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G42" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H42" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I42" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J42" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="24" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B43" s="33" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C43" s="33" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D43" s="33" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E43" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F43" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G43" s="30" t="n">
-        <v>682</v>
-      </c>
-      <c r="H43" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I43" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J43" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
-        </is>
-      </c>
+      <c r="B43" s="32" t="n"/>
+      <c r="C43" s="32" t="n"/>
+      <c r="D43" s="32" t="n"/>
+      <c r="E43" s="32" t="n"/>
+      <c r="F43" s="32" t="n"/>
+      <c r="G43" s="32" t="n"/>
+      <c r="H43" s="32" t="n"/>
+      <c r="I43" s="32" t="n"/>
+      <c r="J43" s="32" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="24" t="inlineStr">
         <is>
-          <t>Point Loma Nazarene University</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B44" s="33" t="inlineStr">
         <is>
-          <t>Loma Beat</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C44" s="33" t="inlineStr">
         <is>
-          <t>lomabeat</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D44" s="33" t="inlineStr">
         <is>
-          <t>lomabeat.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E44" s="33" t="inlineStr">
@@ -2413,7 +2415,7 @@
         </is>
       </c>
       <c r="G44" s="30" t="n">
-        <v>3950</v>
+        <v>11331</v>
       </c>
       <c r="H44" s="33" t="inlineStr">
         <is>
@@ -2421,38 +2423,38 @@
         </is>
       </c>
       <c r="I44" s="35" t="n">
-        <v>46293</v>
+        <v>46291</v>
       </c>
       <c r="J44" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="24" t="inlineStr">
         <is>
-          <t>Southern Methodist University</t>
+          <t>Lipscomb University</t>
         </is>
       </c>
       <c r="B45" s="33" t="inlineStr">
         <is>
-          <t>The Daily Campus</t>
+          <t>Lipscomb Media</t>
         </is>
       </c>
       <c r="C45" s="33" t="inlineStr">
         <is>
-          <t>smu</t>
+          <t>lipscomb</t>
         </is>
       </c>
       <c r="D45" s="33" t="inlineStr">
         <is>
-          <t>smudailycampus.com</t>
+          <t>lipscombmedia.com</t>
         </is>
       </c>
       <c r="E45" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | National Universities</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F45" s="24" t="inlineStr">
@@ -2461,7 +2463,7 @@
         </is>
       </c>
       <c r="G45" s="30" t="n">
-        <v>26208</v>
+        <v>682</v>
       </c>
       <c r="H45" s="33" t="inlineStr">
         <is>
@@ -2469,38 +2471,38 @@
         </is>
       </c>
       <c r="I45" s="35" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="J45" s="34" t="inlineStr">
         <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Point Loma Nazarene University</t>
         </is>
       </c>
       <c r="B46" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>Loma Beat</t>
         </is>
       </c>
       <c r="C46" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>lomabeat</t>
         </is>
       </c>
       <c r="D46" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>lomabeat.com</t>
         </is>
       </c>
       <c r="E46" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F46" s="24" t="inlineStr">
@@ -2509,7 +2511,7 @@
         </is>
       </c>
       <c r="G46" s="30" t="n">
-        <v>5048</v>
+        <v>3950</v>
       </c>
       <c r="H46" s="33" t="inlineStr">
         <is>
@@ -2517,33 +2519,33 @@
         </is>
       </c>
       <c r="I46" s="35" t="n">
-        <v>46292</v>
+        <v>46293</v>
       </c>
       <c r="J46" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="24" t="inlineStr">
         <is>
-          <t>Texas Christian University</t>
+          <t>Southern Methodist University</t>
         </is>
       </c>
       <c r="B47" s="33" t="inlineStr">
         <is>
-          <t>TCU 360</t>
+          <t>The Daily Campus</t>
         </is>
       </c>
       <c r="C47" s="33" t="inlineStr">
         <is>
-          <t>tcu</t>
+          <t>smu</t>
         </is>
       </c>
       <c r="D47" s="33" t="inlineStr">
         <is>
-          <t>tcu360.com</t>
+          <t>smudailycampus.com</t>
         </is>
       </c>
       <c r="E47" s="33" t="inlineStr">
@@ -2557,7 +2559,7 @@
         </is>
       </c>
       <c r="G47" s="30" t="n">
-        <v>25690</v>
+        <v>26208</v>
       </c>
       <c r="H47" s="33" t="inlineStr">
         <is>
@@ -2568,6 +2570,102 @@
         <v>46291</v>
       </c>
       <c r="J47" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B48" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C48" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D48" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E48" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F48" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G48" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H48" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I48" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J48" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="24" t="inlineStr">
+        <is>
+          <t>Texas Christian University</t>
+        </is>
+      </c>
+      <c r="B49" s="33" t="inlineStr">
+        <is>
+          <t>TCU 360</t>
+        </is>
+      </c>
+      <c r="C49" s="33" t="inlineStr">
+        <is>
+          <t>tcu</t>
+        </is>
+      </c>
+      <c r="D49" s="33" t="inlineStr">
+        <is>
+          <t>tcu360.com</t>
+        </is>
+      </c>
+      <c r="E49" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F49" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G49" s="30" t="n">
+        <v>25690</v>
+      </c>
+      <c r="H49" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I49" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J49" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>

</xml_diff>

<commit_message>
Mark Colgate and Bucknellian running after their 200-tests passed.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -1618,7 +1618,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" s="0" t="n">
         <v>7337</v>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -2162,7 +2162,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G38" t="n">
+      <c r="G38" s="0" t="n">
         <v>7805</v>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -2303,10 +2303,12 @@
       </c>
       <c r="F41" s="0" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G41" s="0" t="n"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G41" s="0" t="n">
+        <v>200</v>
+      </c>
       <c r="H41" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -2317,7 +2319,7 @@
       </c>
       <c r="J41" s="0" t="inlineStr">
         <is>
-          <t>Wave 14 Liberal Arts SNO. ~15458 URLs, Cloudflare 10–14 s. Use wp-sitemap.xml. Fills a slot after Carleton. Probe + 200-test next.</t>
+          <t>newspaper-scraper@colgate; 200-test OK (200/200, no failures). systemd enabled 2026-10-07 16:27 UTC. Liberal Arts SNO, ~15489 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
         </is>
       </c>
     </row>
@@ -2349,10 +2351,12 @@
       </c>
       <c r="F42" s="0" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G42" s="0" t="n"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="n">
+        <v>200</v>
+      </c>
       <c r="H42" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -2363,7 +2367,7 @@
       </c>
       <c r="J42" s="0" t="inlineStr">
         <is>
-          <t>Wave 14 Liberal Arts SNO (Yoast). ~11585 URLs, Cloudflare 10–14 s. Fills a slot after Clemson. Probe + 200-test next.</t>
+          <t>newspaper-scraper@bucknellian; 200-test OK (200/200, no failures). systemd enabled 2026-10-07 16:27 UTC. Liberal Arts SNO Yoast, ~11583 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a scrape queue and auto-fill only papers that passed a 200-test.
Keep the VM at 12 by starting the next ready site_key from scrape_queue.csv
when a unit stops. Yale stays Mac-only; Duke other sections stay a later pass.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -1064,7 +1064,9 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G14" s="33" t="n"/>
+      <c r="G14" s="33" t="n">
+        <v>99943</v>
+      </c>
       <c r="H14" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1075,7 +1077,7 @@
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan; 78143 of 119764 (65.2%) as of 2026-10-06 14:31 UTC. http_429=15 (stable).</t>
+          <t>newspaper-scraper@michigan; 99943 of 119764 (83.4%) as of 2026-10-08 17:11 UTC. http_429=21 (was 16 on Oct 7). http_301=1821.</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1160,9 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G16" s="33" t="n"/>
+      <c r="G16" s="33" t="n">
+        <v>45147</v>
+      </c>
       <c r="H16" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1169,7 +1173,7 @@
       </c>
       <c r="J16" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@texan; 31397 of 51636 (60.8%) as of 2026-10-06 14:31 UTC.</t>
+          <t>newspaper-scraper@texan; 45147 of 51636 (87.4%) as of 2026-10-08 17:11 UTC. empty_body=407, http_403=7.</t>
         </is>
       </c>
     </row>
@@ -1201,10 +1205,12 @@
       </c>
       <c r="F17" s="33" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G17" s="33" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="n">
+        <v>37215</v>
+      </c>
       <c r="H17" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1215,7 +1221,7 @@
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@nexus; 28787 of 40465 (71.1%) as of 2026-10-06 14:31 UTC. empty_body=3838.</t>
+          <t>Finished 2026-10-07. 37215 of 40465 (92.0%); empty_body=4202, http_404=1. systemd inactive. File: ~/Downloads/nexus.csv</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1256,9 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G18" s="33" t="n"/>
+      <c r="G18" s="33" t="n">
+        <v>44450</v>
+      </c>
       <c r="H18" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1261,7 +1269,7 @@
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@illini; 31000 of 100022 (31.0%) as of 2026-10-06 14:31 UTC.</t>
+          <t>newspaper-scraper@illini; 44450 of 100022 (44.4%) as of 2026-10-08 17:11 UTC.</t>
         </is>
       </c>
     </row>
@@ -1293,10 +1301,12 @@
       </c>
       <c r="F19" s="33" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G19" s="33" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="n">
+        <v>40280</v>
+      </c>
       <c r="H19" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1307,7 +1317,7 @@
       </c>
       <c r="J19" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@technician; 32283 of 41051 (78.6%) as of 2026-10-06 14:31 UTC. empty_body=750.</t>
+          <t>Finished 2026-10-07. 40280 of 41051 (98.1%); empty_body=1017, http_521=1. systemd inactive. File: ~/Downloads/technician.csv</t>
         </is>
       </c>
     </row>
@@ -1390,6 +1400,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G21" s="0" t="n">
+        <v>36129</v>
+      </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1400,7 +1413,7 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tarheel; 23379 of 81683 (28.6%) as of 2026-10-06 14:31 UTC. empty_body=3581, http_403=19.</t>
+          <t>newspaper-scraper@tarheel; 36129 of 81683 (44.2%) as of 2026-10-08 17:11 UTC. empty_body=5194, http_403=28.</t>
         </is>
       </c>
     </row>
@@ -1483,6 +1496,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G23" s="0" t="n">
+        <v>24237</v>
+      </c>
       <c r="H23" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1493,7 +1509,7 @@
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@collegian; 10537 of 52185 (20.2%) as of 2026-10-06 14:31 UTC. empty_body=26, pre_2000=234.</t>
+          <t>newspaper-scraper@collegian; 24237 of 52185 (46.4%) as of 2026-10-08 17:11 UTC. empty_body=306, pre_2000=234.</t>
         </is>
       </c>
     </row>
@@ -1528,6 +1544,9 @@
           <t>running</t>
         </is>
       </c>
+      <c r="G24" s="0" t="n">
+        <v>21590</v>
+      </c>
       <c r="H24" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
@@ -1538,7 +1557,7 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@mndaily; 7240 of 80516 (9.0%) as of 2026-10-06 14:31 UTC. pre_2000=14440 skipped.</t>
+          <t>newspaper-scraper@mndaily; 21590 of 80516 (26.8%) as of 2026-10-08 17:11 UTC. pre_2000=14440 skipped.</t>
         </is>
       </c>
     </row>
@@ -2207,11 +2226,11 @@
       </c>
       <c r="F39" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G39" s="0" t="n">
-        <v>6141</v>
+        <v>9036</v>
       </c>
       <c r="H39" s="0" t="inlineStr">
         <is>
@@ -2223,7 +2242,7 @@
       </c>
       <c r="J39" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@macweekly; 6141 of 9420 (65.2%) as of 2026-10-07 14:02 UTC. empty_body=218.</t>
+          <t>Finished 2026-10-08. 9036 of 9420 (95.9%); empty_body=392, network_error=1. systemd inactive. File: ~/Downloads/macweekly.csv</t>
         </is>
       </c>
     </row>
@@ -2255,11 +2274,11 @@
       </c>
       <c r="F40" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G40" s="0" t="n">
-        <v>6190</v>
+        <v>9054</v>
       </c>
       <c r="H40" s="0" t="inlineStr">
         <is>
@@ -2271,7 +2290,7 @@
       </c>
       <c r="J40" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@sandb; 6190 of 9228 (67.1%) as of 2026-10-07 14:02 UTC. empty_body=80.</t>
+          <t>Finished 2026-10-08. 9054 of 9228 (98.1%); empty_body=184. systemd inactive. File: ~/Downloads/sandb.csv</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2326,7 @@
         </is>
       </c>
       <c r="G41" s="0" t="n">
-        <v>200</v>
+        <v>7250</v>
       </c>
       <c r="H41" s="0" t="inlineStr">
         <is>
@@ -2319,7 +2338,7 @@
       </c>
       <c r="J41" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@colgate; 200-test OK (200/200, no failures). systemd enabled 2026-10-07 16:27 UTC. Liberal Arts SNO, ~15489 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
+          <t>newspaper-scraper@colgate; 7250 of 15489 (46.8%) as of 2026-10-08 17:11 UTC. http_500=1.</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2374,7 @@
         </is>
       </c>
       <c r="G42" s="0" t="n">
-        <v>200</v>
+        <v>7300</v>
       </c>
       <c r="H42" s="0" t="inlineStr">
         <is>
@@ -2367,7 +2386,7 @@
       </c>
       <c r="J42" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@bucknellian; 200-test OK (200/200, no failures). systemd enabled 2026-10-07 16:27 UTC. Liberal Arts SNO Yoast, ~11583 URLs, Cloudflare 10–14 s. Resumes from 200-test CSV.</t>
+          <t>newspaper-scraper@bucknellian; 7300 of 11583 (63.0%) as of 2026-10-08 17:11 UTC. empty_body=11, http_404=2.</t>
         </is>
       </c>
     </row>
@@ -5497,6 +5516,11 @@
           <t>#50</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://bachelor.wabash.edu/</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
@@ -5507,6 +5531,11 @@
       <c r="B55" s="9" t="inlineStr">
         <is>
           <t>#50</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://wheatonwire.com/</t>
         </is>
       </c>
     </row>
@@ -6138,6 +6167,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add GW Hatchet, Stanford Daily, Marquette Wire, and NYU WSN as a ready buffer.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -970,280 +970,272 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
-        <is>
-          <t>Public Universities</t>
-        </is>
-      </c>
-      <c r="B12" s="32" t="n"/>
-      <c r="C12" s="32" t="n"/>
-      <c r="D12" s="32" t="n"/>
-      <c r="E12" s="32" t="n"/>
-      <c r="F12" s="32" t="n"/>
-      <c r="G12" s="32" t="n"/>
-      <c r="H12" s="32" t="n"/>
-      <c r="I12" s="32" t="n"/>
-      <c r="J12" s="32" t="n"/>
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>George Washington University</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>The Hatchet</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>hatchet</t>
+        </is>
+      </c>
+      <c r="D12" s="33" t="inlineStr">
+        <is>
+          <t>gwhatchet.com</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="n"/>
+      <c r="H12" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I12" s="36" t="n">
+        <v>46303</v>
+      </c>
+      <c r="J12" s="34" t="inlineStr">
+        <is>
+          <t>Wave 15 ready buffer. Cloudflare SNO ~60k URLs. Probe + 200-test next.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
-          <t>University of California, Irvine</t>
-        </is>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>New University</t>
+          <t>Stanford University</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>The Stanford Daily</t>
         </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>uci</t>
+          <t>stanford</t>
         </is>
       </c>
       <c r="D13" s="33" t="inlineStr">
         <is>
-          <t>newuniversity.org</t>
+          <t>stanforddaily.com</t>
         </is>
       </c>
       <c r="E13" s="33" t="inlineStr">
         <is>
-          <t>National Universities | Public Universities</t>
+          <t>National Universities</t>
         </is>
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G13" s="30" t="n">
-        <v>17411</v>
-      </c>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="n"/>
       <c r="H13" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I13" s="35" t="n">
-        <v>46293</v>
+      <c r="I13" s="36" t="n">
+        <v>46303</v>
       </c>
       <c r="J13" s="34" t="inlineStr">
         <is>
-          <t>Finished. 17411 articles of 17447 URLs (99.8%); 165 empty_body. systemd inactive. File: ~/Downloads/uci.csv</t>
+          <t>Wave 15 ready buffer. Cloudflare WP Yoast ~39k URLs. Probe + 200-test next.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>University of Michigan</t>
-        </is>
-      </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>The Michigan Daily</t>
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Marquette University</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Marquette Wire</t>
         </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>michigan</t>
+          <t>marquette</t>
         </is>
       </c>
       <c r="D14" s="33" t="inlineStr">
         <is>
-          <t>michigandaily.com</t>
+          <t>marquettewire.org</t>
         </is>
       </c>
       <c r="E14" s="33" t="inlineStr">
         <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F14" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G14" s="33" t="n">
-        <v>99943</v>
-      </c>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="n"/>
       <c r="H14" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I14" s="35" t="n">
-        <v>46293</v>
+      <c r="I14" s="36" t="n">
+        <v>46303</v>
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan; 99943 of 119764 (83.4%) as of 2026-10-08 17:11 UTC. http_429=21 (was 16 on Oct 7). http_301=1821.</t>
+          <t>Wave 15 ready buffer. Cloudflare SNO ~32k URLs. Probe + 200-test next.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="24" t="inlineStr">
         <is>
-          <t>University of California San Diego</t>
+          <t>New York University</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">
         <is>
-          <t>The UCSD Guardian</t>
+          <t>Washington Square News</t>
         </is>
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
-          <t>ucsd</t>
+          <t>nyu</t>
         </is>
       </c>
       <c r="D15" s="33" t="inlineStr">
         <is>
-          <t>ucsdguardian.org</t>
+          <t>nyunews.com</t>
         </is>
       </c>
       <c r="E15" s="33" t="inlineStr">
         <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="n"/>
+      <c r="H15" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I15" s="36" t="n">
+        <v>46303</v>
+      </c>
+      <c r="J15" s="34" t="inlineStr">
+        <is>
+          <t>Wave 15 ready buffer. Cloudflare SNO Yoast ~22k URLs. Probe + 200-test next.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="32" t="inlineStr">
+        <is>
+          <t>Public Universities</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="n"/>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="32" t="n"/>
+      <c r="F16" s="32" t="n"/>
+      <c r="G16" s="32" t="n"/>
+      <c r="H16" s="32" t="n"/>
+      <c r="I16" s="32" t="n"/>
+      <c r="J16" s="32" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>University of California, Irvine</t>
+        </is>
+      </c>
+      <c r="B17" s="33" t="inlineStr">
+        <is>
+          <t>New University</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>uci</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>newuniversity.org</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F15" s="24" t="inlineStr">
+      <c r="F17" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G15" s="33" t="n">
-        <v>21079</v>
-      </c>
-      <c r="H15" s="33" t="inlineStr">
+      <c r="G17" s="30" t="n">
+        <v>17411</v>
+      </c>
+      <c r="H17" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I15" s="36" t="n">
-        <v>46296</v>
-      </c>
-      <c r="J15" s="34" t="inlineStr">
-        <is>
-          <t>Finished 2026-10-05 before later downloads. 21079 articles of 22605 URLs (93.2%); 1660 empty_body, 2 http_500. systemd inactive. File: ~/Downloads/ucsd.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>University of Texas at Austin</t>
-        </is>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>The Daily Texan</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>texan</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>thedailytexan.com</t>
-        </is>
-      </c>
-      <c r="E16" s="33" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F16" s="33" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G16" s="33" t="n">
-        <v>45147</v>
-      </c>
-      <c r="H16" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I16" s="36" t="n">
-        <v>46296</v>
-      </c>
-      <c r="J16" s="34" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@texan; 45147 of 51636 (87.4%) as of 2026-10-08 17:11 UTC. empty_body=407, http_403=7.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>University of California, Santa Barbara</t>
-        </is>
-      </c>
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>Daily Nexus</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>nexus</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
-        <is>
-          <t>dailynexus.com</t>
-        </is>
-      </c>
-      <c r="E17" s="33" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F17" s="33" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G17" s="33" t="n">
-        <v>37215</v>
-      </c>
-      <c r="H17" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I17" s="36" t="n">
-        <v>46296</v>
+      <c r="I17" s="35" t="n">
+        <v>46293</v>
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-07. 37215 of 40465 (92.0%); empty_body=4202, http_404=1. systemd inactive. File: ~/Downloads/nexus.csv</t>
+          <t>Finished. 17411 articles of 17447 URLs (99.8%); 165 empty_body. systemd inactive. File: ~/Downloads/uci.csv</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="33" t="inlineStr">
         <is>
-          <t>University of Illinois Urbana-Champaign</t>
+          <t>University of Michigan</t>
         </is>
       </c>
       <c r="B18" s="33" t="inlineStr">
         <is>
-          <t>The Daily Illini</t>
+          <t>The Michigan Daily</t>
         </is>
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>illini</t>
+          <t>michigan</t>
         </is>
       </c>
       <c r="D18" s="33" t="inlineStr">
         <is>
-          <t>dailyillini.com</t>
+          <t>michigandaily.com</t>
         </is>
       </c>
       <c r="E18" s="33" t="inlineStr">
@@ -1257,41 +1249,41 @@
         </is>
       </c>
       <c r="G18" s="33" t="n">
-        <v>44450</v>
+        <v>99943</v>
       </c>
       <c r="H18" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I18" s="36" t="n">
-        <v>46296</v>
+      <c r="I18" s="35" t="n">
+        <v>46293</v>
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@illini; 44450 of 100022 (44.4%) as of 2026-10-08 17:11 UTC.</t>
+          <t>newspaper-scraper@michigan; 99943 of 119764 (83.4%) as of 2026-10-08 17:11 UTC. http_429=21 (was 16 on Oct 7). http_301=1821.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>North Carolina State University</t>
-        </is>
-      </c>
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>Technician</t>
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>University of California San Diego</t>
+        </is>
+      </c>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t>The UCSD Guardian</t>
         </is>
       </c>
       <c r="C19" s="33" t="inlineStr">
         <is>
-          <t>technician</t>
+          <t>ucsd</t>
         </is>
       </c>
       <c r="D19" s="33" t="inlineStr">
         <is>
-          <t>technicianonline.com</t>
+          <t>ucsdguardian.org</t>
         </is>
       </c>
       <c r="E19" s="33" t="inlineStr">
@@ -1299,13 +1291,13 @@
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F19" s="33" t="inlineStr">
+      <c r="F19" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
       <c r="G19" s="33" t="n">
-        <v>40280</v>
+        <v>21079</v>
       </c>
       <c r="H19" s="33" t="inlineStr">
         <is>
@@ -1317,29 +1309,29 @@
       </c>
       <c r="J19" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-07. 40280 of 41051 (98.1%); empty_body=1017, http_521=1. systemd inactive. File: ~/Downloads/technician.csv</t>
+          <t>Finished 2026-10-05 before later downloads. 21079 articles of 22605 URLs (93.2%); 1660 empty_body, 2 http_500. systemd inactive. File: ~/Downloads/ucsd.csv</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
-        <is>
-          <t>Stony Brook University</t>
-        </is>
-      </c>
-      <c r="B20" s="24" t="inlineStr">
-        <is>
-          <t>The Statesman</t>
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>University of Texas at Austin</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Texan</t>
         </is>
       </c>
       <c r="C20" s="33" t="inlineStr">
         <is>
-          <t>statesman</t>
+          <t>texan</t>
         </is>
       </c>
       <c r="D20" s="33" t="inlineStr">
         <is>
-          <t>sbstatesman.com</t>
+          <t>thedailytexan.com</t>
         </is>
       </c>
       <c r="E20" s="33" t="inlineStr">
@@ -1347,13 +1339,13 @@
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F20" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="F20" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
         </is>
       </c>
       <c r="G20" s="33" t="n">
-        <v>13354</v>
+        <v>45147</v>
       </c>
       <c r="H20" s="33" t="inlineStr">
         <is>
@@ -1365,570 +1357,570 @@
       </c>
       <c r="J20" s="34" t="inlineStr">
         <is>
+          <t>newspaper-scraper@texan; 45147 of 51636 (87.4%) as of 2026-10-08 17:11 UTC. empty_body=407, http_403=7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>University of California, Santa Barbara</t>
+        </is>
+      </c>
+      <c r="B21" s="33" t="inlineStr">
+        <is>
+          <t>Daily Nexus</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>nexus</t>
+        </is>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>dailynexus.com</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="n">
+        <v>37215</v>
+      </c>
+      <c r="H21" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I21" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J21" s="34" t="inlineStr">
+        <is>
+          <t>Finished 2026-10-07. 37215 of 40465 (92.0%); empty_body=4202, http_404=1. systemd inactive. File: ~/Downloads/nexus.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>University of Illinois Urbana-Champaign</t>
+        </is>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Illini</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>illini</t>
+        </is>
+      </c>
+      <c r="D22" s="33" t="inlineStr">
+        <is>
+          <t>dailyillini.com</t>
+        </is>
+      </c>
+      <c r="E22" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F22" s="33" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G22" s="33" t="n">
+        <v>44450</v>
+      </c>
+      <c r="H22" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I22" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J22" s="34" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@illini; 44450 of 100022 (44.4%) as of 2026-10-08 17:11 UTC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>North Carolina State University</t>
+        </is>
+      </c>
+      <c r="B23" s="33" t="inlineStr">
+        <is>
+          <t>Technician</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>technician</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="inlineStr">
+        <is>
+          <t>technicianonline.com</t>
+        </is>
+      </c>
+      <c r="E23" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F23" s="33" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="n">
+        <v>40280</v>
+      </c>
+      <c r="H23" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I23" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J23" s="34" t="inlineStr">
+        <is>
+          <t>Finished 2026-10-07. 40280 of 41051 (98.1%); empty_body=1017, http_521=1. systemd inactive. File: ~/Downloads/technician.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Stony Brook University</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>The Statesman</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>statesman</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="inlineStr">
+        <is>
+          <t>sbstatesman.com</t>
+        </is>
+      </c>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F24" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="n">
+        <v>13354</v>
+      </c>
+      <c r="H24" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I24" s="36" t="n">
+        <v>46296</v>
+      </c>
+      <c r="J24" s="34" t="inlineStr">
+        <is>
           <t>Finished 2026-10-04. 13354 of 13650 (97.8%); 517 empty_body, 32 pre_2000. File: ~/Downloads/statesman.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t>University of North Carolina, Chapel Hill</t>
-        </is>
-      </c>
-      <c r="B21" s="0" t="inlineStr">
-        <is>
-          <t>The Daily Tar Heel</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="inlineStr">
-        <is>
-          <t>tarheel</t>
-        </is>
-      </c>
-      <c r="D21" s="0" t="inlineStr">
-        <is>
-          <t>dailytarheel.com</t>
-        </is>
-      </c>
-      <c r="E21" s="0" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F21" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G21" s="0" t="n">
-        <v>36129</v>
-      </c>
-      <c r="H21" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I21" s="37" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J21" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@tarheel; 36129 of 81683 (44.2%) as of 2026-10-08 17:11 UTC. empty_body=5194, http_403=28.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="38" t="inlineStr">
-        <is>
-          <t>University of California, Riverside</t>
-        </is>
-      </c>
-      <c r="B22" s="38" t="inlineStr">
-        <is>
-          <t>The Highlander</t>
-        </is>
-      </c>
-      <c r="C22" s="0" t="inlineStr">
-        <is>
-          <t>highlander</t>
-        </is>
-      </c>
-      <c r="D22" s="0" t="inlineStr">
-        <is>
-          <t>highlandernews.org</t>
-        </is>
-      </c>
-      <c r="E22" s="0" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F22" s="38" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G22" s="0" t="n">
-        <v>9791</v>
-      </c>
-      <c r="H22" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I22" s="37" t="n">
-        <v>46297</v>
-      </c>
-      <c r="J22" s="0" t="inlineStr">
-        <is>
-          <t>Finished 2026-10-04. 9791 of 10144 (96.5%); 550 empty_body, 1 http_520, 1 http_525. File: ~/Downloads/highlander.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="0" t="inlineStr">
-        <is>
-          <t>University of Massachusetts, Amherst</t>
-        </is>
-      </c>
-      <c r="B23" s="0" t="inlineStr">
-        <is>
-          <t>The Massachusetts Daily Collegian</t>
-        </is>
-      </c>
-      <c r="C23" s="0" t="inlineStr">
-        <is>
-          <t>collegian</t>
-        </is>
-      </c>
-      <c r="D23" s="0" t="inlineStr">
-        <is>
-          <t>dailycollegian.com</t>
-        </is>
-      </c>
-      <c r="E23" s="0" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F23" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G23" s="0" t="n">
-        <v>24237</v>
-      </c>
-      <c r="H23" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I23" s="37" t="n">
-        <v>46299</v>
-      </c>
-      <c r="J23" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@collegian; 24237 of 52185 (46.4%) as of 2026-10-08 17:11 UTC. empty_body=306, pre_2000=234.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="0" t="inlineStr">
-        <is>
-          <t>University of Minnesota, Twin Cities</t>
-        </is>
-      </c>
-      <c r="B24" s="0" t="inlineStr">
-        <is>
-          <t>The Minnesota Daily</t>
-        </is>
-      </c>
-      <c r="C24" s="0" t="inlineStr">
-        <is>
-          <t>mndaily</t>
-        </is>
-      </c>
-      <c r="D24" s="0" t="inlineStr">
-        <is>
-          <t>mndaily.com</t>
-        </is>
-      </c>
-      <c r="E24" s="0" t="inlineStr">
-        <is>
-          <t>National Universities | Public Universities</t>
-        </is>
-      </c>
-      <c r="F24" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G24" s="0" t="n">
-        <v>21590</v>
-      </c>
-      <c r="H24" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I24" s="37" t="n">
-        <v>46299</v>
-      </c>
-      <c r="J24" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@mndaily; 21590 of 80516 (26.8%) as of 2026-10-08 17:11 UTC. pre_2000=14440 skipped.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
+          <t>University of North Carolina, Chapel Hill</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>The Daily Tar Heel</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>tarheel</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>dailytarheel.com</t>
+        </is>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F25" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G25" s="0" t="n">
+        <v>36129</v>
+      </c>
+      <c r="H25" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I25" s="37" t="n">
+        <v>46297</v>
+      </c>
+      <c r="J25" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@tarheel; 36129 of 81683 (44.2%) as of 2026-10-08 17:11 UTC. empty_body=5194, http_403=28.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>University of California, Riverside</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="inlineStr">
+        <is>
+          <t>The Highlander</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>highlander</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>highlandernews.org</t>
+        </is>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F26" s="38" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G26" s="0" t="n">
+        <v>9791</v>
+      </c>
+      <c r="H26" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I26" s="37" t="n">
+        <v>46297</v>
+      </c>
+      <c r="J26" s="0" t="inlineStr">
+        <is>
+          <t>Finished 2026-10-04. 9791 of 10144 (96.5%); 550 empty_body, 1 http_520, 1 http_525. File: ~/Downloads/highlander.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>University of Massachusetts, Amherst</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>The Massachusetts Daily Collegian</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>collegian</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>dailycollegian.com</t>
+        </is>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F27" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G27" s="0" t="n">
+        <v>24237</v>
+      </c>
+      <c r="H27" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I27" s="37" t="n">
+        <v>46299</v>
+      </c>
+      <c r="J27" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@collegian; 24237 of 52185 (46.4%) as of 2026-10-08 17:11 UTC. empty_body=306, pre_2000=234.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>University of Minnesota, Twin Cities</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>The Minnesota Daily</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>mndaily</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>mndaily.com</t>
+        </is>
+      </c>
+      <c r="E28" s="0" t="inlineStr">
+        <is>
+          <t>National Universities | Public Universities</t>
+        </is>
+      </c>
+      <c r="F28" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G28" s="0" t="n">
+        <v>21590</v>
+      </c>
+      <c r="H28" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I28" s="37" t="n">
+        <v>46299</v>
+      </c>
+      <c r="J28" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@mndaily; 21590 of 80516 (26.8%) as of 2026-10-08 17:11 UTC. pre_2000=14440 skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
           <t>University of Pittsburgh</t>
         </is>
       </c>
-      <c r="B25" s="0" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>The Pitt News</t>
         </is>
       </c>
-      <c r="C25" s="0" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>pitt</t>
         </is>
       </c>
-      <c r="D25" s="0" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>pittnews.com</t>
         </is>
       </c>
-      <c r="E25" s="0" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F25" s="0" t="inlineStr">
+      <c r="F29" s="0" t="inlineStr">
         <is>
           <t>queued</t>
         </is>
       </c>
-      <c r="H25" s="0" t="inlineStr">
+      <c r="H29" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I25" s="37" t="n">
+      <c r="I29" s="37" t="n">
         <v>46299</v>
       </c>
-      <c r="J25" s="0" t="inlineStr">
+      <c r="J29" s="0" t="inlineStr">
         <is>
           <t>Not cleared. VM 200-test HTTP 403 on /opinions/satire/; block cooldown. Probe of two news articles OK. Do not start full until a later 200-test passes.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="0" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>Clemson University</t>
         </is>
       </c>
-      <c r="B26" s="0" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>The Tiger</t>
         </is>
       </c>
-      <c r="C26" s="0" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>tiger</t>
         </is>
       </c>
-      <c r="D26" s="0" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>thetigercu.com</t>
         </is>
       </c>
-      <c r="E26" s="0" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F26" s="0" t="inlineStr">
+      <c r="F30" s="0" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G26" s="0" t="n">
+      <c r="G30" s="0" t="n">
         <v>7337</v>
       </c>
-      <c r="H26" s="0" t="inlineStr">
+      <c r="H30" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I26" s="37" t="n">
+      <c r="I30" s="37" t="n">
         <v>46300</v>
       </c>
-      <c r="J26" s="0" t="inlineStr">
+      <c r="J30" s="0" t="inlineStr">
         <is>
           <t>Finished 2026-10-06. 7337 of 7455 (98.4%); empty_body=130. systemd inactive. File: ~/Downloads/tiger.csv</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="38" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="38" t="inlineStr">
         <is>
           <t>New Jersey Institute of Technology</t>
         </is>
       </c>
-      <c r="B27" s="38" t="inlineStr">
+      <c r="B31" s="38" t="inlineStr">
         <is>
           <t>The Vector</t>
         </is>
       </c>
-      <c r="C27" s="0" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>vector</t>
         </is>
       </c>
-      <c r="D27" s="0" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>njitvector.com</t>
         </is>
       </c>
-      <c r="E27" s="0" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>National Universities | Public Universities</t>
         </is>
       </c>
-      <c r="F27" s="38" t="inlineStr">
+      <c r="F31" s="38" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G27" s="0" t="n">
+      <c r="G31" s="0" t="n">
         <v>335</v>
       </c>
-      <c r="H27" s="0" t="inlineStr">
+      <c r="H31" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I27" s="37" t="n">
+      <c r="I31" s="37" t="n">
         <v>46300</v>
       </c>
-      <c r="J27" s="0" t="inlineStr">
+      <c r="J31" s="0" t="inlineStr">
         <is>
           <t>Finished 2026-10-05. 335 of 336 (99.7%); 1 empty_body. File: ~/Downloads/vector.csv</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="32" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n"/>
-      <c r="C28" s="32" t="n"/>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="32" t="n"/>
-      <c r="G28" s="32" t="n"/>
-      <c r="H28" s="32" t="n"/>
-      <c r="I28" s="32" t="n"/>
-      <c r="J28" s="32" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="24" t="inlineStr">
-        <is>
-          <t>Connecticut College</t>
-        </is>
-      </c>
-      <c r="B29" s="33" t="inlineStr">
-        <is>
-          <t>The College Voice</t>
-        </is>
-      </c>
-      <c r="C29" s="33" t="inlineStr">
-        <is>
-          <t>conncoll</t>
-        </is>
-      </c>
-      <c r="D29" s="33" t="inlineStr">
-        <is>
-          <t>thecollegevoice.org</t>
-        </is>
-      </c>
-      <c r="E29" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F29" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G29" s="30" t="n">
-        <v>4039</v>
-      </c>
-      <c r="H29" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I29" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J29" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="24" t="inlineStr">
-        <is>
-          <t>Denison University</t>
-        </is>
-      </c>
-      <c r="B30" s="33" t="inlineStr">
-        <is>
-          <t>The Denisonian</t>
-        </is>
-      </c>
-      <c r="C30" s="33" t="inlineStr">
-        <is>
-          <t>denison</t>
-        </is>
-      </c>
-      <c r="D30" s="33" t="inlineStr">
-        <is>
-          <t>denisonian.com</t>
-        </is>
-      </c>
-      <c r="E30" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F30" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G30" s="30" t="n">
-        <v>3671</v>
-      </c>
-      <c r="H30" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I30" s="35" t="n">
-        <v>46294</v>
-      </c>
-      <c r="J30" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="24" t="inlineStr">
-        <is>
-          <t>Franklin &amp; Marshall College</t>
-        </is>
-      </c>
-      <c r="B31" s="33" t="inlineStr">
-        <is>
-          <t>The College Reporter</t>
-        </is>
-      </c>
-      <c r="C31" s="33" t="inlineStr">
-        <is>
-          <t>fandm</t>
-        </is>
-      </c>
-      <c r="D31" s="33" t="inlineStr">
-        <is>
-          <t>the-college-reporter.com</t>
-        </is>
-      </c>
-      <c r="E31" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F31" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G31" s="30" t="n">
-        <v>3449</v>
-      </c>
-      <c r="H31" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I31" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J31" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="24" t="inlineStr">
-        <is>
-          <t>Hillsdale College</t>
-        </is>
-      </c>
-      <c r="B32" s="33" t="inlineStr">
-        <is>
-          <t>The Collegian</t>
-        </is>
-      </c>
-      <c r="C32" s="33" t="inlineStr">
-        <is>
-          <t>hillsdale</t>
-        </is>
-      </c>
-      <c r="D32" s="33" t="inlineStr">
-        <is>
-          <t>hillsdalecollegian.com</t>
-        </is>
-      </c>
-      <c r="E32" s="33" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F32" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G32" s="30" t="n">
-        <v>15573</v>
-      </c>
-      <c r="H32" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I32" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J32" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
-        </is>
-      </c>
+      <c r="B32" s="32" t="n"/>
+      <c r="C32" s="32" t="n"/>
+      <c r="D32" s="32" t="n"/>
+      <c r="E32" s="32" t="n"/>
+      <c r="F32" s="32" t="n"/>
+      <c r="G32" s="32" t="n"/>
+      <c r="H32" s="32" t="n"/>
+      <c r="I32" s="32" t="n"/>
+      <c r="J32" s="32" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="24" t="inlineStr">
         <is>
-          <t>Occidental College</t>
+          <t>Connecticut College</t>
         </is>
       </c>
       <c r="B33" s="33" t="inlineStr">
         <is>
-          <t>The Occidental</t>
+          <t>The College Voice</t>
         </is>
       </c>
       <c r="C33" s="33" t="inlineStr">
         <is>
-          <t>occidental</t>
+          <t>conncoll</t>
         </is>
       </c>
       <c r="D33" s="33" t="inlineStr">
         <is>
-          <t>theoccidentalnews.com</t>
+          <t>thecollegevoice.org</t>
         </is>
       </c>
       <c r="E33" s="33" t="inlineStr">
@@ -1942,7 +1934,7 @@
         </is>
       </c>
       <c r="G33" s="30" t="n">
-        <v>9892</v>
+        <v>4039</v>
       </c>
       <c r="H33" s="33" t="inlineStr">
         <is>
@@ -1954,29 +1946,29 @@
       </c>
       <c r="J33" s="34" t="inlineStr">
         <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>Swarthmore College</t>
+          <t>Denison University</t>
         </is>
       </c>
       <c r="B34" s="33" t="inlineStr">
         <is>
-          <t>The Phoenix</t>
+          <t>The Denisonian</t>
         </is>
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
-          <t>swarthmore</t>
+          <t>denison</t>
         </is>
       </c>
       <c r="D34" s="33" t="inlineStr">
         <is>
-          <t>swarthmorephoenix.com</t>
+          <t>denisonian.com</t>
         </is>
       </c>
       <c r="E34" s="33" t="inlineStr">
@@ -1990,7 +1982,7 @@
         </is>
       </c>
       <c r="G34" s="30" t="n">
-        <v>12798</v>
+        <v>3671</v>
       </c>
       <c r="H34" s="33" t="inlineStr">
         <is>
@@ -1998,33 +1990,33 @@
         </is>
       </c>
       <c r="I34" s="35" t="n">
-        <v>46292</v>
+        <v>46294</v>
       </c>
       <c r="J34" s="34" t="inlineStr">
         <is>
-          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>Union College (NY)</t>
+          <t>Franklin &amp; Marshall College</t>
         </is>
       </c>
       <c r="B35" s="33" t="inlineStr">
         <is>
-          <t>Concordiensis</t>
+          <t>The College Reporter</t>
         </is>
       </c>
       <c r="C35" s="33" t="inlineStr">
         <is>
-          <t>union</t>
+          <t>fandm</t>
         </is>
       </c>
       <c r="D35" s="33" t="inlineStr">
         <is>
-          <t>concordiensis.com</t>
+          <t>the-college-reporter.com</t>
         </is>
       </c>
       <c r="E35" s="33" t="inlineStr">
@@ -2038,7 +2030,7 @@
         </is>
       </c>
       <c r="G35" s="30" t="n">
-        <v>1604</v>
+        <v>3449</v>
       </c>
       <c r="H35" s="33" t="inlineStr">
         <is>
@@ -2050,29 +2042,29 @@
       </c>
       <c r="J35" s="34" t="inlineStr">
         <is>
-          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>Wesleyan University</t>
+          <t>Hillsdale College</t>
         </is>
       </c>
       <c r="B36" s="33" t="inlineStr">
         <is>
-          <t>The Wesleyan Argus</t>
+          <t>The Collegian</t>
         </is>
       </c>
       <c r="C36" s="33" t="inlineStr">
         <is>
-          <t>wesleyan</t>
+          <t>hillsdale</t>
         </is>
       </c>
       <c r="D36" s="33" t="inlineStr">
         <is>
-          <t>wesleyanargus.com</t>
+          <t>hillsdalecollegian.com</t>
         </is>
       </c>
       <c r="E36" s="33" t="inlineStr">
@@ -2085,8 +2077,8 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G36" s="24" t="n">
-        <v>21881</v>
+      <c r="G36" s="30" t="n">
+        <v>15573</v>
       </c>
       <c r="H36" s="33" t="inlineStr">
         <is>
@@ -2094,534 +2086,534 @@
         </is>
       </c>
       <c r="I36" s="35" t="n">
-        <v>46294</v>
+        <v>46292</v>
       </c>
       <c r="J36" s="34" t="inlineStr">
         <is>
-          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="24" t="inlineStr">
         <is>
+          <t>Occidental College</t>
+        </is>
+      </c>
+      <c r="B37" s="33" t="inlineStr">
+        <is>
+          <t>The Occidental</t>
+        </is>
+      </c>
+      <c r="C37" s="33" t="inlineStr">
+        <is>
+          <t>occidental</t>
+        </is>
+      </c>
+      <c r="D37" s="33" t="inlineStr">
+        <is>
+          <t>theoccidentalnews.com</t>
+        </is>
+      </c>
+      <c r="E37" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F37" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G37" s="30" t="n">
+        <v>9892</v>
+      </c>
+      <c r="H37" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I37" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J37" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="24" t="inlineStr">
+        <is>
+          <t>Swarthmore College</t>
+        </is>
+      </c>
+      <c r="B38" s="33" t="inlineStr">
+        <is>
+          <t>The Phoenix</t>
+        </is>
+      </c>
+      <c r="C38" s="33" t="inlineStr">
+        <is>
+          <t>swarthmore</t>
+        </is>
+      </c>
+      <c r="D38" s="33" t="inlineStr">
+        <is>
+          <t>swarthmorephoenix.com</t>
+        </is>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F38" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G38" s="30" t="n">
+        <v>12798</v>
+      </c>
+      <c r="H38" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I38" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J38" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>Union College (NY)</t>
+        </is>
+      </c>
+      <c r="B39" s="33" t="inlineStr">
+        <is>
+          <t>Concordiensis</t>
+        </is>
+      </c>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>union</t>
+        </is>
+      </c>
+      <c r="D39" s="33" t="inlineStr">
+        <is>
+          <t>concordiensis.com</t>
+        </is>
+      </c>
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G39" s="30" t="n">
+        <v>1604</v>
+      </c>
+      <c r="H39" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I39" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J39" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>Wesleyan University</t>
+        </is>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>The Wesleyan Argus</t>
+        </is>
+      </c>
+      <c r="C40" s="33" t="inlineStr">
+        <is>
+          <t>wesleyan</t>
+        </is>
+      </c>
+      <c r="D40" s="33" t="inlineStr">
+        <is>
+          <t>wesleyanargus.com</t>
+        </is>
+      </c>
+      <c r="E40" s="33" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F40" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G40" s="24" t="n">
+        <v>21881</v>
+      </c>
+      <c r="H40" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I40" s="35" t="n">
+        <v>46294</v>
+      </c>
+      <c r="J40" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
           <t>Claremont Colleges</t>
         </is>
       </c>
-      <c r="B37" s="24" t="inlineStr">
+      <c r="B41" s="24" t="inlineStr">
         <is>
           <t>The Student Life</t>
         </is>
       </c>
-      <c r="C37" s="33" t="inlineStr">
+      <c r="C41" s="33" t="inlineStr">
         <is>
           <t>tsl</t>
         </is>
       </c>
-      <c r="D37" s="33" t="inlineStr">
+      <c r="D41" s="33" t="inlineStr">
         <is>
           <t>tsl.news</t>
         </is>
       </c>
-      <c r="E37" s="33" t="inlineStr">
+      <c r="E41" s="33" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F37" s="24" t="inlineStr">
+      <c r="F41" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G37" s="33" t="n">
+      <c r="G41" s="33" t="n">
         <v>11405</v>
       </c>
-      <c r="H37" s="33" t="inlineStr">
+      <c r="H41" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I37" s="35" t="n">
+      <c r="I41" s="35" t="n">
         <v>46295</v>
       </c>
-      <c r="J37" s="34" t="inlineStr">
+      <c r="J41" s="34" t="inlineStr">
         <is>
           <t>Finished 2026-10-04. 11405 of 11437 (99.7%); 16 empty_body, 15 http_403, 1 http_404. File: ~/Downloads/tsl.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="0" t="inlineStr">
-        <is>
-          <t>Carleton College</t>
-        </is>
-      </c>
-      <c r="B38" s="0" t="inlineStr">
-        <is>
-          <t>The Carletonian</t>
-        </is>
-      </c>
-      <c r="C38" s="0" t="inlineStr">
-        <is>
-          <t>carleton</t>
-        </is>
-      </c>
-      <c r="D38" s="0" t="inlineStr">
-        <is>
-          <t>thecarletonian.com</t>
-        </is>
-      </c>
-      <c r="E38" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F38" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G38" s="0" t="n">
-        <v>7805</v>
-      </c>
-      <c r="H38" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I38" s="37" t="n">
-        <v>46300</v>
-      </c>
-      <c r="J38" s="0" t="inlineStr">
-        <is>
-          <t>Finished 2026-10-06. 7805 of 7941 (98.3%); empty_body=135, http_404=1. systemd inactive. File: ~/Downloads/carleton.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="0" t="inlineStr">
-        <is>
-          <t>Macalester College</t>
-        </is>
-      </c>
-      <c r="B39" s="0" t="inlineStr">
-        <is>
-          <t>The Mac Weekly</t>
-        </is>
-      </c>
-      <c r="C39" s="0" t="inlineStr">
-        <is>
-          <t>macweekly</t>
-        </is>
-      </c>
-      <c r="D39" s="0" t="inlineStr">
-        <is>
-          <t>themacweekly.com</t>
-        </is>
-      </c>
-      <c r="E39" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F39" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G39" s="0" t="n">
-        <v>9036</v>
-      </c>
-      <c r="H39" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I39" s="37" t="n">
-        <v>46301</v>
-      </c>
-      <c r="J39" s="0" t="inlineStr">
-        <is>
-          <t>Finished 2026-10-08. 9036 of 9420 (95.9%); empty_body=392, network_error=1. systemd inactive. File: ~/Downloads/macweekly.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="0" t="inlineStr">
-        <is>
-          <t>Grinnell College</t>
-        </is>
-      </c>
-      <c r="B40" s="0" t="inlineStr">
-        <is>
-          <t>Scarlet &amp; Black</t>
-        </is>
-      </c>
-      <c r="C40" s="0" t="inlineStr">
-        <is>
-          <t>sandb</t>
-        </is>
-      </c>
-      <c r="D40" s="0" t="inlineStr">
-        <is>
-          <t>thesandb.com</t>
-        </is>
-      </c>
-      <c r="E40" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F40" s="0" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G40" s="0" t="n">
-        <v>9054</v>
-      </c>
-      <c r="H40" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I40" s="37" t="n">
-        <v>46301</v>
-      </c>
-      <c r="J40" s="0" t="inlineStr">
-        <is>
-          <t>Finished 2026-10-08. 9054 of 9228 (98.1%); empty_body=184. systemd inactive. File: ~/Downloads/sandb.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="0" t="inlineStr">
-        <is>
-          <t>Colgate University</t>
-        </is>
-      </c>
-      <c r="B41" s="0" t="inlineStr">
-        <is>
-          <t>The Colgate Maroon-News</t>
-        </is>
-      </c>
-      <c r="C41" s="0" t="inlineStr">
-        <is>
-          <t>colgate</t>
-        </is>
-      </c>
-      <c r="D41" s="0" t="inlineStr">
-        <is>
-          <t>thecolgatemaroonnews.com</t>
-        </is>
-      </c>
-      <c r="E41" s="0" t="inlineStr">
-        <is>
-          <t>Liberal Arts</t>
-        </is>
-      </c>
-      <c r="F41" s="0" t="inlineStr">
-        <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G41" s="0" t="n">
-        <v>7250</v>
-      </c>
-      <c r="H41" s="0" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I41" s="37" t="n">
-        <v>46302</v>
-      </c>
-      <c r="J41" s="0" t="inlineStr">
-        <is>
-          <t>newspaper-scraper@colgate; 7250 of 15489 (46.8%) as of 2026-10-08 17:11 UTC. http_500=1.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
+          <t>Carleton College</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>The Carletonian</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>carleton</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>thecarletonian.com</t>
+        </is>
+      </c>
+      <c r="E42" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F42" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G42" s="0" t="n">
+        <v>7805</v>
+      </c>
+      <c r="H42" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I42" s="37" t="n">
+        <v>46300</v>
+      </c>
+      <c r="J42" s="0" t="inlineStr">
+        <is>
+          <t>Finished 2026-10-06. 7805 of 7941 (98.3%); empty_body=135, http_404=1. systemd inactive. File: ~/Downloads/carleton.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>Macalester College</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>The Mac Weekly</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>macweekly</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>themacweekly.com</t>
+        </is>
+      </c>
+      <c r="E43" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F43" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G43" s="0" t="n">
+        <v>9036</v>
+      </c>
+      <c r="H43" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I43" s="37" t="n">
+        <v>46301</v>
+      </c>
+      <c r="J43" s="0" t="inlineStr">
+        <is>
+          <t>Finished 2026-10-08. 9036 of 9420 (95.9%); empty_body=392, network_error=1. systemd inactive. File: ~/Downloads/macweekly.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>Grinnell College</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>Scarlet &amp; Black</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>sandb</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>thesandb.com</t>
+        </is>
+      </c>
+      <c r="E44" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F44" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G44" s="0" t="n">
+        <v>9054</v>
+      </c>
+      <c r="H44" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I44" s="37" t="n">
+        <v>46301</v>
+      </c>
+      <c r="J44" s="0" t="inlineStr">
+        <is>
+          <t>Finished 2026-10-08. 9054 of 9228 (98.1%); empty_body=184. systemd inactive. File: ~/Downloads/sandb.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>Colgate University</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>The Colgate Maroon-News</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>colgate</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>thecolgatemaroonnews.com</t>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F45" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G45" s="0" t="n">
+        <v>7250</v>
+      </c>
+      <c r="H45" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I45" s="37" t="n">
+        <v>46302</v>
+      </c>
+      <c r="J45" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@colgate; 7250 of 15489 (46.8%) as of 2026-10-08 17:11 UTC. http_500=1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
           <t>Bucknell University</t>
         </is>
       </c>
-      <c r="B42" s="0" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>The Bucknellian</t>
         </is>
       </c>
-      <c r="C42" s="0" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>bucknellian</t>
         </is>
       </c>
-      <c r="D42" s="0" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>bucknellian.net</t>
         </is>
       </c>
-      <c r="E42" s="0" t="inlineStr">
+      <c r="E46" s="0" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F42" s="0" t="inlineStr">
+      <c r="F46" s="0" t="inlineStr">
         <is>
           <t>running</t>
         </is>
       </c>
-      <c r="G42" s="0" t="n">
+      <c r="G46" s="0" t="n">
         <v>7300</v>
       </c>
-      <c r="H42" s="0" t="inlineStr">
+      <c r="H46" s="0" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I42" s="37" t="n">
+      <c r="I46" s="37" t="n">
         <v>46302</v>
       </c>
-      <c r="J42" s="0" t="inlineStr">
+      <c r="J46" s="0" t="inlineStr">
         <is>
           <t>newspaper-scraper@bucknellian; 7300 of 11583 (63.0%) as of 2026-10-08 17:11 UTC. empty_body=11, http_404=2.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="32" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="32" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="B43" s="32" t="n"/>
-      <c r="C43" s="32" t="n"/>
-      <c r="D43" s="32" t="n"/>
-      <c r="E43" s="32" t="n"/>
-      <c r="F43" s="32" t="n"/>
-      <c r="G43" s="32" t="n"/>
-      <c r="H43" s="32" t="n"/>
-      <c r="I43" s="32" t="n"/>
-      <c r="J43" s="32" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="24" t="inlineStr">
-        <is>
-          <t>Biola University</t>
-        </is>
-      </c>
-      <c r="B44" s="33" t="inlineStr">
-        <is>
-          <t>The Chimes</t>
-        </is>
-      </c>
-      <c r="C44" s="33" t="inlineStr">
-        <is>
-          <t>biola</t>
-        </is>
-      </c>
-      <c r="D44" s="33" t="inlineStr">
-        <is>
-          <t>chimesnewspaper.com</t>
-        </is>
-      </c>
-      <c r="E44" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F44" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G44" s="30" t="n">
-        <v>11331</v>
-      </c>
-      <c r="H44" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I44" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J44" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="24" t="inlineStr">
-        <is>
-          <t>Lipscomb University</t>
-        </is>
-      </c>
-      <c r="B45" s="33" t="inlineStr">
-        <is>
-          <t>Lipscomb Media</t>
-        </is>
-      </c>
-      <c r="C45" s="33" t="inlineStr">
-        <is>
-          <t>lipscomb</t>
-        </is>
-      </c>
-      <c r="D45" s="33" t="inlineStr">
-        <is>
-          <t>lipscombmedia.com</t>
-        </is>
-      </c>
-      <c r="E45" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F45" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G45" s="30" t="n">
-        <v>682</v>
-      </c>
-      <c r="H45" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I45" s="35" t="n">
-        <v>46292</v>
-      </c>
-      <c r="J45" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="24" t="inlineStr">
-        <is>
-          <t>Point Loma Nazarene University</t>
-        </is>
-      </c>
-      <c r="B46" s="33" t="inlineStr">
-        <is>
-          <t>Loma Beat</t>
-        </is>
-      </c>
-      <c r="C46" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat</t>
-        </is>
-      </c>
-      <c r="D46" s="33" t="inlineStr">
-        <is>
-          <t>lomabeat.com</t>
-        </is>
-      </c>
-      <c r="E46" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges</t>
-        </is>
-      </c>
-      <c r="F46" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G46" s="30" t="n">
-        <v>3950</v>
-      </c>
-      <c r="H46" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I46" s="35" t="n">
-        <v>46293</v>
-      </c>
-      <c r="J46" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="24" t="inlineStr">
-        <is>
-          <t>Southern Methodist University</t>
-        </is>
-      </c>
-      <c r="B47" s="33" t="inlineStr">
-        <is>
-          <t>The Daily Campus</t>
-        </is>
-      </c>
-      <c r="C47" s="33" t="inlineStr">
-        <is>
-          <t>smu</t>
-        </is>
-      </c>
-      <c r="D47" s="33" t="inlineStr">
-        <is>
-          <t>smudailycampus.com</t>
-        </is>
-      </c>
-      <c r="E47" s="33" t="inlineStr">
-        <is>
-          <t>Christian Colleges | National Universities</t>
-        </is>
-      </c>
-      <c r="F47" s="24" t="inlineStr">
-        <is>
-          <t>done</t>
-        </is>
-      </c>
-      <c r="G47" s="30" t="n">
-        <v>26208</v>
-      </c>
-      <c r="H47" s="33" t="inlineStr">
-        <is>
-          <t>AWS VM</t>
-        </is>
-      </c>
-      <c r="I47" s="35" t="n">
-        <v>46291</v>
-      </c>
-      <c r="J47" s="34" t="inlineStr">
-        <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
-        </is>
-      </c>
+      <c r="B47" s="32" t="n"/>
+      <c r="C47" s="32" t="n"/>
+      <c r="D47" s="32" t="n"/>
+      <c r="E47" s="32" t="n"/>
+      <c r="F47" s="32" t="n"/>
+      <c r="G47" s="32" t="n"/>
+      <c r="H47" s="32" t="n"/>
+      <c r="I47" s="32" t="n"/>
+      <c r="J47" s="32" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="24" t="inlineStr">
         <is>
-          <t>St. Olaf College</t>
+          <t>Biola University</t>
         </is>
       </c>
       <c r="B48" s="33" t="inlineStr">
         <is>
-          <t>Manitou Messenger</t>
+          <t>The Chimes</t>
         </is>
       </c>
       <c r="C48" s="33" t="inlineStr">
         <is>
-          <t>stolaf</t>
+          <t>biola</t>
         </is>
       </c>
       <c r="D48" s="33" t="inlineStr">
         <is>
-          <t>olafmessenger.com</t>
+          <t>chimesnewspaper.com</t>
         </is>
       </c>
       <c r="E48" s="33" t="inlineStr">
         <is>
-          <t>Christian Colleges | Liberal Arts</t>
+          <t>Christian Colleges</t>
         </is>
       </c>
       <c r="F48" s="24" t="inlineStr">
@@ -2630,7 +2622,7 @@
         </is>
       </c>
       <c r="G48" s="30" t="n">
-        <v>5048</v>
+        <v>11331</v>
       </c>
       <c r="H48" s="33" t="inlineStr">
         <is>
@@ -2638,57 +2630,249 @@
         </is>
       </c>
       <c r="I48" s="35" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="J48" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="24" t="inlineStr">
         <is>
+          <t>Lipscomb University</t>
+        </is>
+      </c>
+      <c r="B49" s="33" t="inlineStr">
+        <is>
+          <t>Lipscomb Media</t>
+        </is>
+      </c>
+      <c r="C49" s="33" t="inlineStr">
+        <is>
+          <t>lipscomb</t>
+        </is>
+      </c>
+      <c r="D49" s="33" t="inlineStr">
+        <is>
+          <t>lipscombmedia.com</t>
+        </is>
+      </c>
+      <c r="E49" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F49" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G49" s="30" t="n">
+        <v>682</v>
+      </c>
+      <c r="H49" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I49" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J49" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="24" t="inlineStr">
+        <is>
+          <t>Point Loma Nazarene University</t>
+        </is>
+      </c>
+      <c r="B50" s="33" t="inlineStr">
+        <is>
+          <t>Loma Beat</t>
+        </is>
+      </c>
+      <c r="C50" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat</t>
+        </is>
+      </c>
+      <c r="D50" s="33" t="inlineStr">
+        <is>
+          <t>lomabeat.com</t>
+        </is>
+      </c>
+      <c r="E50" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F50" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G50" s="30" t="n">
+        <v>3950</v>
+      </c>
+      <c r="H50" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I50" s="35" t="n">
+        <v>46293</v>
+      </c>
+      <c r="J50" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="24" t="inlineStr">
+        <is>
+          <t>Southern Methodist University</t>
+        </is>
+      </c>
+      <c r="B51" s="33" t="inlineStr">
+        <is>
+          <t>The Daily Campus</t>
+        </is>
+      </c>
+      <c r="C51" s="33" t="inlineStr">
+        <is>
+          <t>smu</t>
+        </is>
+      </c>
+      <c r="D51" s="33" t="inlineStr">
+        <is>
+          <t>smudailycampus.com</t>
+        </is>
+      </c>
+      <c r="E51" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | National Universities</t>
+        </is>
+      </c>
+      <c r="F51" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G51" s="30" t="n">
+        <v>26208</v>
+      </c>
+      <c r="H51" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I51" s="35" t="n">
+        <v>46291</v>
+      </c>
+      <c r="J51" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="24" t="inlineStr">
+        <is>
+          <t>St. Olaf College</t>
+        </is>
+      </c>
+      <c r="B52" s="33" t="inlineStr">
+        <is>
+          <t>Manitou Messenger</t>
+        </is>
+      </c>
+      <c r="C52" s="33" t="inlineStr">
+        <is>
+          <t>stolaf</t>
+        </is>
+      </c>
+      <c r="D52" s="33" t="inlineStr">
+        <is>
+          <t>olafmessenger.com</t>
+        </is>
+      </c>
+      <c r="E52" s="33" t="inlineStr">
+        <is>
+          <t>Christian Colleges | Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F52" s="24" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G52" s="30" t="n">
+        <v>5048</v>
+      </c>
+      <c r="H52" s="33" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I52" s="35" t="n">
+        <v>46292</v>
+      </c>
+      <c r="J52" s="34" t="inlineStr">
+        <is>
+          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="inlineStr">
+        <is>
           <t>Texas Christian University</t>
         </is>
       </c>
-      <c r="B49" s="33" t="inlineStr">
+      <c r="B53" s="33" t="inlineStr">
         <is>
           <t>TCU 360</t>
         </is>
       </c>
-      <c r="C49" s="33" t="inlineStr">
+      <c r="C53" s="33" t="inlineStr">
         <is>
           <t>tcu</t>
         </is>
       </c>
-      <c r="D49" s="33" t="inlineStr">
+      <c r="D53" s="33" t="inlineStr">
         <is>
           <t>tcu360.com</t>
         </is>
       </c>
-      <c r="E49" s="33" t="inlineStr">
+      <c r="E53" s="33" t="inlineStr">
         <is>
           <t>Christian Colleges | National Universities</t>
         </is>
       </c>
-      <c r="F49" s="24" t="inlineStr">
+      <c r="F53" s="24" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="G49" s="30" t="n">
+      <c r="G53" s="30" t="n">
         <v>25690</v>
       </c>
-      <c r="H49" s="33" t="inlineStr">
+      <c r="H53" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I49" s="35" t="n">
+      <c r="I53" s="35" t="n">
         <v>46291</v>
       </c>
-      <c r="J49" s="34" t="inlineStr">
+      <c r="J53" s="34" t="inlineStr">
         <is>
           <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
         </is>
@@ -5516,7 +5700,7 @@
           <t>#50</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="0" t="inlineStr">
         <is>
           <t>https://bachelor.wabash.edu/</t>
         </is>
@@ -5533,7 +5717,7 @@
           <t>#50</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="0" t="inlineStr">
         <is>
           <t>https://wheatonwire.com/</t>
         </is>

</xml_diff>

<commit_message>
Raise CAP to 20, stage wave 21, and resolve blank ranking URLs.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -180,6 +180,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -579,11 +582,11 @@
         </is>
       </c>
       <c r="I3" s="35" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="J3" s="34" t="inlineStr">
         <is>
-          <t>Finished. 2137 articles of 2140 URLs (99.9%); 5 empty_body. systemd inactive. File: repo output/rit.csv</t>
+          <t>Finished as of 2026-10-13. 2137 articles. systemd inactive. File: ~/Downloads/rit.csv</t>
         </is>
       </c>
     </row>
@@ -627,11 +630,11 @@
         </is>
       </c>
       <c r="I4" s="35" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="J4" s="34" t="inlineStr">
         <is>
-          <t>Finished. 6899 articles of 6992 URLs (98.7%); 67 empty_body, 26 pre_2000. systemd inactive. File: ~/Downloads/ucsc.csv</t>
+          <t>Finished as of 2026-10-13. 6899 articles. systemd inactive. File: ~/Downloads/ucsc.csv</t>
         </is>
       </c>
     </row>
@@ -675,11 +678,11 @@
         </is>
       </c>
       <c r="I5" s="35" t="n">
-        <v>46291</v>
+        <v>46308</v>
       </c>
       <c r="J5" s="34" t="inlineStr">
         <is>
-          <t>Finished. 22117 articles of 22493 URLs (98.3%); 371 empty_body, 2 http_301, 3 http_404. systemd inactive. File: repo output/chicago.csv</t>
+          <t>Finished as of 2026-10-13. 22117 articles. systemd inactive. File: ~/Downloads/chicago.csv</t>
         </is>
       </c>
     </row>
@@ -723,11 +726,11 @@
         </is>
       </c>
       <c r="I6" s="35" t="n">
-        <v>46294</v>
+        <v>46308</v>
       </c>
       <c r="J6" s="34" t="inlineStr">
         <is>
-          <t>Finished. 4175 articles of 4678 URLs (89.2%); 41 empty_body, 464 pre_2000. systemd inactive. File: ~/Downloads/yu.csv</t>
+          <t>Finished as of 2026-10-13. 4175 articles. systemd inactive. File: ~/Downloads/yu.csv</t>
         </is>
       </c>
     </row>
@@ -762,7 +765,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G7" s="33" t="n">
+      <c r="G7" s="39" t="n">
         <v>69041</v>
       </c>
       <c r="H7" s="33" t="inlineStr">
@@ -771,11 +774,11 @@
         </is>
       </c>
       <c r="I7" s="35" t="n">
-        <v>46290</v>
+        <v>46308</v>
       </c>
       <c r="J7" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-06. 69041 articles of 70720 URLs (97.6%); empty_body=3558, http_301=11, http_403=32, network_error=1083, pre_2000=46. systemd inactive. File: ~/Downloads/northwestern.csv</t>
+          <t>Finished as of 2026-10-13. 69041 articles. systemd inactive. File: ~/Downloads/northwestern.csv</t>
         </is>
       </c>
     </row>
@@ -810,8 +813,8 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G8" s="33" t="n">
-        <v>25622</v>
+      <c r="G8" s="39" t="n">
+        <v>25632</v>
       </c>
       <c r="H8" s="33" t="inlineStr">
         <is>
@@ -819,11 +822,11 @@
         </is>
       </c>
       <c r="I8" s="35" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="J8" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-02. 25622 articles of 25641 URLs (99.9%); 8 empty_body, 2 http_403, 9 http_500, 5 network_error. systemd inactive. File: ~/Downloads/miami.csv</t>
+          <t>Finished as of 2026-10-13. 25632 articles. systemd inactive. File: ~/Downloads/miami.csv</t>
         </is>
       </c>
     </row>
@@ -858,7 +861,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G9" s="33" t="n">
+      <c r="G9" s="39" t="n">
         <v>31894</v>
       </c>
       <c r="H9" s="33" t="inlineStr">
@@ -867,11 +870,11 @@
         </is>
       </c>
       <c r="I9" s="35" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="J9" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-01. 31894 articles of 32243 URLs (98.9%); 501 empty_body, 2 network_error, 9 pre_2000. systemd inactive. File: ~/Downloads/usf.csv</t>
+          <t>Finished as of 2026-10-13. 31894 articles. systemd inactive. File: ~/Downloads/usf.csv</t>
         </is>
       </c>
     </row>
@@ -952,7 +955,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G11" s="33" t="n">
+      <c r="G11" s="39" t="n">
         <v>22155</v>
       </c>
       <c r="H11" s="33" t="inlineStr">
@@ -960,12 +963,12 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I11" s="36" t="n">
-        <v>46296</v>
+      <c r="I11" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J11" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-05. News-section listings only, 22155 articles; 217 empty_body, 3 pre_2000. Other Chronicle sections later. File: ~/Downloads/duke.csv</t>
+          <t>Finished as of 2026-10-13. 22155 articles. systemd inactive. File: ~/Downloads/duke.csv</t>
         </is>
       </c>
     </row>
@@ -997,21 +1000,23 @@
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G12" s="33" t="n"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G12" s="39" t="n">
+        <v>30994</v>
+      </c>
       <c r="H12" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I12" s="36" t="n">
-        <v>46303</v>
+      <c r="I12" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J12" s="34" t="inlineStr">
         <is>
-          <t>Wave 15 ready buffer. Cloudflare SNO ~60k URLs. Probe + 200-test next.</t>
+          <t>newspaper-scraper@hatchet; 30994 articles as of 2026-10-13. systemd active on AWS VM.</t>
         </is>
       </c>
     </row>
@@ -1043,21 +1048,23 @@
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G13" s="33" t="n"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>30550</v>
+      </c>
       <c r="H13" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I13" s="36" t="n">
-        <v>46303</v>
+      <c r="I13" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J13" s="34" t="inlineStr">
         <is>
-          <t>Wave 15 ready buffer. Cloudflare WP Yoast ~39k URLs. Probe + 200-test next.</t>
+          <t>newspaper-scraper@stanford; 30550 articles as of 2026-10-13. systemd active on AWS VM.</t>
         </is>
       </c>
     </row>
@@ -1089,21 +1096,23 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G14" s="33" t="n"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G14" s="39" t="n">
+        <v>30250</v>
+      </c>
       <c r="H14" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I14" s="36" t="n">
-        <v>46303</v>
+      <c r="I14" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>Wave 15 ready buffer. Cloudflare SNO ~32k URLs. Probe + 200-test next.</t>
+          <t>newspaper-scraper@marquette; 30250 articles as of 2026-10-13. systemd active on AWS VM.</t>
         </is>
       </c>
     </row>
@@ -1135,21 +1144,23 @@
       </c>
       <c r="F15" s="24" t="inlineStr">
         <is>
-          <t>queued</t>
-        </is>
-      </c>
-      <c r="G15" s="33" t="n"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G15" s="39" t="n">
+        <v>21935</v>
+      </c>
       <c r="H15" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I15" s="36" t="n">
-        <v>46303</v>
+      <c r="I15" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>Wave 15 ready buffer. Cloudflare SNO Yoast ~22k URLs. Probe + 200-test next.</t>
+          <t>Finished as of 2026-10-13. 21935 articles. systemd inactive. File: ~/Downloads/nyu.csv</t>
         </is>
       </c>
     </row>
@@ -1209,11 +1220,11 @@
         </is>
       </c>
       <c r="I17" s="35" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="J17" s="34" t="inlineStr">
         <is>
-          <t>Finished. 17411 articles of 17447 URLs (99.8%); 165 empty_body. systemd inactive. File: ~/Downloads/uci.csv</t>
+          <t>Finished as of 2026-10-13. 17411 articles. systemd inactive. File: ~/Downloads/uci.csv</t>
         </is>
       </c>
     </row>
@@ -1245,11 +1256,11 @@
       </c>
       <c r="F18" s="33" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G18" s="33" t="n">
-        <v>99943</v>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G18" s="39" t="n">
+        <v>118949</v>
       </c>
       <c r="H18" s="33" t="inlineStr">
         <is>
@@ -1257,11 +1268,11 @@
         </is>
       </c>
       <c r="I18" s="35" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="J18" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@michigan; 99943 of 119764 (83.4%) as of 2026-10-08 17:11 UTC. http_429=21 (was 16 on Oct 7). http_301=1821.</t>
+          <t>Finished as of 2026-10-13. 118949 articles. systemd inactive. File: ~/Downloads/michigan.csv</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1307,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G19" s="33" t="n">
+      <c r="G19" s="39" t="n">
         <v>21079</v>
       </c>
       <c r="H19" s="33" t="inlineStr">
@@ -1304,12 +1315,12 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I19" s="36" t="n">
-        <v>46296</v>
+      <c r="I19" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J19" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-05 before later downloads. 21079 articles of 22605 URLs (93.2%); 1660 empty_body, 2 http_500. systemd inactive. File: ~/Downloads/ucsd.csv</t>
+          <t>Finished as of 2026-10-13. 21079 articles. systemd inactive. File: ~/Downloads/ucsd.csv</t>
         </is>
       </c>
     </row>
@@ -1341,23 +1352,23 @@
       </c>
       <c r="F20" s="33" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G20" s="33" t="n">
-        <v>45147</v>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G20" s="39" t="n">
+        <v>50898</v>
       </c>
       <c r="H20" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I20" s="36" t="n">
-        <v>46296</v>
+      <c r="I20" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J20" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@texan; 45147 of 51636 (87.4%) as of 2026-10-08 17:11 UTC. empty_body=407, http_403=7.</t>
+          <t>Finished as of 2026-10-13. 50898 articles. systemd inactive. File: ~/Downloads/texan.csv</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1403,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G21" s="33" t="n">
+      <c r="G21" s="39" t="n">
         <v>37215</v>
       </c>
       <c r="H21" s="33" t="inlineStr">
@@ -1400,12 +1411,12 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I21" s="36" t="n">
-        <v>46296</v>
+      <c r="I21" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J21" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-07. 37215 of 40465 (92.0%); empty_body=4202, http_404=1. systemd inactive. File: ~/Downloads/nexus.csv</t>
+          <t>Finished as of 2026-10-13. 37215 articles. systemd inactive. File: ~/Downloads/nexus.csv</t>
         </is>
       </c>
     </row>
@@ -1440,20 +1451,20 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G22" s="33" t="n">
-        <v>44450</v>
+      <c r="G22" s="39" t="n">
+        <v>75850</v>
       </c>
       <c r="H22" s="33" t="inlineStr">
         <is>
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I22" s="36" t="n">
-        <v>46296</v>
+      <c r="I22" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J22" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@illini; 44450 of 100022 (44.4%) as of 2026-10-08 17:11 UTC.</t>
+          <t>newspaper-scraper@illini; 75850 articles as of 2026-10-13. systemd active on AWS VM.</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1499,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G23" s="33" t="n">
+      <c r="G23" s="39" t="n">
         <v>40280</v>
       </c>
       <c r="H23" s="33" t="inlineStr">
@@ -1496,12 +1507,12 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I23" s="36" t="n">
-        <v>46296</v>
+      <c r="I23" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J23" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-07. 40280 of 41051 (98.1%); empty_body=1017, http_521=1. systemd inactive. File: ~/Downloads/technician.csv</t>
+          <t>Finished as of 2026-10-13. 40280 articles. systemd inactive. File: ~/Downloads/technician.csv</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1547,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G24" s="33" t="n">
+      <c r="G24" s="39" t="n">
         <v>13354</v>
       </c>
       <c r="H24" s="33" t="inlineStr">
@@ -1544,12 +1555,12 @@
           <t>AWS VM</t>
         </is>
       </c>
-      <c r="I24" s="36" t="n">
-        <v>46296</v>
+      <c r="I24" s="35" t="n">
+        <v>46308</v>
       </c>
       <c r="J24" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-04. 13354 of 13650 (97.8%); 517 empty_body, 32 pre_2000. File: ~/Downloads/statesman.csv</t>
+          <t>Finished as of 2026-10-13. 13354 articles. systemd inactive. File: ~/Downloads/statesman.csv</t>
         </is>
       </c>
     </row>
@@ -1584,8 +1595,8 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G25" s="0" t="n">
-        <v>36129</v>
+      <c r="G25" s="22" t="n">
+        <v>56979</v>
       </c>
       <c r="H25" s="0" t="inlineStr">
         <is>
@@ -1593,11 +1604,11 @@
         </is>
       </c>
       <c r="I25" s="37" t="n">
-        <v>46297</v>
+        <v>46308</v>
       </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tarheel; 36129 of 81683 (44.2%) as of 2026-10-08 17:11 UTC. empty_body=5194, http_403=28.</t>
+          <t>newspaper-scraper@tarheel; 56979 articles as of 2026-10-13. systemd active on AWS VM.</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1643,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G26" s="0" t="n">
+      <c r="G26" s="22" t="n">
         <v>9791</v>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1641,11 +1652,11 @@
         </is>
       </c>
       <c r="I26" s="37" t="n">
-        <v>46297</v>
+        <v>46308</v>
       </c>
       <c r="J26" s="0" t="inlineStr">
         <is>
-          <t>Finished 2026-10-04. 9791 of 10144 (96.5%); 550 empty_body, 1 http_520, 1 http_525. File: ~/Downloads/highlander.csv</t>
+          <t>Finished as of 2026-10-13. 9791 articles. systemd inactive. File: ~/Downloads/highlander.csv</t>
         </is>
       </c>
     </row>
@@ -1677,11 +1688,11 @@
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G27" s="0" t="n">
-        <v>24237</v>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="n">
+        <v>51122</v>
       </c>
       <c r="H27" s="0" t="inlineStr">
         <is>
@@ -1689,11 +1700,11 @@
         </is>
       </c>
       <c r="I27" s="37" t="n">
-        <v>46299</v>
+        <v>46308</v>
       </c>
       <c r="J27" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@collegian; 24237 of 52185 (46.4%) as of 2026-10-08 17:11 UTC. empty_body=306, pre_2000=234.</t>
+          <t>Finished as of 2026-10-13. 51122 articles. systemd inactive. File: ~/Downloads/collegian.csv</t>
         </is>
       </c>
     </row>
@@ -1728,8 +1739,8 @@
           <t>running</t>
         </is>
       </c>
-      <c r="G28" s="0" t="n">
-        <v>21590</v>
+      <c r="G28" s="22" t="n">
+        <v>53190</v>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
@@ -1737,11 +1748,11 @@
         </is>
       </c>
       <c r="I28" s="37" t="n">
-        <v>46299</v>
+        <v>46308</v>
       </c>
       <c r="J28" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@mndaily; 21590 of 80516 (26.8%) as of 2026-10-08 17:11 UTC. pre_2000=14440 skipped.</t>
+          <t>newspaper-scraper@mndaily; 53190 articles as of 2026-10-13. systemd active on AWS VM.</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1832,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G30" s="0" t="n">
+      <c r="G30" s="22" t="n">
         <v>7337</v>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1830,11 +1841,11 @@
         </is>
       </c>
       <c r="I30" s="37" t="n">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="J30" s="0" t="inlineStr">
         <is>
-          <t>Finished 2026-10-06. 7337 of 7455 (98.4%); empty_body=130. systemd inactive. File: ~/Downloads/tiger.csv</t>
+          <t>Finished as of 2026-10-13. 7337 articles. systemd inactive. File: ~/Downloads/tiger.csv</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1880,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G31" s="0" t="n">
+      <c r="G31" s="22" t="n">
         <v>335</v>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -1878,11 +1889,11 @@
         </is>
       </c>
       <c r="I31" s="37" t="n">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="J31" s="0" t="inlineStr">
         <is>
-          <t>Finished 2026-10-05. 335 of 336 (99.7%); 1 empty_body. File: ~/Downloads/vector.csv</t>
+          <t>Finished as of 2026-10-13. 335 articles. systemd inactive. File: ~/Downloads/vector.csv</t>
         </is>
       </c>
     </row>
@@ -1942,11 +1953,11 @@
         </is>
       </c>
       <c r="I33" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J33" s="34" t="inlineStr">
         <is>
-          <t>Finished. 4039 articles of 4320 URLs (93.5%); 288 empty_body. systemd inactive. File: ~/Downloads/conncoll.csv</t>
+          <t>Finished as of 2026-10-13. 4039 articles. systemd inactive. File: ~/Downloads/conncoll.csv</t>
         </is>
       </c>
     </row>
@@ -1990,11 +2001,11 @@
         </is>
       </c>
       <c r="I34" s="35" t="n">
-        <v>46294</v>
+        <v>46308</v>
       </c>
       <c r="J34" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3671 articles of 3696 URLs (99.3%); 29 empty_body. systemd inactive. File: ~/Downloads/denison.csv</t>
+          <t>Finished as of 2026-10-13. 3671 articles. systemd inactive. File: ~/Downloads/denison.csv</t>
         </is>
       </c>
     </row>
@@ -2038,11 +2049,11 @@
         </is>
       </c>
       <c r="I35" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J35" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3449 articles of 3583 URLs (96.3%); 135 empty_body, 3 network_error. systemd inactive. File: ~/Downloads/fandm.csv</t>
+          <t>Finished as of 2026-10-13. 3449 articles. systemd inactive. File: ~/Downloads/fandm.csv</t>
         </is>
       </c>
     </row>
@@ -2086,11 +2097,11 @@
         </is>
       </c>
       <c r="I36" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J36" s="34" t="inlineStr">
         <is>
-          <t>Finished. 15573 articles of 15690 URLs (99.3%); 124 empty_body. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
+          <t>Finished as of 2026-10-13. 15573 articles. systemd inactive. File: ~/Downloads/hillsdale.csv</t>
         </is>
       </c>
     </row>
@@ -2134,11 +2145,11 @@
         </is>
       </c>
       <c r="I37" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J37" s="34" t="inlineStr">
         <is>
-          <t>Finished. 9892 articles of 10055 URLs (98.4%); 176 empty_body, 1 http_500, 3 network_error. systemd inactive. File: ~/Downloads/occidental.csv</t>
+          <t>Finished as of 2026-10-13. 9892 articles. systemd inactive. File: ~/Downloads/occidental.csv</t>
         </is>
       </c>
     </row>
@@ -2182,11 +2193,11 @@
         </is>
       </c>
       <c r="I38" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J38" s="34" t="inlineStr">
         <is>
-          <t>Finished. 12798 articles of 13251 URLs (96.6%); 75 empty_body, 578 pre_2000. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
+          <t>Finished as of 2026-10-13. 12798 articles. systemd inactive. File: ~/Downloads/swarthmore.csv</t>
         </is>
       </c>
     </row>
@@ -2230,11 +2241,11 @@
         </is>
       </c>
       <c r="I39" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J39" s="34" t="inlineStr">
         <is>
-          <t>Finished. 1604 articles of 1626 URLs (98.6%); 44 empty_body. systemd inactive. File: ~/Downloads/union.csv</t>
+          <t>Finished as of 2026-10-13. 1604 articles. systemd inactive. File: ~/Downloads/union.csv</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2280,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G40" s="24" t="n">
+      <c r="G40" s="30" t="n">
         <v>21881</v>
       </c>
       <c r="H40" s="33" t="inlineStr">
@@ -2278,11 +2289,11 @@
         </is>
       </c>
       <c r="I40" s="35" t="n">
-        <v>46294</v>
+        <v>46308</v>
       </c>
       <c r="J40" s="34" t="inlineStr">
         <is>
-          <t>Finished. 21881 articles of 21917 URLs (99.8%); 43 empty_body. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
+          <t>Finished as of 2026-10-13. 21881 articles. systemd inactive. File: ~/Downloads/wesleyan.csv</t>
         </is>
       </c>
     </row>
@@ -2317,8 +2328,8 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G41" s="33" t="n">
-        <v>11405</v>
+      <c r="G41" s="39" t="n">
+        <v>11420</v>
       </c>
       <c r="H41" s="33" t="inlineStr">
         <is>
@@ -2326,11 +2337,11 @@
         </is>
       </c>
       <c r="I41" s="35" t="n">
-        <v>46295</v>
+        <v>46308</v>
       </c>
       <c r="J41" s="34" t="inlineStr">
         <is>
-          <t>Finished 2026-10-04. 11405 of 11437 (99.7%); 16 empty_body, 15 http_403, 1 http_404. File: ~/Downloads/tsl.csv</t>
+          <t>Finished as of 2026-10-13. 11420 articles. systemd inactive. File: ~/Downloads/tsl.csv</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2376,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G42" s="0" t="n">
+      <c r="G42" s="22" t="n">
         <v>7805</v>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -2374,11 +2385,11 @@
         </is>
       </c>
       <c r="I42" s="37" t="n">
-        <v>46300</v>
+        <v>46308</v>
       </c>
       <c r="J42" s="0" t="inlineStr">
         <is>
-          <t>Finished 2026-10-06. 7805 of 7941 (98.3%); empty_body=135, http_404=1. systemd inactive. File: ~/Downloads/carleton.csv</t>
+          <t>Finished as of 2026-10-13. 7805 articles. systemd inactive. File: ~/Downloads/carleton.csv</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2424,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G43" s="0" t="n">
+      <c r="G43" s="22" t="n">
         <v>9036</v>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -2422,11 +2433,11 @@
         </is>
       </c>
       <c r="I43" s="37" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="J43" s="0" t="inlineStr">
         <is>
-          <t>Finished 2026-10-08. 9036 of 9420 (95.9%); empty_body=392, network_error=1. systemd inactive. File: ~/Downloads/macweekly.csv</t>
+          <t>Finished as of 2026-10-13. 9036 articles. systemd inactive. File: ~/Downloads/macweekly.csv</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2472,7 @@
           <t>done</t>
         </is>
       </c>
-      <c r="G44" s="0" t="n">
+      <c r="G44" s="22" t="n">
         <v>9054</v>
       </c>
       <c r="H44" s="0" t="inlineStr">
@@ -2470,11 +2481,11 @@
         </is>
       </c>
       <c r="I44" s="37" t="n">
-        <v>46301</v>
+        <v>46308</v>
       </c>
       <c r="J44" s="0" t="inlineStr">
         <is>
-          <t>Finished 2026-10-08. 9054 of 9228 (98.1%); empty_body=184. systemd inactive. File: ~/Downloads/sandb.csv</t>
+          <t>Finished as of 2026-10-13. 9054 articles. systemd inactive. File: ~/Downloads/sandb.csv</t>
         </is>
       </c>
     </row>
@@ -2506,11 +2517,11 @@
       </c>
       <c r="F45" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G45" s="0" t="n">
-        <v>7250</v>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G45" s="22" t="n">
+        <v>15466</v>
       </c>
       <c r="H45" s="0" t="inlineStr">
         <is>
@@ -2518,11 +2529,11 @@
         </is>
       </c>
       <c r="I45" s="37" t="n">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="J45" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@colgate; 7250 of 15489 (46.8%) as of 2026-10-08 17:11 UTC. http_500=1.</t>
+          <t>Finished as of 2026-10-13. 15466 articles. systemd inactive. File: ~/Downloads/colgate.csv</t>
         </is>
       </c>
     </row>
@@ -2554,11 +2565,11 @@
       </c>
       <c r="F46" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
-      </c>
-      <c r="G46" s="0" t="n">
-        <v>7300</v>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G46" s="22" t="n">
+        <v>11555</v>
       </c>
       <c r="H46" s="0" t="inlineStr">
         <is>
@@ -2566,11 +2577,11 @@
         </is>
       </c>
       <c r="I46" s="37" t="n">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="J46" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@bucknellian; 7300 of 11583 (63.0%) as of 2026-10-08 17:11 UTC. empty_body=11, http_404=2.</t>
+          <t>Finished as of 2026-10-13. 11555 articles. systemd inactive. File: ~/Downloads/bucknellian.csv</t>
         </is>
       </c>
     </row>
@@ -2630,11 +2641,11 @@
         </is>
       </c>
       <c r="I48" s="35" t="n">
-        <v>46291</v>
+        <v>46308</v>
       </c>
       <c r="J48" s="34" t="inlineStr">
         <is>
-          <t>Finished. 11331 articles of 11390 URLs (99.5%); 569 empty_body, 1 http_404. systemd inactive. File: ~/Downloads/biola.csv</t>
+          <t>Finished as of 2026-10-13. 11331 articles. systemd inactive. File: ~/Downloads/biola.csv</t>
         </is>
       </c>
     </row>
@@ -2678,11 +2689,11 @@
         </is>
       </c>
       <c r="I49" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J49" s="34" t="inlineStr">
         <is>
-          <t>Finished. 682 articles of 698 URLs (97.7%); 2 empty_body, 28 pre_2000. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
+          <t>Finished as of 2026-10-13. 682 articles. systemd inactive. File: ~/Downloads/lipscomb.csv</t>
         </is>
       </c>
     </row>
@@ -2726,11 +2737,11 @@
         </is>
       </c>
       <c r="I50" s="35" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="J50" s="34" t="inlineStr">
         <is>
-          <t>Finished. 3950 articles of 4044 URLs (97.7%); 98 empty_body. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
+          <t>Finished as of 2026-10-13. 3950 articles. systemd inactive. File: ~/Downloads/lomabeat.csv</t>
         </is>
       </c>
     </row>
@@ -2774,11 +2785,11 @@
         </is>
       </c>
       <c r="I51" s="35" t="n">
-        <v>46291</v>
+        <v>46308</v>
       </c>
       <c r="J51" s="34" t="inlineStr">
         <is>
-          <t>Finished. 26208 articles of 26572 URLs (98.6%); 649 empty_body, 1 network_error. systemd inactive. File: ~/Downloads/smu.csv</t>
+          <t>Finished as of 2026-10-13. 26208 articles. systemd inactive. File: ~/Downloads/smu.csv</t>
         </is>
       </c>
     </row>
@@ -2822,11 +2833,11 @@
         </is>
       </c>
       <c r="I52" s="35" t="n">
-        <v>46292</v>
+        <v>46308</v>
       </c>
       <c r="J52" s="34" t="inlineStr">
         <is>
-          <t>Finished. 5048 articles of 5208 URLs (96.9%); 320 empty_body. systemd inactive. File: ~/Downloads/stolaf.csv</t>
+          <t>Finished as of 2026-10-13. 5048 articles. systemd inactive. File: ~/Downloads/stolaf.csv | Blank Liberal Arts ranking row; covered under Christian Colleges / stolaf (already finished).</t>
         </is>
       </c>
     </row>
@@ -2870,11 +2881,1500 @@
         </is>
       </c>
       <c r="I53" s="35" t="n">
-        <v>46291</v>
+        <v>46308</v>
       </c>
       <c r="J53" s="34" t="inlineStr">
         <is>
-          <t>Finished. 25690 articles of 26172 URLs (98.2%); 862 empty_body, 6 http_404, 6 pre_2000. systemd inactive. File: ~/Downloads/tcu.csv</t>
+          <t>Finished as of 2026-10-13. 25690 articles. systemd inactive. File: ~/Downloads/tcu.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>Wabash College</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="inlineStr">
+        <is>
+          <t>The Bachelor</t>
+        </is>
+      </c>
+      <c r="C54" s="0" t="inlineStr">
+        <is>
+          <t>bachelor</t>
+        </is>
+      </c>
+      <c r="D54" s="0" t="inlineStr">
+        <is>
+          <t>bachelor.wabash.edu</t>
+        </is>
+      </c>
+      <c r="E54" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F54" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G54" s="21" t="n">
+        <v>692</v>
+      </c>
+      <c r="H54" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I54" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J54" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 692 articles. systemd inactive. File: ~/Downloads/bachelor.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>Bates College</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t>The Bates Student</t>
+        </is>
+      </c>
+      <c r="C55" s="0" t="inlineStr">
+        <is>
+          <t>bates</t>
+        </is>
+      </c>
+      <c r="D55" s="0" t="inlineStr">
+        <is>
+          <t>thebatesstudent.com</t>
+        </is>
+      </c>
+      <c r="E55" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G55" s="21" t="n">
+        <v>2297</v>
+      </c>
+      <c r="H55" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I55" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J55" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 2297 articles. systemd inactive. File: ~/Downloads/bates.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t>Baylor University</t>
+        </is>
+      </c>
+      <c r="B56" s="0" t="inlineStr">
+        <is>
+          <t>The Baylor Lariat</t>
+        </is>
+      </c>
+      <c r="C56" s="0" t="inlineStr">
+        <is>
+          <t>baylor</t>
+        </is>
+      </c>
+      <c r="D56" s="0" t="inlineStr">
+        <is>
+          <t>baylorlariat.com</t>
+        </is>
+      </c>
+      <c r="E56" s="0" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F56" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G56" s="21" t="n">
+        <v>4796</v>
+      </c>
+      <c r="H56" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I56" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J56" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@baylor; 4796 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t>Bowdoin College</t>
+        </is>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t>The Bowdoin Orient</t>
+        </is>
+      </c>
+      <c r="C57" s="0" t="inlineStr">
+        <is>
+          <t>bowdoin</t>
+        </is>
+      </c>
+      <c r="D57" s="0" t="inlineStr">
+        <is>
+          <t>bowdoinorient.com</t>
+        </is>
+      </c>
+      <c r="E57" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F57" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G57" s="21" t="n">
+        <v>5981</v>
+      </c>
+      <c r="H57" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I57" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J57" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 5981 articles. systemd inactive. File: ~/Downloads/bowdoin.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t>University of Rochester</t>
+        </is>
+      </c>
+      <c r="B58" s="0" t="inlineStr">
+        <is>
+          <t>Campus Times</t>
+        </is>
+      </c>
+      <c r="C58" s="0" t="inlineStr">
+        <is>
+          <t>campustimes</t>
+        </is>
+      </c>
+      <c r="D58" s="0" t="inlineStr">
+        <is>
+          <t>campustimes.org</t>
+        </is>
+      </c>
+      <c r="E58" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F58" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G58" s="21" t="n">
+        <v>7948</v>
+      </c>
+      <c r="H58" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I58" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J58" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@campustimes; 7948 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t>Case Western Reserve University</t>
+        </is>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t>The Observer</t>
+        </is>
+      </c>
+      <c r="C59" s="0" t="inlineStr">
+        <is>
+          <t>case</t>
+        </is>
+      </c>
+      <c r="D59" s="0" t="inlineStr">
+        <is>
+          <t>observer.case.edu</t>
+        </is>
+      </c>
+      <c r="E59" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F59" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G59" s="21" t="n">
+        <v>10125</v>
+      </c>
+      <c r="H59" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I59" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J59" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 10125 articles. systemd inactive. File: ~/Downloads/case.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="inlineStr">
+        <is>
+          <t>Davidson College</t>
+        </is>
+      </c>
+      <c r="B60" s="0" t="inlineStr">
+        <is>
+          <t>The Davidsonian</t>
+        </is>
+      </c>
+      <c r="C60" s="0" t="inlineStr">
+        <is>
+          <t>davidson</t>
+        </is>
+      </c>
+      <c r="D60" s="0" t="inlineStr">
+        <is>
+          <t>thedavidsonian.news</t>
+        </is>
+      </c>
+      <c r="E60" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F60" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G60" s="21" t="n">
+        <v>518</v>
+      </c>
+      <c r="H60" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I60" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J60" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 518 articles. systemd inactive. File: ~/Downloads/davidson.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="inlineStr">
+        <is>
+          <t>Dickinson College</t>
+        </is>
+      </c>
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t>The Dickinsonian</t>
+        </is>
+      </c>
+      <c r="C61" s="0" t="inlineStr">
+        <is>
+          <t>dickinson</t>
+        </is>
+      </c>
+      <c r="D61" s="0" t="inlineStr">
+        <is>
+          <t>thedickinsonian.com</t>
+        </is>
+      </c>
+      <c r="E61" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G61" s="21" t="n">
+        <v>4871</v>
+      </c>
+      <c r="H61" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I61" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J61" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 4871 articles. systemd inactive. File: ~/Downloads/dickinson.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="inlineStr">
+        <is>
+          <t>Fordham University</t>
+        </is>
+      </c>
+      <c r="B62" s="0" t="inlineStr">
+        <is>
+          <t>The Fordham Ram</t>
+        </is>
+      </c>
+      <c r="C62" s="0" t="inlineStr">
+        <is>
+          <t>fordham</t>
+        </is>
+      </c>
+      <c r="D62" s="0" t="inlineStr">
+        <is>
+          <t>thefordhamram.com</t>
+        </is>
+      </c>
+      <c r="E62" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F62" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G62" s="21" t="n">
+        <v>6575</v>
+      </c>
+      <c r="H62" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I62" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J62" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@fordham; 6575 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="inlineStr">
+        <is>
+          <t>Boston University</t>
+        </is>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t>The Daily Free Press</t>
+        </is>
+      </c>
+      <c r="C63" s="0" t="inlineStr">
+        <is>
+          <t>freepress</t>
+        </is>
+      </c>
+      <c r="D63" s="0" t="inlineStr">
+        <is>
+          <t>dailyfreepress.com</t>
+        </is>
+      </c>
+      <c r="E63" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F63" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G63" s="21" t="n">
+        <v>2050</v>
+      </c>
+      <c r="H63" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I63" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J63" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@freepress; 2050 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="inlineStr">
+        <is>
+          <t>Rutgers University, Camden</t>
+        </is>
+      </c>
+      <c r="B64" s="0" t="inlineStr">
+        <is>
+          <t>The Gleaner</t>
+        </is>
+      </c>
+      <c r="C64" s="0" t="inlineStr">
+        <is>
+          <t>gleaner</t>
+        </is>
+      </c>
+      <c r="D64" s="0" t="inlineStr">
+        <is>
+          <t>gleaner.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="E64" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F64" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G64" s="21" t="n">
+        <v>373</v>
+      </c>
+      <c r="H64" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I64" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J64" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 373 articles. systemd inactive. File: ~/Downloads/gleaner.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="inlineStr">
+        <is>
+          <t>Hamilton College</t>
+        </is>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t>The Spectator</t>
+        </is>
+      </c>
+      <c r="C65" s="0" t="inlineStr">
+        <is>
+          <t>hamilton</t>
+        </is>
+      </c>
+      <c r="D65" s="0" t="inlineStr">
+        <is>
+          <t>hcspectator.com</t>
+        </is>
+      </c>
+      <c r="E65" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F65" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G65" s="21" t="n">
+        <v>2884</v>
+      </c>
+      <c r="H65" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I65" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J65" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 2884 articles. systemd inactive. File: ~/Downloads/hamilton.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="inlineStr">
+        <is>
+          <t>Tulane University of Louisiana</t>
+        </is>
+      </c>
+      <c r="B66" s="0" t="inlineStr">
+        <is>
+          <t>The Tulane Hullabaloo</t>
+        </is>
+      </c>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t>hullabaloo</t>
+        </is>
+      </c>
+      <c r="D66" s="0" t="inlineStr">
+        <is>
+          <t>tulanehullabaloo.com</t>
+        </is>
+      </c>
+      <c r="E66" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F66" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G66" s="21" t="n">
+        <v>650</v>
+      </c>
+      <c r="H66" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I66" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J66" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@hullabaloo; 650 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t>Lafayette College</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t>The Lafayette</t>
+        </is>
+      </c>
+      <c r="C67" s="0" t="inlineStr">
+        <is>
+          <t>lafayette</t>
+        </is>
+      </c>
+      <c r="D67" s="0" t="inlineStr">
+        <is>
+          <t>lafayettestudentnews.com</t>
+        </is>
+      </c>
+      <c r="E67" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F67" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G67" s="21" t="n">
+        <v>8987</v>
+      </c>
+      <c r="H67" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I67" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J67" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 8987 articles. systemd inactive. File: ~/Downloads/lafayette.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
+          <t>Lehigh University</t>
+        </is>
+      </c>
+      <c r="B68" s="0" t="inlineStr">
+        <is>
+          <t>The Brown and White</t>
+        </is>
+      </c>
+      <c r="C68" s="0" t="inlineStr">
+        <is>
+          <t>lehigh</t>
+        </is>
+      </c>
+      <c r="D68" s="0" t="inlineStr">
+        <is>
+          <t>thebrownandwhite.com</t>
+        </is>
+      </c>
+      <c r="E68" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F68" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G68" s="21" t="n">
+        <v>6399</v>
+      </c>
+      <c r="H68" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I68" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J68" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@lehigh; 6399 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t>Northeastern University</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t>The Huntington News</t>
+        </is>
+      </c>
+      <c r="C69" s="0" t="inlineStr">
+        <is>
+          <t>northeastern</t>
+        </is>
+      </c>
+      <c r="D69" s="0" t="inlineStr">
+        <is>
+          <t>huntnewsnu.com</t>
+        </is>
+      </c>
+      <c r="E69" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F69" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G69" s="21" t="n">
+        <v>6298</v>
+      </c>
+      <c r="H69" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I69" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J69" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@northeastern; 6298 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
+          <t>Furman Univeristy</t>
+        </is>
+      </c>
+      <c r="B70" s="0" t="inlineStr">
+        <is>
+          <t>The Paladin</t>
+        </is>
+      </c>
+      <c r="C70" s="0" t="inlineStr">
+        <is>
+          <t>paladin</t>
+        </is>
+      </c>
+      <c r="D70" s="0" t="inlineStr">
+        <is>
+          <t>thepaladin.news</t>
+        </is>
+      </c>
+      <c r="E70" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G70" s="21" t="n">
+        <v>2798</v>
+      </c>
+      <c r="H70" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I70" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J70" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 2798 articles. systemd inactive. File: ~/Downloads/paladin.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t>Pepperdine University</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t>Pepperdine Graphic</t>
+        </is>
+      </c>
+      <c r="C71" s="0" t="inlineStr">
+        <is>
+          <t>pepperdine</t>
+        </is>
+      </c>
+      <c r="D71" s="0" t="inlineStr">
+        <is>
+          <t>pepperdine-graphic.com</t>
+        </is>
+      </c>
+      <c r="E71" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F71" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G71" s="21" t="n">
+        <v>1036</v>
+      </c>
+      <c r="H71" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I71" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J71" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 1036 articles. systemd inactive. File: ~/Downloads/pepperdine.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t>Washington and Lee Univeristy</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="inlineStr">
+        <is>
+          <t>The Ring-tum Phi</t>
+        </is>
+      </c>
+      <c r="C72" s="0" t="inlineStr">
+        <is>
+          <t>ringtumphi</t>
+        </is>
+      </c>
+      <c r="D72" s="0" t="inlineStr">
+        <is>
+          <t>ringtumphi.net</t>
+        </is>
+      </c>
+      <c r="E72" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F72" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G72" s="21" t="n">
+        <v>2673</v>
+      </c>
+      <c r="H72" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I72" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J72" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 2673 articles. systemd inactive. File: ~/Downloads/ringtumphi.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t>Smith College</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t>The Sophian</t>
+        </is>
+      </c>
+      <c r="C73" s="0" t="inlineStr">
+        <is>
+          <t>sophian</t>
+        </is>
+      </c>
+      <c r="D73" s="0" t="inlineStr">
+        <is>
+          <t>thesophian.com</t>
+        </is>
+      </c>
+      <c r="E73" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G73" s="21" t="n">
+        <v>2087</v>
+      </c>
+      <c r="H73" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I73" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J73" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 2087 articles. systemd inactive. File: ~/Downloads/sophian.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t>Trinity University</t>
+        </is>
+      </c>
+      <c r="B74" s="0" t="inlineStr">
+        <is>
+          <t>The Trinitonian</t>
+        </is>
+      </c>
+      <c r="C74" s="0" t="inlineStr">
+        <is>
+          <t>trinitonian</t>
+        </is>
+      </c>
+      <c r="D74" s="0" t="inlineStr">
+        <is>
+          <t>trinitonian.com</t>
+        </is>
+      </c>
+      <c r="E74" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F74" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G74" s="21" t="n">
+        <v>5500</v>
+      </c>
+      <c r="H74" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I74" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J74" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@trinitonian; 5500 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t>Trinity College</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t>The Trinity Tripod</t>
+        </is>
+      </c>
+      <c r="C75" s="0" t="inlineStr">
+        <is>
+          <t>tripod</t>
+        </is>
+      </c>
+      <c r="D75" s="0" t="inlineStr">
+        <is>
+          <t>trinitytripod.com</t>
+        </is>
+      </c>
+      <c r="E75" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F75" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G75" s="21" t="n">
+        <v>3925</v>
+      </c>
+      <c r="H75" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I75" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J75" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 3925 articles. systemd inactive. File: ~/Downloads/tripod.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t>Vanderbilt University</t>
+        </is>
+      </c>
+      <c r="B76" s="0" t="inlineStr">
+        <is>
+          <t>The Vanderbilt Hustler</t>
+        </is>
+      </c>
+      <c r="C76" s="0" t="inlineStr">
+        <is>
+          <t>vanderbilt</t>
+        </is>
+      </c>
+      <c r="D76" s="0" t="inlineStr">
+        <is>
+          <t>vanderbilthustler.com</t>
+        </is>
+      </c>
+      <c r="E76" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F76" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G76" s="21" t="n">
+        <v>6398</v>
+      </c>
+      <c r="H76" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I76" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J76" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@vanderbilt; 6398 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t>Villanova University</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t>The Villanovan</t>
+        </is>
+      </c>
+      <c r="C77" s="0" t="inlineStr">
+        <is>
+          <t>villanova</t>
+        </is>
+      </c>
+      <c r="D77" s="0" t="inlineStr">
+        <is>
+          <t>villanovan.com</t>
+        </is>
+      </c>
+      <c r="E77" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F77" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G77" s="21" t="n">
+        <v>6745</v>
+      </c>
+      <c r="H77" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I77" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J77" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@villanova; 6745 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="inlineStr">
+        <is>
+          <t>Wake Forest University</t>
+        </is>
+      </c>
+      <c r="B78" s="0" t="inlineStr">
+        <is>
+          <t>Old Gold &amp; Black</t>
+        </is>
+      </c>
+      <c r="C78" s="0" t="inlineStr">
+        <is>
+          <t>wakeforest</t>
+        </is>
+      </c>
+      <c r="D78" s="0" t="inlineStr">
+        <is>
+          <t>wfuogb.com</t>
+        </is>
+      </c>
+      <c r="E78" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F78" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="G78" s="21" t="n">
+        <v>6482</v>
+      </c>
+      <c r="H78" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I78" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J78" s="0" t="inlineStr">
+        <is>
+          <t>newspaper-scraper@wakeforest; 6482 articles as of 2026-10-13. systemd active on AWS VM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t>Wellesley College</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t>The Wellesley News</t>
+        </is>
+      </c>
+      <c r="C79" s="0" t="inlineStr">
+        <is>
+          <t>wellesley</t>
+        </is>
+      </c>
+      <c r="D79" s="0" t="inlineStr">
+        <is>
+          <t>thewellesleynews.com</t>
+        </is>
+      </c>
+      <c r="E79" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F79" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G79" s="21" t="n">
+        <v>4796</v>
+      </c>
+      <c r="H79" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I79" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J79" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 4796 articles. systemd inactive. File: ~/Downloads/wellesley.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t>Wheaton College</t>
+        </is>
+      </c>
+      <c r="B80" s="0" t="inlineStr">
+        <is>
+          <t>The Wheaton Wire</t>
+        </is>
+      </c>
+      <c r="C80" s="0" t="inlineStr">
+        <is>
+          <t>wheatonwire</t>
+        </is>
+      </c>
+      <c r="D80" s="0" t="inlineStr">
+        <is>
+          <t>wheatonwire.com</t>
+        </is>
+      </c>
+      <c r="E80" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F80" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G80" s="21" t="n">
+        <v>947</v>
+      </c>
+      <c r="H80" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I80" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J80" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 947 articles. systemd inactive. File: ~/Downloads/wheatonwire.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t>Williams College</t>
+        </is>
+      </c>
+      <c r="B81" s="0" t="inlineStr">
+        <is>
+          <t>The Williams Record</t>
+        </is>
+      </c>
+      <c r="C81" s="0" t="inlineStr">
+        <is>
+          <t>williams</t>
+        </is>
+      </c>
+      <c r="D81" s="0" t="inlineStr">
+        <is>
+          <t>williamsrecord.com</t>
+        </is>
+      </c>
+      <c r="E81" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F81" s="0" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G81" s="21" t="n">
+        <v>4226</v>
+      </c>
+      <c r="H81" s="0" t="inlineStr">
+        <is>
+          <t>AWS VM</t>
+        </is>
+      </c>
+      <c r="I81" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J81" s="0" t="inlineStr">
+        <is>
+          <t>Finished as of 2026-10-13. 4226 articles. systemd inactive. File: ~/Downloads/williams.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>College of the Ozarks</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>The Outlook</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>excluded</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="I82" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>No dedicated student-paper site found. cofo.edu/News is institutional only (2026-10-13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Moody Bible Institute</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>The Moody Standard</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>excluded</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="I83" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Closed 2019 after 84 years. moodystandard.com DNS dead; historical archive only (2026-10-13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>United States Air Force Academy</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Academy Spirit</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>excluded</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="I84" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Print ended 2015. usafa.af.mil is institutional, not independent student paper (2026-10-13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>United States Military Academy at West Point</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Pointer View</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>westpoint.edu</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>needs_adapter</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="I85" s="37" t="n">
+        <v>46308</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Live: westpoint.edu/pointer-view. Historical: usmalibrary.contentdm. Needs adapter (2026-10-13).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Status tracker for overnight finishes and CAP-20 wave 21.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -4234,27 +4234,27 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="0" t="inlineStr">
         <is>
           <t>College of the Ozarks</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="0" t="inlineStr">
         <is>
           <t>The Outlook</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E82" s="0" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="0" t="inlineStr">
         <is>
           <t>excluded</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="H82" s="0" t="inlineStr">
         <is>
           <t>research</t>
         </is>
@@ -4262,34 +4262,34 @@
       <c r="I82" s="37" t="n">
         <v>46308</v>
       </c>
-      <c r="J82" t="inlineStr">
+      <c r="J82" s="0" t="inlineStr">
         <is>
           <t>No dedicated student-paper site found. cofo.edu/News is institutional only (2026-10-13).</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="0" t="inlineStr">
         <is>
           <t>Moody Bible Institute</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="0" t="inlineStr">
         <is>
           <t>The Moody Standard</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E83" s="0" t="inlineStr">
         <is>
           <t>Christian Colleges</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F83" s="0" t="inlineStr">
         <is>
           <t>excluded</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr">
+      <c r="H83" s="0" t="inlineStr">
         <is>
           <t>research</t>
         </is>
@@ -4297,34 +4297,34 @@
       <c r="I83" s="37" t="n">
         <v>46308</v>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="J83" s="0" t="inlineStr">
         <is>
           <t>Closed 2019 after 84 years. moodystandard.com DNS dead; historical archive only (2026-10-13).</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="0" t="inlineStr">
         <is>
           <t>United States Air Force Academy</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="0" t="inlineStr">
         <is>
           <t>Academy Spirit</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E84" s="0" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F84" s="0" t="inlineStr">
         <is>
           <t>excluded</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H84" s="0" t="inlineStr">
         <is>
           <t>research</t>
         </is>
@@ -4332,39 +4332,39 @@
       <c r="I84" s="37" t="n">
         <v>46308</v>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="J84" s="0" t="inlineStr">
         <is>
           <t>Print ended 2015. usafa.af.mil is institutional, not independent student paper (2026-10-13).</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="0" t="inlineStr">
         <is>
           <t>United States Military Academy at West Point</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="0" t="inlineStr">
         <is>
           <t>Pointer View</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="0" t="inlineStr">
         <is>
           <t>westpoint.edu</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E85" s="0" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F85" s="0" t="inlineStr">
         <is>
           <t>needs_adapter</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H85" s="0" t="inlineStr">
         <is>
           <t>research</t>
         </is>
@@ -4372,9 +4372,150 @@
       <c r="I85" s="37" t="n">
         <v>46308</v>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="J85" s="0" t="inlineStr">
         <is>
           <t>Live: westpoint.edu/pointer-view. Historical: usmalibrary.contentdm. Needs adapter (2026-10-13).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="inlineStr">
+        <is>
+          <t>Boston College</t>
+        </is>
+      </c>
+      <c r="B86" s="0" t="inlineStr">
+        <is>
+          <t>The Heights</t>
+        </is>
+      </c>
+      <c r="C86" s="0" t="inlineStr">
+        <is>
+          <t>bc</t>
+        </is>
+      </c>
+      <c r="D86" s="0" t="inlineStr">
+        <is>
+          <t>bcheights.com</t>
+        </is>
+      </c>
+      <c r="E86" s="0" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F86" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H86" s="0" t="inlineStr">
+        <is>
+          <t>t3.xlarge</t>
+        </is>
+      </c>
+      <c r="I86" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="J86" s="0" t="inlineStr">
+        <is>
+          <t>Started wave21 full scrape 2026-10-13 (CAP 20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="inlineStr">
+        <is>
+          <t>Berea College</t>
+        </is>
+      </c>
+      <c r="B87" s="0" t="inlineStr">
+        <is>
+          <t>The Pinnacle</t>
+        </is>
+      </c>
+      <c r="C87" s="0" t="inlineStr">
+        <is>
+          <t>berea</t>
+        </is>
+      </c>
+      <c r="D87" s="0" t="inlineStr">
+        <is>
+          <t>pinnacle.berea.edu</t>
+        </is>
+      </c>
+      <c r="E87" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F87" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H87" s="0" t="inlineStr">
+        <is>
+          <t>t3.xlarge</t>
+        </is>
+      </c>
+      <c r="I87" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="J87" s="0" t="inlineStr">
+        <is>
+          <t>Started wave21 full scrape 2026-10-13 (CAP 20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="inlineStr">
+        <is>
+          <t>The University of the South</t>
+        </is>
+      </c>
+      <c r="B88" s="0" t="inlineStr">
+        <is>
+          <t>The Sewanee Purple</t>
+        </is>
+      </c>
+      <c r="C88" s="0" t="inlineStr">
+        <is>
+          <t>sewanee</t>
+        </is>
+      </c>
+      <c r="D88" s="0" t="inlineStr">
+        <is>
+          <t>thesewaneepurple.org</t>
+        </is>
+      </c>
+      <c r="E88" s="0" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F88" s="0" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="H88" s="0" t="inlineStr">
+        <is>
+          <t>t3.xlarge</t>
+        </is>
+      </c>
+      <c r="I88" s="0" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="J88" s="0" t="inlineStr">
+        <is>
+          <t>Started wave21 full scrape 2026-10-13 (CAP 20).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage wave 22 refill and mark Oct-14 403 stops as blocked.
</commit_message>
<xml_diff>
--- a/data/targets_raw.xlsx
+++ b/data/targets_raw.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="19" min="1" max="1"/>
@@ -920,7 +920,7 @@
       </c>
       <c r="J10" s="34" t="inlineStr">
         <is>
-          <t>Not cleared on the VM: homepage timeout, article pages HTTP 508. Crawl-delay 30; ~8.2k URLs. Retry from Mac, wait, or skip.</t>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
         </is>
       </c>
     </row>
@@ -1000,11 +1000,11 @@
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G12" s="39" t="n">
-        <v>30994</v>
+        <v>33200</v>
       </c>
       <c r="H12" s="33" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J12" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@hatchet; 30994 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@hatchet; 30994 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (33200 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -1048,11 +1048,11 @@
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G13" s="39" t="n">
-        <v>30550</v>
+        <v>36807</v>
       </c>
       <c r="H13" s="33" t="inlineStr">
         <is>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="J13" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@stanford; 30550 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@stanford; 30550 articles as of 2026-10-13. systemd active on AWS VM. | Finished as of 2026-10-14. 36807 articles. File: ~/Downloads/stanford.csv</t>
         </is>
       </c>
     </row>
@@ -1096,11 +1096,11 @@
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G14" s="39" t="n">
-        <v>30250</v>
+        <v>31890</v>
       </c>
       <c r="H14" s="33" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="J14" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@marquette; 30250 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@marquette; 30250 articles as of 2026-10-13. systemd active on AWS VM. | Finished as of 2026-10-14. 31890 articles. File: ~/Downloads/marquette.csv</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="E22" s="33" t="inlineStr">
         <is>
-          <t>National Universities | Public Universities</t>
+          <t>Public Universities</t>
         </is>
       </c>
       <c r="F22" s="33" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="H22" s="33" t="inlineStr">
         <is>
-          <t>AWS VM</t>
+          <t>t3.xlarge</t>
         </is>
       </c>
       <c r="I22" s="35" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J22" s="34" t="inlineStr">
         <is>
-          <t>newspaper-scraper@illini; 75850 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@illini; 75850 articles as of 2026-10-13. systemd active on AWS VM. | Still running as of 2026-10-14 (CAP 20).</t>
         </is>
       </c>
     </row>
@@ -1587,16 +1587,16 @@
       </c>
       <c r="E25" s="0" t="inlineStr">
         <is>
-          <t>National Universities | Public Universities</t>
+          <t>Public Universities</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G25" s="22" t="n">
-        <v>56979</v>
+        <v>58600</v>
       </c>
       <c r="H25" s="0" t="inlineStr">
         <is>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@tarheel; 56979 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@tarheel; 56979 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (58600 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t>University of Minnesota, Twin Cities</t>
+          <t>University of Minnesota</t>
         </is>
       </c>
       <c r="B28" s="0" t="inlineStr">
@@ -1731,16 +1731,16 @@
       </c>
       <c r="E28" s="0" t="inlineStr">
         <is>
-          <t>National Universities | Public Universities</t>
+          <t>National Universities</t>
         </is>
       </c>
       <c r="F28" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G28" s="22" t="n">
-        <v>53190</v>
+        <v>54761</v>
       </c>
       <c r="H28" s="0" t="inlineStr">
         <is>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="J28" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@mndaily; 53190 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@mndaily; 53190 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (54761 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t>Not cleared. VM 200-test HTTP 403 on /opinions/satire/; block cooldown. Probe of two news articles OK. Do not start full until a later 200-test passes.</t>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="H56" s="0" t="inlineStr">
         <is>
-          <t>AWS VM</t>
+          <t>t3.xlarge</t>
         </is>
       </c>
       <c r="I56" s="37" t="n">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="J56" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@baylor; 4796 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@baylor; 4796 articles as of 2026-10-13. systemd active on AWS VM. | Still running as of 2026-10-14 (CAP 20).</t>
         </is>
       </c>
     </row>
@@ -3109,11 +3109,11 @@
       </c>
       <c r="F58" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G58" s="21" t="n">
-        <v>7948</v>
+        <v>14989</v>
       </c>
       <c r="H58" s="0" t="inlineStr">
         <is>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="J58" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@campustimes; 7948 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@campustimes; 7948 articles as of 2026-10-13. systemd active on AWS VM. | Finished as of 2026-10-14. 14989 articles. File: ~/Downloads/campustimes.csv</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="J59" s="0" t="inlineStr">
         <is>
-          <t>Finished as of 2026-10-13. 10125 articles. systemd inactive. File: ~/Downloads/case.csv</t>
+          <t>Finished as of 2026-10-13. 10125 articles. systemd inactive. File: ~/Downloads/case.csv | Finished as of 2026-10-14. 10125 articles. File: ~/Downloads/case.csv</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="D62" s="0" t="inlineStr">
         <is>
-          <t>thefordhamram.com</t>
+          <t>fordhamram.com</t>
         </is>
       </c>
       <c r="E62" s="0" t="inlineStr">
@@ -3301,11 +3301,11 @@
       </c>
       <c r="F62" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G62" s="21" t="n">
-        <v>6575</v>
+        <v>8902</v>
       </c>
       <c r="H62" s="0" t="inlineStr">
         <is>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="J62" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@fordham; 6575 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@fordham; 6575 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (8902 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -3349,11 +3349,11 @@
       </c>
       <c r="F63" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G63" s="21" t="n">
-        <v>2050</v>
+        <v>4379</v>
       </c>
       <c r="H63" s="0" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="J63" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@freepress; 2050 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@freepress; 2050 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (4379 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
     <row r="66">
       <c r="A66" s="0" t="inlineStr">
         <is>
-          <t>Tulane University of Louisiana</t>
+          <t>Tulane University</t>
         </is>
       </c>
       <c r="B66" s="0" t="inlineStr">
@@ -3493,11 +3493,11 @@
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G66" s="21" t="n">
-        <v>650</v>
+        <v>2991</v>
       </c>
       <c r="H66" s="0" t="inlineStr">
         <is>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="J66" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@hullabaloo; 650 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@hullabaloo; 650 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (2991 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -3589,11 +3589,11 @@
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G68" s="21" t="n">
-        <v>6399</v>
+        <v>9739</v>
       </c>
       <c r="H68" s="0" t="inlineStr">
         <is>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="J68" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@lehigh; 6399 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@lehigh; 6399 articles as of 2026-10-13. systemd active on AWS VM. | Finished as of 2026-10-14. 9739 articles. File: ~/Downloads/lehigh.csv</t>
         </is>
       </c>
     </row>
@@ -3637,11 +3637,11 @@
       </c>
       <c r="F69" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G69" s="21" t="n">
-        <v>6298</v>
+        <v>8556</v>
       </c>
       <c r="H69" s="0" t="inlineStr">
         <is>
@@ -3653,7 +3653,7 @@
       </c>
       <c r="J69" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@northeastern; 6298 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@northeastern; 6298 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (8556 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3701,7 @@
       </c>
       <c r="J70" s="0" t="inlineStr">
         <is>
-          <t>Finished as of 2026-10-13. 2798 articles. systemd inactive. File: ~/Downloads/paladin.csv</t>
+          <t>Finished as of 2026-10-13. 2798 articles. systemd inactive. File: ~/Downloads/paladin.csv | Finished as of 2026-10-14. 2798 articles. File: ~/Downloads/paladin.csv</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="J72" s="0" t="inlineStr">
         <is>
-          <t>Finished as of 2026-10-13. 2673 articles. systemd inactive. File: ~/Downloads/ringtumphi.csv</t>
+          <t>Finished as of 2026-10-13. 2673 articles. systemd inactive. File: ~/Downloads/ringtumphi.csv | Finished as of 2026-10-14. 2673 articles. File: ~/Downloads/ringtumphi.csv</t>
         </is>
       </c>
     </row>
@@ -3877,11 +3877,11 @@
       </c>
       <c r="F74" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G74" s="21" t="n">
-        <v>5500</v>
+        <v>7754</v>
       </c>
       <c r="H74" s="0" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="J74" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@trinitonian; 5500 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@trinitonian; 5500 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (7754 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -3973,11 +3973,11 @@
       </c>
       <c r="F76" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G76" s="21" t="n">
-        <v>6398</v>
+        <v>8660</v>
       </c>
       <c r="H76" s="0" t="inlineStr">
         <is>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="J76" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@vanderbilt; 6398 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@vanderbilt; 6398 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (8660 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -4021,11 +4021,11 @@
       </c>
       <c r="F77" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>blocked</t>
         </is>
       </c>
       <c r="G77" s="21" t="n">
-        <v>6745</v>
+        <v>9110</v>
       </c>
       <c r="H77" s="0" t="inlineStr">
         <is>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="J77" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@villanova; 6745 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@villanova; 6745 articles as of 2026-10-13. systemd active on AWS VM. | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (9110 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -4069,11 +4069,11 @@
       </c>
       <c r="F78" s="0" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="G78" s="21" t="n">
-        <v>6482</v>
+        <v>7837</v>
       </c>
       <c r="H78" s="0" t="inlineStr">
         <is>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="J78" s="0" t="inlineStr">
         <is>
-          <t>newspaper-scraper@wakeforest; 6482 articles as of 2026-10-13. systemd active on AWS VM.</t>
+          <t>newspaper-scraper@wakeforest; 6482 articles as of 2026-10-13. systemd active on AWS VM. | Finished as of 2026-10-14. 7837 articles. File: ~/Downloads/wakeforest.csv</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="J79" s="0" t="inlineStr">
         <is>
-          <t>Finished as of 2026-10-13. 4796 articles. systemd inactive. File: ~/Downloads/wellesley.csv</t>
+          <t>Finished as of 2026-10-13. 4796 articles. systemd inactive. File: ~/Downloads/wellesley.csv | Finished as of 2026-10-14. 4796 articles. File: ~/Downloads/wellesley.csv</t>
         </is>
       </c>
     </row>
@@ -4406,8 +4406,11 @@
       </c>
       <c r="F86" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G86" s="0" t="n">
+        <v>1210</v>
       </c>
       <c r="H86" s="0" t="inlineStr">
         <is>
@@ -4421,7 +4424,7 @@
       </c>
       <c r="J86" s="0" t="inlineStr">
         <is>
-          <t>Started wave21 full scrape 2026-10-13 (CAP 20).</t>
+          <t>Started wave21 full scrape 2026-10-13 (CAP 20). | SITE BLOCKED exit-75 after 4x 403 cooldowns ~2026-10-14 02:36Z. Progress saved (1210 rows). Left alone for now.</t>
         </is>
       </c>
     </row>
@@ -4453,8 +4456,11 @@
       </c>
       <c r="F87" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G87" s="0" t="n">
+        <v>874</v>
       </c>
       <c r="H87" s="0" t="inlineStr">
         <is>
@@ -4468,7 +4474,7 @@
       </c>
       <c r="J87" s="0" t="inlineStr">
         <is>
-          <t>Started wave21 full scrape 2026-10-13 (CAP 20).</t>
+          <t>Started wave21 full scrape 2026-10-13 (CAP 20). | Finished as of 2026-10-14. 874 articles. File: ~/Downloads/berea.csv</t>
         </is>
       </c>
     </row>
@@ -4500,8 +4506,11 @@
       </c>
       <c r="F88" s="0" t="inlineStr">
         <is>
-          <t>running</t>
-        </is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="G88" s="0" t="n">
+        <v>3230</v>
       </c>
       <c r="H88" s="0" t="inlineStr">
         <is>
@@ -4515,7 +4524,469 @@
       </c>
       <c r="J88" s="0" t="inlineStr">
         <is>
-          <t>Started wave21 full scrape 2026-10-13 (CAP 20).</t>
+          <t>Started wave21 full scrape 2026-10-13 (CAP 20). | Finished as of 2026-10-14. 3230 articles. File: ~/Downloads/sewanee.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Colby College</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>The Colby Echo</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>colby</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>colbyecho.news</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Colorado College</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>The Catalyst</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>catalyst</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>thecatalystnews.com</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>College of the Holy Cross</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>The Spire</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>holycross</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>hcspire.com</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Liberal Arts</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Wheaton College--Illinois</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>The Wheaton Record</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>wheatonrecord</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>thewheatonrecord.com</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Christian Colleges</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>University of Connecticut</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>The Daily Campus</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>dailycampus</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>dailycampus.com</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Florida International University</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>PantherNOW</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>panthernow</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>panthernow.com</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Drexel University</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>The Triangle</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>triangle</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>thetriangle.org</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>The Ohio State University</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>The Lantern</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>lantern</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>thelantern.com</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Public Universities</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Texas A&amp;M University</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>The Battalion</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>batt</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>thebatt.com</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Washington University in St. Louis</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Student Life</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>studlife</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>studlife.com</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Santa Clara University</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>The Santa Clara</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>santaclara</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>thesantaclara.org</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>National Universities</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Wave 22 staged 2026-10-14 (refill after 403 blocks; blocked SNO left alone).</t>
         </is>
       </c>
     </row>

</xml_diff>